<commit_message>
Fix Excel table names and verify native opening
</commit_message>
<xml_diff>
--- a/01_要件定義/outputs/requirements-v01/PhotonCam_AWS_要件定義_v0.1.xlsx
+++ b/01_要件定義/outputs/requirements-v01/PhotonCam_AWS_要件定義_v0.1.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_概要" sheetId="1" r:id="R6644ca4298ae467a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_范围" sheetId="2" r:id="R0541a99d79c7487e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_现状依据" sheetId="3" r:id="R203cc4d07f6f4382"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_要件清单" sheetId="4" r:id="R47b83de9e0564fe1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_验收条件" sheetId="5" r:id="R68127ff48af6451d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_待确认" sheetId="6" r:id="R21db108eea8e4b75"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_阶段评审" sheetId="7" r:id="Rb251b7828d7d4e49"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_页面基线" sheetId="8" r:id="R1109de958a354ca1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_概要" sheetId="1" r:id="R039a350206384f48"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_范围" sheetId="2" r:id="Rad3654f4580f4701"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_现状依据" sheetId="3" r:id="R28b04c20aceb4fd6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_要件清单" sheetId="4" r:id="R33960a5505c34d34"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_验收条件" sheetId="5" r:id="R21f11258adf0482d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_待确认" sheetId="6" r:id="Rab78b13c780942e5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_阶段评审" sheetId="7" r:id="Recca37135f104b82"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_页面基线" sheetId="8" r:id="R46345a4ce813438b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -140,7 +140,7 @@
   <x:dxfs count="1">
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE4D6"/>
         </x:patternFill>
       </x:fill>
@@ -150,7 +150,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="T0" displayName="T0" ref="A5:C18" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PhotonCamRequirements_1" displayName="PhotonCamRequirements_1" ref="A5:C18" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:C18"/>
   <x:tableColumns count="3">
     <x:tableColumn id="1" name="项目／項目"/>
@@ -162,7 +162,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="T1" displayName="T1" ref="A5:F13" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="PhotonCamRequirements_2" displayName="PhotonCamRequirements_2" ref="A5:F13" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:F13"/>
   <x:tableColumns count="6">
     <x:tableColumn id="1" name="编号"/>
@@ -177,7 +177,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="T2" displayName="T2" ref="A5:F15" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="PhotonCamRequirements_3" displayName="PhotonCamRequirements_3" ref="A5:F15" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:F15"/>
   <x:tableColumns count="6">
     <x:tableColumn id="1" name="依据ID"/>
@@ -192,7 +192,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="T3" displayName="T3" ref="A5:G31" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="PhotonCamRequirements_4" displayName="PhotonCamRequirements_4" ref="A5:G31" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:G31"/>
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="要件ID"/>
@@ -208,7 +208,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="T4" displayName="T4" ref="A5:G31" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="PhotonCamRequirements_5" displayName="PhotonCamRequirements_5" ref="A5:G31" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:G31"/>
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="验收ID／要件ID"/>
@@ -224,7 +224,7 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="T5" displayName="T5" ref="A5:I16" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="PhotonCamRequirements_6" displayName="PhotonCamRequirements_6" ref="A5:I16" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:I16"/>
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="课题ID"/>
@@ -242,7 +242,7 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="T6" displayName="T6" ref="A5:H13" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="PhotonCamRequirements_7" displayName="PhotonCamRequirements_7" ref="A5:H13" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:H13"/>
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="阶段ID"/>
@@ -259,7 +259,7 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="T7" displayName="T7" ref="A5:G55" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="PhotonCamRequirements_8" displayName="PhotonCamRequirements_8" ref="A5:G55" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A5:G55"/>
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="页面ID"/>
@@ -661,7 +661,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra89afb6d199e4166"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6b47d792bd774458"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -897,7 +897,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9ce0eb67a43e4bfc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4d6c0347e1d841cb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1173,7 +1173,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9327381fd6c24d23"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R403be64a1fe54e10"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1866,7 +1866,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7345b1242a0d454f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re8f054bf47e64105"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2553,7 +2553,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3485904b176c4236"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R46f7d45a92b84599"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2955,7 +2955,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3df2fca7eead4ded"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R62415dcba0314168"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3260,7 +3260,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6ebf432af2d74c24"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf9c7154bcbd440f7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4494,7 +4494,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4995650a1c164c4f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R97b30d35de6143da"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Distinguish dev source copy from production source repository
</commit_message>
<xml_diff>
--- a/01_要件定義/outputs/requirements-v01/PhotonCam_AWS_要件定義_v0.1.xlsx
+++ b/01_要件定義/outputs/requirements-v01/PhotonCam_AWS_要件定義_v0.1.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_概要" sheetId="1" r:id="R82065fc3cb2c4b15"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_范围" sheetId="2" r:id="R403cf62cc67e4d51"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_现状依据" sheetId="3" r:id="R65feb101366344cb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_要件清单" sheetId="4" r:id="Rb52624502707420a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_验收条件" sheetId="5" r:id="R7f544260d7234484"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_待确认" sheetId="6" r:id="R806117529847497d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_阶段评审" sheetId="7" r:id="R5b28083be9d44c93"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_页面基线" sheetId="8" r:id="R87e99716ae764a21"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_概要" sheetId="1" r:id="Rb880a7089ffa4e70"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_范围" sheetId="2" r:id="R7d507f3a29344388"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_现状依据" sheetId="3" r:id="R0cda765281f64896"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_要件清单" sheetId="4" r:id="R039dd51158bb4e92"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_验收条件" sheetId="5" r:id="R25b80ccfb539499d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_待确认" sheetId="6" r:id="R1e2dd30bf396471d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_阶段评审" sheetId="7" r:id="R2950eabd305b4dd4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_页面基线" sheetId="8" r:id="R6f71628a7b6b4fdf"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -323,15 +323,6 @@
     <x:t xml:space="preserve">S07</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">私有源码工作副本与 origin main 已核对为同一提交</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">源码 Git 检查；源码与发布包构建调查.md</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">572c5a1311151acd45a361aa718f59070bfde32d</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">S08</x:t>
   </x:si>
   <x:si>
@@ -941,9 +932,6 @@
     <x:t xml:space="preserve">A22 / R22</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">dev 验收完成</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">正式前</x:t>
   </x:si>
   <x:si>
@@ -1092,9 +1080,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">自动部署规则</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">触发分支、提交权限、dev 是否自动发布及失败处理？</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">影响流水线及 GitHub 连接授权</x:t>
@@ -2229,7 +2214,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="3" t="str">
-        <x:v>v0.1 评审草案／レビュー草案　更新 2026-10-08</x:v>
+        <x:v>v0.1 评审草案／レビュー草案　更新 2026-10-13</x:v>
       </x:c>
       <x:c r="B3" s="1"/>
       <x:c r="C3" s="1"/>
@@ -2399,7 +2384,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf514c1ba0af440bc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R153778ef704a4ffb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2635,7 +2620,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4e002c9a33b0406a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R852f621e560e403c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2828,69 +2813,69 @@
         <x:v>100</x:v>
       </x:c>
     </x:row>
-    <x:row r="12" ht="42" customHeight="1">
+    <x:row r="12" ht="110" customHeight="1">
       <x:c r="A12" s="5" t="s">
         <x:v>101</x:v>
       </x:c>
-      <x:c r="B12" s="5" t="s">
-        <x:v>79</x:v>
-      </x:c>
-      <x:c r="C12" s="5" t="s">
-        <x:v>102</x:v>
-      </x:c>
-      <x:c r="D12" s="5" t="s">
-        <x:v>81</x:v>
-      </x:c>
-      <x:c r="E12" s="5" t="s">
-        <x:v>103</x:v>
-      </x:c>
-      <x:c r="F12" s="5" t="s">
-        <x:v>104</x:v>
+      <x:c r="B12" s="5" t="str">
+        <x:v>调查事实／用户约定</x:v>
+      </x:c>
+      <x:c r="C12" s="5" t="str">
+        <x:v>dev暂用用户私有仓库源码副本；曾核对本地与该origin main一致。正式发布以开发者私有原仓库为准</x:v>
+      </x:c>
+      <x:c r="D12" s="5" t="str">
+        <x:v>dev已核对，正式未核验</x:v>
+      </x:c>
+      <x:c r="E12" s="5" t="str">
+        <x:v>源码Git调查；2026-10-13用户约定；源码仓库边界说明.md</x:v>
+      </x:c>
+      <x:c r="F12" s="5" t="str">
+        <x:v>dev提交572c5a1311151acd45a361aa718f59070bfde32d；未核对正式原仓库，不证明两库同版</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="42" customHeight="1">
       <x:c r="A13" s="6" t="s">
-        <x:v>105</x:v>
+        <x:v>102</x:v>
       </x:c>
       <x:c r="B13" s="6" t="s">
         <x:v>79</x:v>
       </x:c>
       <x:c r="C13" s="6" t="s">
-        <x:v>106</x:v>
+        <x:v>103</x:v>
       </x:c>
       <x:c r="D13" s="6" t="s">
         <x:v>81</x:v>
       </x:c>
       <x:c r="E13" s="6" t="s">
-        <x:v>107</x:v>
+        <x:v>104</x:v>
       </x:c>
       <x:c r="F13" s="6" t="s">
-        <x:v>108</x:v>
+        <x:v>105</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="42" customHeight="1">
       <x:c r="A14" s="5" t="s">
-        <x:v>109</x:v>
+        <x:v>106</x:v>
       </x:c>
       <x:c r="B14" s="5" t="s">
         <x:v>79</x:v>
       </x:c>
       <x:c r="C14" s="5" t="s">
-        <x:v>110</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="D14" s="5" t="s">
         <x:v>90</x:v>
       </x:c>
       <x:c r="E14" s="5" t="s">
-        <x:v>111</x:v>
+        <x:v>108</x:v>
       </x:c>
       <x:c r="F14" s="5" t="s">
-        <x:v>112</x:v>
+        <x:v>109</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="42" customHeight="1">
       <x:c r="A15" s="6" t="s">
-        <x:v>113</x:v>
+        <x:v>110</x:v>
       </x:c>
       <x:c r="B15" s="6" t="str">
         <x:v>开发者说明与调查</x:v>
@@ -2991,7 +2976,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf7c6690aca4f44c3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R20a091d018994d41"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3020,7 +3005,7 @@
     </x:row>
     <x:row r="2" ht="21">
       <x:c r="A2" s="2" t="s">
-        <x:v>114</x:v>
+        <x:v>111</x:v>
       </x:c>
       <x:c r="B2" s="1"/>
       <x:c r="C2" s="1"/>
@@ -3031,7 +3016,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="3" t="s">
-        <x:v>115</x:v>
+        <x:v>112</x:v>
       </x:c>
       <x:c r="B3" s="1"/>
       <x:c r="C3" s="1"/>
@@ -3051,148 +3036,148 @@
     </x:row>
     <x:row r="5" ht="37.95000076293945" customHeight="1">
       <x:c r="A5" s="4" t="s">
-        <x:v>116</x:v>
+        <x:v>113</x:v>
       </x:c>
       <x:c r="B5" s="4" t="s">
-        <x:v>117</x:v>
+        <x:v>114</x:v>
       </x:c>
       <x:c r="C5" s="4" t="s">
-        <x:v>118</x:v>
+        <x:v>115</x:v>
       </x:c>
       <x:c r="D5" s="4" t="s">
         <x:v>68</x:v>
       </x:c>
       <x:c r="E5" s="4" t="s">
-        <x:v>119</x:v>
+        <x:v>116</x:v>
       </x:c>
       <x:c r="F5" s="4" t="s">
-        <x:v>120</x:v>
+        <x:v>117</x:v>
       </x:c>
       <x:c r="G5" s="4" t="s">
-        <x:v>121</x:v>
+        <x:v>118</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="42" customHeight="1">
       <x:c r="A6" s="5" t="s">
-        <x:v>122</x:v>
+        <x:v>119</x:v>
       </x:c>
       <x:c r="B6" s="5" t="s">
-        <x:v>123</x:v>
+        <x:v>120</x:v>
       </x:c>
       <x:c r="C6" s="5" t="s">
-        <x:v>124</x:v>
+        <x:v>121</x:v>
       </x:c>
       <x:c r="D6" s="5" t="s">
         <x:v>46</x:v>
       </x:c>
       <x:c r="E6" s="7" t="s">
-        <x:v>125</x:v>
+        <x:v>122</x:v>
       </x:c>
       <x:c r="F6" s="7" t="s">
-        <x:v>126</x:v>
+        <x:v>123</x:v>
       </x:c>
       <x:c r="G6" s="5" t="s">
-        <x:v>127</x:v>
+        <x:v>124</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="42" customHeight="1">
       <x:c r="A7" s="6" t="s">
+        <x:v>125</x:v>
+      </x:c>
+      <x:c r="B7" s="6" t="s">
+        <x:v>126</x:v>
+      </x:c>
+      <x:c r="C7" s="6" t="s">
+        <x:v>127</x:v>
+      </x:c>
+      <x:c r="D7" s="6" t="s">
         <x:v>128</x:v>
       </x:c>
-      <x:c r="B7" s="6" t="s">
+      <x:c r="E7" s="7" t="s">
+        <x:v>122</x:v>
+      </x:c>
+      <x:c r="F7" s="7" t="s">
+        <x:v>123</x:v>
+      </x:c>
+      <x:c r="G7" s="6" t="s">
         <x:v>129</x:v>
-      </x:c>
-      <x:c r="C7" s="6" t="s">
-        <x:v>130</x:v>
-      </x:c>
-      <x:c r="D7" s="6" t="s">
-        <x:v>131</x:v>
-      </x:c>
-      <x:c r="E7" s="7" t="s">
-        <x:v>125</x:v>
-      </x:c>
-      <x:c r="F7" s="7" t="s">
-        <x:v>126</x:v>
-      </x:c>
-      <x:c r="G7" s="6" t="s">
-        <x:v>132</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="42" customHeight="1">
       <x:c r="A8" s="5" t="s">
-        <x:v>133</x:v>
+        <x:v>130</x:v>
       </x:c>
       <x:c r="B8" s="5" t="s">
-        <x:v>129</x:v>
+        <x:v>126</x:v>
       </x:c>
       <x:c r="C8" s="5" t="s">
-        <x:v>134</x:v>
+        <x:v>131</x:v>
       </x:c>
       <x:c r="D8" s="5" t="s">
         <x:v>84</x:v>
       </x:c>
       <x:c r="E8" s="7" t="s">
-        <x:v>135</x:v>
+        <x:v>132</x:v>
       </x:c>
       <x:c r="F8" s="7" t="s">
-        <x:v>126</x:v>
+        <x:v>123</x:v>
       </x:c>
       <x:c r="G8" s="5" t="s">
-        <x:v>136</x:v>
+        <x:v>133</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="42" customHeight="1">
       <x:c r="A9" s="6" t="s">
-        <x:v>137</x:v>
+        <x:v>134</x:v>
       </x:c>
       <x:c r="B9" s="6" t="s">
-        <x:v>129</x:v>
+        <x:v>126</x:v>
       </x:c>
       <x:c r="C9" s="6" t="s">
-        <x:v>138</x:v>
+        <x:v>135</x:v>
       </x:c>
       <x:c r="D9" s="6" t="s">
         <x:v>84</x:v>
       </x:c>
       <x:c r="E9" s="7" t="s">
-        <x:v>135</x:v>
+        <x:v>132</x:v>
       </x:c>
       <x:c r="F9" s="7" t="s">
-        <x:v>126</x:v>
+        <x:v>123</x:v>
       </x:c>
       <x:c r="G9" s="6" t="s">
-        <x:v>139</x:v>
+        <x:v>136</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="42" customHeight="1">
       <x:c r="A10" s="5" t="s">
-        <x:v>140</x:v>
+        <x:v>137</x:v>
       </x:c>
       <x:c r="B10" s="5" t="s">
-        <x:v>129</x:v>
+        <x:v>126</x:v>
       </x:c>
       <x:c r="C10" s="5" t="s">
-        <x:v>141</x:v>
+        <x:v>138</x:v>
       </x:c>
       <x:c r="D10" s="5" t="s">
-        <x:v>131</x:v>
+        <x:v>128</x:v>
       </x:c>
       <x:c r="E10" s="7" t="s">
-        <x:v>135</x:v>
+        <x:v>132</x:v>
       </x:c>
       <x:c r="F10" s="7" t="s">
-        <x:v>126</x:v>
+        <x:v>123</x:v>
       </x:c>
       <x:c r="G10" s="5" t="s">
-        <x:v>136</x:v>
+        <x:v>133</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="42" customHeight="1">
       <x:c r="A11" s="6" t="s">
-        <x:v>142</x:v>
+        <x:v>139</x:v>
       </x:c>
       <x:c r="B11" s="6" t="s">
-        <x:v>129</x:v>
+        <x:v>126</x:v>
       </x:c>
       <x:c r="C11" s="6" t="str">
         <x:v>正式环境续用 juniperphoton.dev/photoncam/，深层链接、刷新和资源路径正常；dev地址另定。</x:v>
@@ -3201,366 +3186,366 @@
         <x:v>S02,S04,S11</x:v>
       </x:c>
       <x:c r="E11" s="7" t="s">
-        <x:v>125</x:v>
+        <x:v>122</x:v>
       </x:c>
       <x:c r="F11" s="7" t="s">
-        <x:v>126</x:v>
+        <x:v>123</x:v>
       </x:c>
       <x:c r="G11" s="6" t="s">
-        <x:v>132</x:v>
+        <x:v>129</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="42" customHeight="1">
       <x:c r="A12" s="5" t="s">
-        <x:v>143</x:v>
+        <x:v>140</x:v>
       </x:c>
       <x:c r="B12" s="5" t="s">
+        <x:v>126</x:v>
+      </x:c>
+      <x:c r="C12" s="5" t="s">
+        <x:v>141</x:v>
+      </x:c>
+      <x:c r="D12" s="5" t="s">
+        <x:v>142</x:v>
+      </x:c>
+      <x:c r="E12" s="7" t="s">
+        <x:v>132</x:v>
+      </x:c>
+      <x:c r="F12" s="7" t="s">
+        <x:v>123</x:v>
+      </x:c>
+      <x:c r="G12" s="5" t="s">
         <x:v>129</x:v>
-      </x:c>
-      <x:c r="C12" s="5" t="s">
-        <x:v>144</x:v>
-      </x:c>
-      <x:c r="D12" s="5" t="s">
-        <x:v>145</x:v>
-      </x:c>
-      <x:c r="E12" s="7" t="s">
-        <x:v>135</x:v>
-      </x:c>
-      <x:c r="F12" s="7" t="s">
-        <x:v>126</x:v>
-      </x:c>
-      <x:c r="G12" s="5" t="s">
-        <x:v>132</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="42" customHeight="1">
       <x:c r="A13" s="6" t="s">
+        <x:v>143</x:v>
+      </x:c>
+      <x:c r="B13" s="6" t="s">
+        <x:v>144</x:v>
+      </x:c>
+      <x:c r="C13" s="6" t="s">
+        <x:v>145</x:v>
+      </x:c>
+      <x:c r="D13" s="6" t="s">
         <x:v>146</x:v>
       </x:c>
-      <x:c r="B13" s="6" t="s">
+      <x:c r="E13" s="7" t="s">
+        <x:v>122</x:v>
+      </x:c>
+      <x:c r="F13" s="7" t="s">
+        <x:v>123</x:v>
+      </x:c>
+      <x:c r="G13" s="6" t="s">
         <x:v>147</x:v>
-      </x:c>
-      <x:c r="C13" s="6" t="s">
-        <x:v>148</x:v>
-      </x:c>
-      <x:c r="D13" s="6" t="s">
-        <x:v>149</x:v>
-      </x:c>
-      <x:c r="E13" s="7" t="s">
-        <x:v>125</x:v>
-      </x:c>
-      <x:c r="F13" s="7" t="s">
-        <x:v>126</x:v>
-      </x:c>
-      <x:c r="G13" s="6" t="s">
-        <x:v>150</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="42" customHeight="1">
       <x:c r="A14" s="5" t="s">
-        <x:v>151</x:v>
+        <x:v>148</x:v>
       </x:c>
       <x:c r="B14" s="5" t="s">
+        <x:v>144</x:v>
+      </x:c>
+      <x:c r="C14" s="5" t="s">
+        <x:v>149</x:v>
+      </x:c>
+      <x:c r="D14" s="5" t="s">
+        <x:v>150</x:v>
+      </x:c>
+      <x:c r="E14" s="7" t="s">
+        <x:v>122</x:v>
+      </x:c>
+      <x:c r="F14" s="7" t="s">
+        <x:v>123</x:v>
+      </x:c>
+      <x:c r="G14" s="5" t="s">
         <x:v>147</x:v>
-      </x:c>
-      <x:c r="C14" s="5" t="s">
-        <x:v>152</x:v>
-      </x:c>
-      <x:c r="D14" s="5" t="s">
-        <x:v>153</x:v>
-      </x:c>
-      <x:c r="E14" s="7" t="s">
-        <x:v>125</x:v>
-      </x:c>
-      <x:c r="F14" s="7" t="s">
-        <x:v>126</x:v>
-      </x:c>
-      <x:c r="G14" s="5" t="s">
-        <x:v>150</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="42" customHeight="1">
       <x:c r="A15" s="6" t="s">
-        <x:v>154</x:v>
+        <x:v>151</x:v>
       </x:c>
       <x:c r="B15" s="6" t="s">
-        <x:v>155</x:v>
+        <x:v>152</x:v>
       </x:c>
       <x:c r="C15" s="6" t="s">
-        <x:v>156</x:v>
+        <x:v>153</x:v>
       </x:c>
       <x:c r="D15" s="6" t="s">
         <x:v>51</x:v>
       </x:c>
       <x:c r="E15" s="7" t="s">
-        <x:v>125</x:v>
+        <x:v>122</x:v>
       </x:c>
       <x:c r="F15" s="7" t="s">
-        <x:v>126</x:v>
+        <x:v>123</x:v>
       </x:c>
       <x:c r="G15" s="6" t="s">
-        <x:v>150</x:v>
+        <x:v>147</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="42" customHeight="1">
       <x:c r="A16" s="5" t="s">
-        <x:v>157</x:v>
+        <x:v>154</x:v>
       </x:c>
       <x:c r="B16" s="5" t="s">
+        <x:v>152</x:v>
+      </x:c>
+      <x:c r="C16" s="5" t="s">
         <x:v>155</x:v>
       </x:c>
-      <x:c r="C16" s="5" t="s">
-        <x:v>158</x:v>
-      </x:c>
-      <x:c r="D16" s="5" t="s">
-        <x:v>51</x:v>
+      <x:c r="D16" s="5" t="str">
+        <x:v>S01,S06,S07</x:v>
       </x:c>
       <x:c r="E16" s="7" t="s">
-        <x:v>125</x:v>
+        <x:v>122</x:v>
       </x:c>
       <x:c r="F16" s="7" t="s">
-        <x:v>126</x:v>
+        <x:v>123</x:v>
       </x:c>
       <x:c r="G16" s="5" t="s">
-        <x:v>159</x:v>
+        <x:v>156</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="42" customHeight="1">
       <x:c r="A17" s="6" t="s">
-        <x:v>160</x:v>
+        <x:v>157</x:v>
       </x:c>
       <x:c r="B17" s="6" t="s">
-        <x:v>155</x:v>
+        <x:v>152</x:v>
       </x:c>
       <x:c r="C17" s="6" t="s">
-        <x:v>161</x:v>
+        <x:v>158</x:v>
       </x:c>
       <x:c r="D17" s="6" t="s">
-        <x:v>145</x:v>
+        <x:v>142</x:v>
       </x:c>
       <x:c r="E17" s="7" t="s">
-        <x:v>135</x:v>
+        <x:v>132</x:v>
       </x:c>
       <x:c r="F17" s="7" t="s">
-        <x:v>126</x:v>
+        <x:v>123</x:v>
       </x:c>
       <x:c r="G17" s="6" t="s">
-        <x:v>159</x:v>
+        <x:v>156</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="42" customHeight="1">
       <x:c r="A18" s="5" t="s">
-        <x:v>162</x:v>
+        <x:v>159</x:v>
       </x:c>
       <x:c r="B18" s="5" t="s">
-        <x:v>155</x:v>
+        <x:v>152</x:v>
       </x:c>
       <x:c r="C18" s="5" t="s">
-        <x:v>163</x:v>
+        <x:v>160</x:v>
       </x:c>
       <x:c r="D18" s="5" t="s">
-        <x:v>145</x:v>
+        <x:v>142</x:v>
       </x:c>
       <x:c r="E18" s="7" t="s">
-        <x:v>135</x:v>
+        <x:v>132</x:v>
       </x:c>
       <x:c r="F18" s="7" t="s">
-        <x:v>126</x:v>
+        <x:v>123</x:v>
       </x:c>
       <x:c r="G18" s="5" t="s">
-        <x:v>164</x:v>
+        <x:v>161</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="42" customHeight="1">
       <x:c r="A19" s="6" t="s">
-        <x:v>165</x:v>
+        <x:v>162</x:v>
       </x:c>
       <x:c r="B19" s="6" t="s">
-        <x:v>166</x:v>
+        <x:v>163</x:v>
       </x:c>
       <x:c r="C19" s="6" t="s">
-        <x:v>167</x:v>
+        <x:v>164</x:v>
       </x:c>
       <x:c r="D19" s="6" t="s">
         <x:v>46</x:v>
       </x:c>
       <x:c r="E19" s="7" t="s">
-        <x:v>125</x:v>
+        <x:v>122</x:v>
       </x:c>
       <x:c r="F19" s="7" t="s">
-        <x:v>126</x:v>
+        <x:v>123</x:v>
       </x:c>
       <x:c r="G19" s="6" t="s">
-        <x:v>139</x:v>
+        <x:v>136</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="42" customHeight="1">
       <x:c r="A20" s="5" t="s">
-        <x:v>168</x:v>
+        <x:v>165</x:v>
       </x:c>
       <x:c r="B20" s="5" t="s">
+        <x:v>163</x:v>
+      </x:c>
+      <x:c r="C20" s="5" t="s">
         <x:v>166</x:v>
       </x:c>
-      <x:c r="C20" s="5" t="s">
-        <x:v>169</x:v>
-      </x:c>
       <x:c r="D20" s="5" t="s">
-        <x:v>170</x:v>
+        <x:v>167</x:v>
       </x:c>
       <x:c r="E20" s="7" t="s">
-        <x:v>125</x:v>
+        <x:v>122</x:v>
       </x:c>
       <x:c r="F20" s="7" t="s">
-        <x:v>126</x:v>
+        <x:v>123</x:v>
       </x:c>
       <x:c r="G20" s="5" t="s">
-        <x:v>127</x:v>
+        <x:v>124</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="42" customHeight="1">
       <x:c r="A21" s="6" t="s">
-        <x:v>171</x:v>
+        <x:v>168</x:v>
       </x:c>
       <x:c r="B21" s="6" t="s">
-        <x:v>166</x:v>
+        <x:v>163</x:v>
       </x:c>
       <x:c r="C21" s="6" t="s">
-        <x:v>172</x:v>
+        <x:v>169</x:v>
       </x:c>
       <x:c r="D21" s="6" t="s">
-        <x:v>145</x:v>
+        <x:v>142</x:v>
       </x:c>
       <x:c r="E21" s="7" t="s">
-        <x:v>135</x:v>
+        <x:v>132</x:v>
       </x:c>
       <x:c r="F21" s="7" t="s">
-        <x:v>126</x:v>
+        <x:v>123</x:v>
       </x:c>
       <x:c r="G21" s="6" t="s">
-        <x:v>127</x:v>
+        <x:v>124</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="42" customHeight="1">
       <x:c r="A22" s="5" t="s">
-        <x:v>173</x:v>
+        <x:v>170</x:v>
       </x:c>
       <x:c r="B22" s="5" t="s">
-        <x:v>174</x:v>
+        <x:v>171</x:v>
       </x:c>
       <x:c r="C22" s="5" t="s">
-        <x:v>175</x:v>
+        <x:v>172</x:v>
       </x:c>
       <x:c r="D22" s="5" t="s">
-        <x:v>145</x:v>
+        <x:v>142</x:v>
       </x:c>
       <x:c r="E22" s="7" t="s">
-        <x:v>135</x:v>
+        <x:v>132</x:v>
       </x:c>
       <x:c r="F22" s="7" t="s">
-        <x:v>126</x:v>
+        <x:v>123</x:v>
       </x:c>
       <x:c r="G22" s="5" t="s">
-        <x:v>136</x:v>
+        <x:v>133</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="42" customHeight="1">
       <x:c r="A23" s="6" t="s">
-        <x:v>176</x:v>
+        <x:v>173</x:v>
       </x:c>
       <x:c r="B23" s="6" t="s">
+        <x:v>171</x:v>
+      </x:c>
+      <x:c r="C23" s="6" t="s">
         <x:v>174</x:v>
-      </x:c>
-      <x:c r="C23" s="6" t="s">
-        <x:v>177</x:v>
       </x:c>
       <x:c r="D23" s="6" t="s">
         <x:v>31</x:v>
       </x:c>
       <x:c r="E23" s="7" t="s">
-        <x:v>178</x:v>
+        <x:v>175</x:v>
       </x:c>
       <x:c r="F23" s="7" t="s">
-        <x:v>126</x:v>
+        <x:v>123</x:v>
       </x:c>
       <x:c r="G23" s="6" t="s">
-        <x:v>179</x:v>
+        <x:v>176</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="42" customHeight="1">
       <x:c r="A24" s="5" t="s">
+        <x:v>177</x:v>
+      </x:c>
+      <x:c r="B24" s="5" t="s">
+        <x:v>171</x:v>
+      </x:c>
+      <x:c r="C24" s="5" t="s">
+        <x:v>178</x:v>
+      </x:c>
+      <x:c r="D24" s="5" t="s">
+        <x:v>179</x:v>
+      </x:c>
+      <x:c r="E24" s="7" t="s">
+        <x:v>122</x:v>
+      </x:c>
+      <x:c r="F24" s="7" t="s">
+        <x:v>123</x:v>
+      </x:c>
+      <x:c r="G24" s="5" t="s">
         <x:v>180</x:v>
-      </x:c>
-      <x:c r="B24" s="5" t="s">
-        <x:v>174</x:v>
-      </x:c>
-      <x:c r="C24" s="5" t="s">
-        <x:v>181</x:v>
-      </x:c>
-      <x:c r="D24" s="5" t="s">
-        <x:v>182</x:v>
-      </x:c>
-      <x:c r="E24" s="7" t="s">
-        <x:v>125</x:v>
-      </x:c>
-      <x:c r="F24" s="7" t="s">
-        <x:v>126</x:v>
-      </x:c>
-      <x:c r="G24" s="5" t="s">
-        <x:v>183</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="42" customHeight="1">
       <x:c r="A25" s="6" t="s">
-        <x:v>184</x:v>
+        <x:v>181</x:v>
       </x:c>
       <x:c r="B25" s="6" t="s">
-        <x:v>185</x:v>
+        <x:v>182</x:v>
       </x:c>
       <x:c r="C25" s="6" t="s">
-        <x:v>186</x:v>
+        <x:v>183</x:v>
       </x:c>
       <x:c r="D25" s="6" t="s">
         <x:v>31</x:v>
       </x:c>
       <x:c r="E25" s="7" t="s">
-        <x:v>178</x:v>
+        <x:v>175</x:v>
       </x:c>
       <x:c r="F25" s="7" t="s">
-        <x:v>126</x:v>
+        <x:v>123</x:v>
       </x:c>
       <x:c r="G25" s="6" t="s">
-        <x:v>187</x:v>
+        <x:v>184</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="42" customHeight="1">
       <x:c r="A26" s="5" t="s">
+        <x:v>185</x:v>
+      </x:c>
+      <x:c r="B26" s="5" t="s">
+        <x:v>186</x:v>
+      </x:c>
+      <x:c r="C26" s="5" t="s">
+        <x:v>187</x:v>
+      </x:c>
+      <x:c r="D26" s="5" t="s">
+        <x:v>167</x:v>
+      </x:c>
+      <x:c r="E26" s="7" t="s">
+        <x:v>122</x:v>
+      </x:c>
+      <x:c r="F26" s="7" t="s">
+        <x:v>123</x:v>
+      </x:c>
+      <x:c r="G26" s="5" t="s">
         <x:v>188</x:v>
-      </x:c>
-      <x:c r="B26" s="5" t="s">
-        <x:v>189</x:v>
-      </x:c>
-      <x:c r="C26" s="5" t="s">
-        <x:v>190</x:v>
-      </x:c>
-      <x:c r="D26" s="5" t="s">
-        <x:v>170</x:v>
-      </x:c>
-      <x:c r="E26" s="7" t="s">
-        <x:v>125</x:v>
-      </x:c>
-      <x:c r="F26" s="7" t="s">
-        <x:v>126</x:v>
-      </x:c>
-      <x:c r="G26" s="5" t="s">
-        <x:v>191</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="85" customHeight="1">
       <x:c r="A27" s="6" t="s">
-        <x:v>192</x:v>
+        <x:v>189</x:v>
       </x:c>
       <x:c r="B27" s="6" t="s">
-        <x:v>189</x:v>
+        <x:v>186</x:v>
       </x:c>
       <x:c r="C27" s="6" t="str">
         <x:v>仅迁移 /photoncam/ 并保留根首页、主站资源与其他产品入口；正式前确认DNS权限、切换窗口、回退与负责人。</x:v>
@@ -3569,105 +3554,105 @@
         <x:v>S01,S11,S12</x:v>
       </x:c>
       <x:c r="E27" s="7" t="s">
-        <x:v>125</x:v>
+        <x:v>122</x:v>
       </x:c>
       <x:c r="F27" s="7" t="s">
-        <x:v>126</x:v>
+        <x:v>123</x:v>
       </x:c>
       <x:c r="G27" s="6" t="s">
-        <x:v>193</x:v>
+        <x:v>190</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="42" customHeight="1">
       <x:c r="A28" s="5" t="s">
-        <x:v>194</x:v>
+        <x:v>191</x:v>
       </x:c>
       <x:c r="B28" s="5" t="s">
-        <x:v>195</x:v>
+        <x:v>192</x:v>
       </x:c>
       <x:c r="C28" s="5" t="s">
-        <x:v>196</x:v>
+        <x:v>193</x:v>
       </x:c>
       <x:c r="D28" s="5" t="s">
         <x:v>46</x:v>
       </x:c>
       <x:c r="E28" s="7" t="s">
-        <x:v>125</x:v>
+        <x:v>122</x:v>
       </x:c>
       <x:c r="F28" s="7" t="s">
-        <x:v>126</x:v>
+        <x:v>123</x:v>
       </x:c>
       <x:c r="G28" s="5" t="s">
-        <x:v>139</x:v>
+        <x:v>136</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="42" customHeight="1">
       <x:c r="A29" s="6" t="s">
-        <x:v>197</x:v>
+        <x:v>194</x:v>
       </x:c>
       <x:c r="B29" s="6" t="s">
+        <x:v>192</x:v>
+      </x:c>
+      <x:c r="C29" s="6" t="s">
         <x:v>195</x:v>
-      </x:c>
-      <x:c r="C29" s="6" t="s">
-        <x:v>198</x:v>
       </x:c>
       <x:c r="D29" s="6" t="s">
         <x:v>46</x:v>
       </x:c>
       <x:c r="E29" s="7" t="s">
-        <x:v>125</x:v>
+        <x:v>122</x:v>
       </x:c>
       <x:c r="F29" s="7" t="s">
-        <x:v>126</x:v>
+        <x:v>123</x:v>
       </x:c>
       <x:c r="G29" s="6" t="s">
-        <x:v>199</x:v>
+        <x:v>196</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="42" customHeight="1">
       <x:c r="A30" s="5" t="s">
-        <x:v>200</x:v>
+        <x:v>197</x:v>
       </x:c>
       <x:c r="B30" s="5" t="s">
-        <x:v>201</x:v>
+        <x:v>198</x:v>
       </x:c>
       <x:c r="C30" s="5" t="s">
-        <x:v>202</x:v>
+        <x:v>199</x:v>
       </x:c>
       <x:c r="D30" s="5" t="s">
         <x:v>46</x:v>
       </x:c>
       <x:c r="E30" s="7" t="s">
-        <x:v>125</x:v>
+        <x:v>122</x:v>
       </x:c>
       <x:c r="F30" s="7" t="s">
-        <x:v>126</x:v>
+        <x:v>123</x:v>
       </x:c>
       <x:c r="G30" s="5" t="s">
-        <x:v>139</x:v>
+        <x:v>136</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="42" customHeight="1">
       <x:c r="A31" s="6" t="s">
-        <x:v>203</x:v>
+        <x:v>200</x:v>
       </x:c>
       <x:c r="B31" s="6" t="s">
-        <x:v>204</x:v>
+        <x:v>201</x:v>
       </x:c>
       <x:c r="C31" s="6" t="s">
-        <x:v>205</x:v>
+        <x:v>202</x:v>
       </x:c>
       <x:c r="D31" s="6" t="s">
         <x:v>46</x:v>
       </x:c>
       <x:c r="E31" s="7" t="s">
-        <x:v>125</x:v>
+        <x:v>122</x:v>
       </x:c>
       <x:c r="F31" s="7" t="s">
-        <x:v>126</x:v>
+        <x:v>123</x:v>
       </x:c>
       <x:c r="G31" s="6" t="s">
-        <x:v>206</x:v>
+        <x:v>203</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -3684,7 +3669,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R31cc3e629c0a4e17"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R04146f0ed12842bf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3713,7 +3698,7 @@
     </x:row>
     <x:row r="2" ht="21">
       <x:c r="A2" s="2" t="s">
-        <x:v>207</x:v>
+        <x:v>204</x:v>
       </x:c>
       <x:c r="B2" s="1"/>
       <x:c r="C2" s="1"/>
@@ -3724,7 +3709,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="3" t="s">
-        <x:v>208</x:v>
+        <x:v>205</x:v>
       </x:c>
       <x:c r="B3" s="1"/>
       <x:c r="C3" s="1"/>
@@ -3744,145 +3729,145 @@
     </x:row>
     <x:row r="5" ht="37.95000076293945" customHeight="1">
       <x:c r="A5" s="4" t="s">
+        <x:v>206</x:v>
+      </x:c>
+      <x:c r="B5" s="4" t="s">
+        <x:v>207</x:v>
+      </x:c>
+      <x:c r="C5" s="4" t="s">
+        <x:v>208</x:v>
+      </x:c>
+      <x:c r="D5" s="4" t="s">
         <x:v>209</x:v>
       </x:c>
-      <x:c r="B5" s="4" t="s">
+      <x:c r="E5" s="4" t="s">
         <x:v>210</x:v>
       </x:c>
-      <x:c r="C5" s="4" t="s">
+      <x:c r="F5" s="4" t="s">
         <x:v>211</x:v>
       </x:c>
-      <x:c r="D5" s="4" t="s">
+      <x:c r="G5" s="4" t="s">
         <x:v>212</x:v>
-      </x:c>
-      <x:c r="E5" s="4" t="s">
-        <x:v>213</x:v>
-      </x:c>
-      <x:c r="F5" s="4" t="s">
-        <x:v>214</x:v>
-      </x:c>
-      <x:c r="G5" s="4" t="s">
-        <x:v>215</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="42" customHeight="1">
       <x:c r="A6" s="5" t="s">
+        <x:v>213</x:v>
+      </x:c>
+      <x:c r="B6" s="5" t="s">
+        <x:v>214</x:v>
+      </x:c>
+      <x:c r="C6" s="5" t="s">
+        <x:v>215</x:v>
+      </x:c>
+      <x:c r="D6" s="5" t="s">
         <x:v>216</x:v>
       </x:c>
-      <x:c r="B6" s="5" t="s">
+      <x:c r="E6" s="5" t="s">
         <x:v>217</x:v>
       </x:c>
-      <x:c r="C6" s="5" t="s">
+      <x:c r="F6" s="7" t="s">
         <x:v>218</x:v>
       </x:c>
-      <x:c r="D6" s="5" t="s">
+      <x:c r="G6" s="7" t="s">
         <x:v>219</x:v>
-      </x:c>
-      <x:c r="E6" s="5" t="s">
-        <x:v>220</x:v>
-      </x:c>
-      <x:c r="F6" s="7" t="s">
-        <x:v>221</x:v>
-      </x:c>
-      <x:c r="G6" s="7" t="s">
-        <x:v>222</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="42" customHeight="1">
       <x:c r="A7" s="6" t="s">
+        <x:v>220</x:v>
+      </x:c>
+      <x:c r="B7" s="6" t="s">
+        <x:v>221</x:v>
+      </x:c>
+      <x:c r="C7" s="6" t="s">
+        <x:v>222</x:v>
+      </x:c>
+      <x:c r="D7" s="6" t="s">
         <x:v>223</x:v>
       </x:c>
-      <x:c r="B7" s="6" t="s">
+      <x:c r="E7" s="6" t="s">
         <x:v>224</x:v>
       </x:c>
-      <x:c r="C7" s="6" t="s">
-        <x:v>225</x:v>
-      </x:c>
-      <x:c r="D7" s="6" t="s">
-        <x:v>226</x:v>
-      </x:c>
-      <x:c r="E7" s="6" t="s">
-        <x:v>227</x:v>
-      </x:c>
       <x:c r="F7" s="7" t="s">
-        <x:v>221</x:v>
+        <x:v>218</x:v>
       </x:c>
       <x:c r="G7" s="7" t="s">
-        <x:v>222</x:v>
+        <x:v>219</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="42" customHeight="1">
       <x:c r="A8" s="5" t="s">
+        <x:v>225</x:v>
+      </x:c>
+      <x:c r="B8" s="5" t="s">
+        <x:v>226</x:v>
+      </x:c>
+      <x:c r="C8" s="5" t="s">
+        <x:v>227</x:v>
+      </x:c>
+      <x:c r="D8" s="5" t="s">
         <x:v>228</x:v>
       </x:c>
-      <x:c r="B8" s="5" t="s">
-        <x:v>229</x:v>
-      </x:c>
-      <x:c r="C8" s="5" t="s">
-        <x:v>230</x:v>
-      </x:c>
-      <x:c r="D8" s="5" t="s">
-        <x:v>231</x:v>
-      </x:c>
       <x:c r="E8" s="5" t="s">
-        <x:v>227</x:v>
+        <x:v>224</x:v>
       </x:c>
       <x:c r="F8" s="7" t="s">
-        <x:v>221</x:v>
+        <x:v>218</x:v>
       </x:c>
       <x:c r="G8" s="7" t="s">
-        <x:v>222</x:v>
+        <x:v>219</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="42" customHeight="1">
       <x:c r="A9" s="6" t="s">
+        <x:v>229</x:v>
+      </x:c>
+      <x:c r="B9" s="6" t="s">
+        <x:v>230</x:v>
+      </x:c>
+      <x:c r="C9" s="6" t="s">
+        <x:v>231</x:v>
+      </x:c>
+      <x:c r="D9" s="6" t="s">
         <x:v>232</x:v>
       </x:c>
-      <x:c r="B9" s="6" t="s">
-        <x:v>233</x:v>
-      </x:c>
-      <x:c r="C9" s="6" t="s">
-        <x:v>234</x:v>
-      </x:c>
-      <x:c r="D9" s="6" t="s">
-        <x:v>235</x:v>
-      </x:c>
       <x:c r="E9" s="6" t="s">
-        <x:v>227</x:v>
+        <x:v>224</x:v>
       </x:c>
       <x:c r="F9" s="7" t="s">
-        <x:v>221</x:v>
+        <x:v>218</x:v>
       </x:c>
       <x:c r="G9" s="7" t="s">
-        <x:v>222</x:v>
+        <x:v>219</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="42" customHeight="1">
       <x:c r="A10" s="5" t="s">
+        <x:v>233</x:v>
+      </x:c>
+      <x:c r="B10" s="5" t="s">
+        <x:v>234</x:v>
+      </x:c>
+      <x:c r="C10" s="5" t="s">
+        <x:v>235</x:v>
+      </x:c>
+      <x:c r="D10" s="5" t="s">
         <x:v>236</x:v>
       </x:c>
-      <x:c r="B10" s="5" t="s">
-        <x:v>237</x:v>
-      </x:c>
-      <x:c r="C10" s="5" t="s">
-        <x:v>238</x:v>
-      </x:c>
-      <x:c r="D10" s="5" t="s">
-        <x:v>239</x:v>
-      </x:c>
       <x:c r="E10" s="5" t="s">
-        <x:v>227</x:v>
+        <x:v>224</x:v>
       </x:c>
       <x:c r="F10" s="7" t="s">
-        <x:v>221</x:v>
+        <x:v>218</x:v>
       </x:c>
       <x:c r="G10" s="7" t="s">
-        <x:v>222</x:v>
+        <x:v>219</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="85" customHeight="1">
       <x:c r="A11" s="6" t="s">
-        <x:v>240</x:v>
+        <x:v>237</x:v>
       </x:c>
       <x:c r="B11" s="6" t="str">
         <x:v>dev地址／正式切换方案已定</x:v>
@@ -3891,369 +3876,369 @@
         <x:v>正式URL保持 juniperphoton.dev/photoncam/；中英深层页面直接访问及刷新成功，资源无迁移引入的404。</x:v>
       </x:c>
       <x:c r="D11" s="6" t="s">
-        <x:v>241</x:v>
+        <x:v>238</x:v>
       </x:c>
       <x:c r="E11" s="6" t="s">
-        <x:v>227</x:v>
+        <x:v>224</x:v>
       </x:c>
       <x:c r="F11" s="7" t="s">
-        <x:v>221</x:v>
+        <x:v>218</x:v>
       </x:c>
       <x:c r="G11" s="7" t="s">
-        <x:v>222</x:v>
+        <x:v>219</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="42" customHeight="1">
       <x:c r="A12" s="5" t="s">
+        <x:v>239</x:v>
+      </x:c>
+      <x:c r="B12" s="5" t="s">
+        <x:v>240</x:v>
+      </x:c>
+      <x:c r="C12" s="5" t="s">
+        <x:v>241</x:v>
+      </x:c>
+      <x:c r="D12" s="5" t="s">
         <x:v>242</x:v>
       </x:c>
-      <x:c r="B12" s="5" t="s">
-        <x:v>243</x:v>
-      </x:c>
-      <x:c r="C12" s="5" t="s">
-        <x:v>244</x:v>
-      </x:c>
-      <x:c r="D12" s="5" t="s">
-        <x:v>245</x:v>
-      </x:c>
       <x:c r="E12" s="5" t="s">
-        <x:v>227</x:v>
+        <x:v>224</x:v>
       </x:c>
       <x:c r="F12" s="7" t="s">
-        <x:v>221</x:v>
+        <x:v>218</x:v>
       </x:c>
       <x:c r="G12" s="7" t="s">
-        <x:v>222</x:v>
+        <x:v>219</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="42" customHeight="1">
       <x:c r="A13" s="6" t="s">
+        <x:v>243</x:v>
+      </x:c>
+      <x:c r="B13" s="6" t="s">
+        <x:v>244</x:v>
+      </x:c>
+      <x:c r="C13" s="6" t="s">
+        <x:v>245</x:v>
+      </x:c>
+      <x:c r="D13" s="6" t="s">
         <x:v>246</x:v>
       </x:c>
-      <x:c r="B13" s="6" t="s">
+      <x:c r="E13" s="6" t="s">
         <x:v>247</x:v>
       </x:c>
-      <x:c r="C13" s="6" t="s">
-        <x:v>248</x:v>
-      </x:c>
-      <x:c r="D13" s="6" t="s">
-        <x:v>249</x:v>
-      </x:c>
-      <x:c r="E13" s="6" t="s">
-        <x:v>250</x:v>
-      </x:c>
       <x:c r="F13" s="7" t="s">
-        <x:v>221</x:v>
+        <x:v>218</x:v>
       </x:c>
       <x:c r="G13" s="7" t="s">
-        <x:v>222</x:v>
+        <x:v>219</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="42" customHeight="1">
       <x:c r="A14" s="5" t="s">
+        <x:v>248</x:v>
+      </x:c>
+      <x:c r="B14" s="5" t="s">
+        <x:v>249</x:v>
+      </x:c>
+      <x:c r="C14" s="5" t="s">
+        <x:v>250</x:v>
+      </x:c>
+      <x:c r="D14" s="5" t="s">
         <x:v>251</x:v>
       </x:c>
-      <x:c r="B14" s="5" t="s">
-        <x:v>252</x:v>
-      </x:c>
-      <x:c r="C14" s="5" t="s">
-        <x:v>253</x:v>
-      </x:c>
-      <x:c r="D14" s="5" t="s">
-        <x:v>254</x:v>
-      </x:c>
       <x:c r="E14" s="5" t="s">
-        <x:v>250</x:v>
+        <x:v>247</x:v>
       </x:c>
       <x:c r="F14" s="7" t="s">
-        <x:v>221</x:v>
+        <x:v>218</x:v>
       </x:c>
       <x:c r="G14" s="7" t="s">
-        <x:v>222</x:v>
+        <x:v>219</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="42" customHeight="1">
       <x:c r="A15" s="6" t="s">
+        <x:v>252</x:v>
+      </x:c>
+      <x:c r="B15" s="6" t="s">
+        <x:v>253</x:v>
+      </x:c>
+      <x:c r="C15" s="6" t="s">
+        <x:v>254</x:v>
+      </x:c>
+      <x:c r="D15" s="6" t="s">
         <x:v>255</x:v>
       </x:c>
-      <x:c r="B15" s="6" t="s">
+      <x:c r="E15" s="6" t="s">
         <x:v>256</x:v>
       </x:c>
-      <x:c r="C15" s="6" t="s">
-        <x:v>257</x:v>
-      </x:c>
-      <x:c r="D15" s="6" t="s">
-        <x:v>258</x:v>
-      </x:c>
-      <x:c r="E15" s="6" t="s">
-        <x:v>259</x:v>
-      </x:c>
       <x:c r="F15" s="7" t="s">
-        <x:v>221</x:v>
+        <x:v>218</x:v>
       </x:c>
       <x:c r="G15" s="7" t="s">
-        <x:v>222</x:v>
+        <x:v>219</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="42" customHeight="1">
       <x:c r="A16" s="5" t="s">
+        <x:v>257</x:v>
+      </x:c>
+      <x:c r="B16" s="5" t="s">
+        <x:v>258</x:v>
+      </x:c>
+      <x:c r="C16" s="5" t="s">
+        <x:v>259</x:v>
+      </x:c>
+      <x:c r="D16" s="5" t="s">
         <x:v>260</x:v>
       </x:c>
-      <x:c r="B16" s="5" t="s">
-        <x:v>261</x:v>
-      </x:c>
-      <x:c r="C16" s="5" t="s">
-        <x:v>262</x:v>
-      </x:c>
-      <x:c r="D16" s="5" t="s">
-        <x:v>263</x:v>
-      </x:c>
       <x:c r="E16" s="5" t="s">
-        <x:v>259</x:v>
+        <x:v>256</x:v>
       </x:c>
       <x:c r="F16" s="7" t="s">
-        <x:v>221</x:v>
+        <x:v>218</x:v>
       </x:c>
       <x:c r="G16" s="7" t="s">
-        <x:v>222</x:v>
+        <x:v>219</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="42" customHeight="1">
       <x:c r="A17" s="6" t="s">
+        <x:v>261</x:v>
+      </x:c>
+      <x:c r="B17" s="6" t="s">
+        <x:v>262</x:v>
+      </x:c>
+      <x:c r="C17" s="6" t="s">
+        <x:v>263</x:v>
+      </x:c>
+      <x:c r="D17" s="6" t="s">
         <x:v>264</x:v>
       </x:c>
-      <x:c r="B17" s="6" t="s">
-        <x:v>265</x:v>
-      </x:c>
-      <x:c r="C17" s="6" t="s">
-        <x:v>266</x:v>
-      </x:c>
-      <x:c r="D17" s="6" t="s">
-        <x:v>267</x:v>
-      </x:c>
       <x:c r="E17" s="6" t="s">
-        <x:v>259</x:v>
+        <x:v>256</x:v>
       </x:c>
       <x:c r="F17" s="7" t="s">
-        <x:v>221</x:v>
+        <x:v>218</x:v>
       </x:c>
       <x:c r="G17" s="7" t="s">
-        <x:v>222</x:v>
+        <x:v>219</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="42" customHeight="1">
       <x:c r="A18" s="5" t="s">
+        <x:v>265</x:v>
+      </x:c>
+      <x:c r="B18" s="5" t="s">
+        <x:v>266</x:v>
+      </x:c>
+      <x:c r="C18" s="5" t="s">
+        <x:v>267</x:v>
+      </x:c>
+      <x:c r="D18" s="5" t="s">
         <x:v>268</x:v>
       </x:c>
-      <x:c r="B18" s="5" t="s">
-        <x:v>269</x:v>
-      </x:c>
-      <x:c r="C18" s="5" t="s">
-        <x:v>270</x:v>
-      </x:c>
-      <x:c r="D18" s="5" t="s">
-        <x:v>271</x:v>
-      </x:c>
       <x:c r="E18" s="5" t="s">
-        <x:v>259</x:v>
+        <x:v>256</x:v>
       </x:c>
       <x:c r="F18" s="7" t="s">
-        <x:v>221</x:v>
+        <x:v>218</x:v>
       </x:c>
       <x:c r="G18" s="7" t="s">
-        <x:v>222</x:v>
+        <x:v>219</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="42" customHeight="1">
       <x:c r="A19" s="6" t="s">
+        <x:v>269</x:v>
+      </x:c>
+      <x:c r="B19" s="6" t="s">
+        <x:v>270</x:v>
+      </x:c>
+      <x:c r="C19" s="6" t="s">
+        <x:v>271</x:v>
+      </x:c>
+      <x:c r="D19" s="6" t="s">
         <x:v>272</x:v>
       </x:c>
-      <x:c r="B19" s="6" t="s">
+      <x:c r="E19" s="6" t="s">
         <x:v>273</x:v>
       </x:c>
-      <x:c r="C19" s="6" t="s">
-        <x:v>274</x:v>
-      </x:c>
-      <x:c r="D19" s="6" t="s">
-        <x:v>275</x:v>
-      </x:c>
-      <x:c r="E19" s="6" t="s">
-        <x:v>276</x:v>
-      </x:c>
       <x:c r="F19" s="7" t="s">
-        <x:v>221</x:v>
+        <x:v>218</x:v>
       </x:c>
       <x:c r="G19" s="7" t="s">
-        <x:v>222</x:v>
+        <x:v>219</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="42" customHeight="1">
       <x:c r="A20" s="5" t="s">
+        <x:v>274</x:v>
+      </x:c>
+      <x:c r="B20" s="5" t="s">
+        <x:v>275</x:v>
+      </x:c>
+      <x:c r="C20" s="5" t="s">
+        <x:v>276</x:v>
+      </x:c>
+      <x:c r="D20" s="5" t="s">
         <x:v>277</x:v>
       </x:c>
-      <x:c r="B20" s="5" t="s">
+      <x:c r="E20" s="5" t="s">
         <x:v>278</x:v>
       </x:c>
-      <x:c r="C20" s="5" t="s">
-        <x:v>279</x:v>
-      </x:c>
-      <x:c r="D20" s="5" t="s">
-        <x:v>280</x:v>
-      </x:c>
-      <x:c r="E20" s="5" t="s">
-        <x:v>281</x:v>
-      </x:c>
       <x:c r="F20" s="7" t="s">
-        <x:v>221</x:v>
+        <x:v>218</x:v>
       </x:c>
       <x:c r="G20" s="7" t="s">
-        <x:v>222</x:v>
+        <x:v>219</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="42" customHeight="1">
       <x:c r="A21" s="6" t="s">
+        <x:v>279</x:v>
+      </x:c>
+      <x:c r="B21" s="6" t="s">
+        <x:v>280</x:v>
+      </x:c>
+      <x:c r="C21" s="6" t="s">
+        <x:v>281</x:v>
+      </x:c>
+      <x:c r="D21" s="6" t="s">
         <x:v>282</x:v>
       </x:c>
-      <x:c r="B21" s="6" t="s">
-        <x:v>283</x:v>
-      </x:c>
-      <x:c r="C21" s="6" t="s">
-        <x:v>284</x:v>
-      </x:c>
-      <x:c r="D21" s="6" t="s">
-        <x:v>285</x:v>
-      </x:c>
       <x:c r="E21" s="6" t="s">
-        <x:v>227</x:v>
+        <x:v>224</x:v>
       </x:c>
       <x:c r="F21" s="7" t="s">
-        <x:v>221</x:v>
+        <x:v>218</x:v>
       </x:c>
       <x:c r="G21" s="7" t="s">
-        <x:v>222</x:v>
+        <x:v>219</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="42" customHeight="1">
       <x:c r="A22" s="5" t="s">
+        <x:v>283</x:v>
+      </x:c>
+      <x:c r="B22" s="5" t="s">
+        <x:v>284</x:v>
+      </x:c>
+      <x:c r="C22" s="5" t="s">
+        <x:v>285</x:v>
+      </x:c>
+      <x:c r="D22" s="5" t="s">
         <x:v>286</x:v>
       </x:c>
-      <x:c r="B22" s="5" t="s">
-        <x:v>287</x:v>
-      </x:c>
-      <x:c r="C22" s="5" t="s">
-        <x:v>288</x:v>
-      </x:c>
-      <x:c r="D22" s="5" t="s">
-        <x:v>289</x:v>
-      </x:c>
       <x:c r="E22" s="5" t="s">
-        <x:v>227</x:v>
+        <x:v>224</x:v>
       </x:c>
       <x:c r="F22" s="7" t="s">
-        <x:v>221</x:v>
+        <x:v>218</x:v>
       </x:c>
       <x:c r="G22" s="7" t="s">
-        <x:v>222</x:v>
+        <x:v>219</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="42" customHeight="1">
       <x:c r="A23" s="6" t="s">
+        <x:v>287</x:v>
+      </x:c>
+      <x:c r="B23" s="6" t="s">
+        <x:v>288</x:v>
+      </x:c>
+      <x:c r="C23" s="6" t="s">
+        <x:v>289</x:v>
+      </x:c>
+      <x:c r="D23" s="6" t="s">
         <x:v>290</x:v>
       </x:c>
-      <x:c r="B23" s="6" t="s">
-        <x:v>291</x:v>
-      </x:c>
-      <x:c r="C23" s="6" t="s">
-        <x:v>292</x:v>
-      </x:c>
-      <x:c r="D23" s="6" t="s">
-        <x:v>293</x:v>
-      </x:c>
       <x:c r="E23" s="6" t="s">
-        <x:v>220</x:v>
+        <x:v>217</x:v>
       </x:c>
       <x:c r="F23" s="7" t="s">
-        <x:v>221</x:v>
+        <x:v>218</x:v>
       </x:c>
       <x:c r="G23" s="7" t="s">
-        <x:v>222</x:v>
+        <x:v>219</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="42" customHeight="1">
       <x:c r="A24" s="5" t="s">
+        <x:v>291</x:v>
+      </x:c>
+      <x:c r="B24" s="5" t="s">
+        <x:v>292</x:v>
+      </x:c>
+      <x:c r="C24" s="5" t="s">
+        <x:v>293</x:v>
+      </x:c>
+      <x:c r="D24" s="5" t="s">
         <x:v>294</x:v>
       </x:c>
-      <x:c r="B24" s="5" t="s">
+      <x:c r="E24" s="5" t="s">
         <x:v>295</x:v>
       </x:c>
-      <x:c r="C24" s="5" t="s">
-        <x:v>296</x:v>
-      </x:c>
-      <x:c r="D24" s="5" t="s">
-        <x:v>297</x:v>
-      </x:c>
-      <x:c r="E24" s="5" t="s">
-        <x:v>298</x:v>
-      </x:c>
       <x:c r="F24" s="7" t="s">
-        <x:v>221</x:v>
+        <x:v>218</x:v>
       </x:c>
       <x:c r="G24" s="7" t="s">
-        <x:v>222</x:v>
+        <x:v>219</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="42" customHeight="1">
       <x:c r="A25" s="6" t="s">
+        <x:v>296</x:v>
+      </x:c>
+      <x:c r="B25" s="6" t="s">
+        <x:v>297</x:v>
+      </x:c>
+      <x:c r="C25" s="6" t="s">
+        <x:v>298</x:v>
+      </x:c>
+      <x:c r="D25" s="6" t="s">
         <x:v>299</x:v>
       </x:c>
-      <x:c r="B25" s="6" t="s">
-        <x:v>300</x:v>
-      </x:c>
-      <x:c r="C25" s="6" t="s">
-        <x:v>301</x:v>
-      </x:c>
-      <x:c r="D25" s="6" t="s">
-        <x:v>302</x:v>
-      </x:c>
       <x:c r="E25" s="6" t="s">
-        <x:v>220</x:v>
+        <x:v>217</x:v>
       </x:c>
       <x:c r="F25" s="7" t="s">
-        <x:v>221</x:v>
+        <x:v>218</x:v>
       </x:c>
       <x:c r="G25" s="7" t="s">
-        <x:v>222</x:v>
+        <x:v>219</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="42" customHeight="1">
       <x:c r="A26" s="5" t="s">
+        <x:v>300</x:v>
+      </x:c>
+      <x:c r="B26" s="5" t="s">
+        <x:v>301</x:v>
+      </x:c>
+      <x:c r="C26" s="5" t="s">
+        <x:v>302</x:v>
+      </x:c>
+      <x:c r="D26" s="5" t="s">
         <x:v>303</x:v>
       </x:c>
-      <x:c r="B26" s="5" t="s">
+      <x:c r="E26" s="5" t="s">
+        <x:v>224</x:v>
+      </x:c>
+      <x:c r="F26" s="7" t="s">
+        <x:v>218</x:v>
+      </x:c>
+      <x:c r="G26" s="7" t="s">
+        <x:v>219</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="95" customHeight="1">
+      <x:c r="A27" s="6" t="s">
         <x:v>304</x:v>
       </x:c>
-      <x:c r="C26" s="5" t="s">
-        <x:v>305</x:v>
-      </x:c>
-      <x:c r="D26" s="5" t="s">
-        <x:v>306</x:v>
-      </x:c>
-      <x:c r="E26" s="5" t="s">
-        <x:v>227</x:v>
-      </x:c>
-      <x:c r="F26" s="7" t="s">
-        <x:v>221</x:v>
-      </x:c>
-      <x:c r="G26" s="7" t="s">
-        <x:v>222</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="27" ht="85" customHeight="1">
-      <x:c r="A27" s="6" t="s">
-        <x:v>307</x:v>
-      </x:c>
-      <x:c r="B27" s="6" t="s">
-        <x:v>308</x:v>
+      <x:c r="B27" s="6" t="str">
+        <x:v>dev验收及正式源码仓库、分支与授权确认完成</x:v>
       </x:c>
       <x:c r="C27" s="6" t="str">
         <x:v>迁移计划与切换回退演练通过；切换前后核对根首页、主站脚本图标、4个其他App入口及返回主站链接正常。</x:v>
@@ -4262,105 +4247,105 @@
         <x:v>迁移计划、DNS记录、演练与主站回归记录</x:v>
       </x:c>
       <x:c r="E27" s="6" t="s">
-        <x:v>309</x:v>
+        <x:v>305</x:v>
       </x:c>
       <x:c r="F27" s="7" t="s">
-        <x:v>221</x:v>
+        <x:v>218</x:v>
       </x:c>
       <x:c r="G27" s="7" t="s">
-        <x:v>222</x:v>
+        <x:v>219</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="42" customHeight="1">
       <x:c r="A28" s="5" t="s">
+        <x:v>306</x:v>
+      </x:c>
+      <x:c r="B28" s="5" t="s">
+        <x:v>307</x:v>
+      </x:c>
+      <x:c r="C28" s="5" t="s">
+        <x:v>308</x:v>
+      </x:c>
+      <x:c r="D28" s="5" t="s">
+        <x:v>309</x:v>
+      </x:c>
+      <x:c r="E28" s="5" t="s">
         <x:v>310</x:v>
       </x:c>
-      <x:c r="B28" s="5" t="s">
-        <x:v>311</x:v>
-      </x:c>
-      <x:c r="C28" s="5" t="s">
-        <x:v>312</x:v>
-      </x:c>
-      <x:c r="D28" s="5" t="s">
-        <x:v>313</x:v>
-      </x:c>
-      <x:c r="E28" s="5" t="s">
-        <x:v>314</x:v>
-      </x:c>
       <x:c r="F28" s="7" t="s">
-        <x:v>221</x:v>
+        <x:v>218</x:v>
       </x:c>
       <x:c r="G28" s="7" t="s">
-        <x:v>222</x:v>
+        <x:v>219</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="42" customHeight="1">
       <x:c r="A29" s="6" t="s">
+        <x:v>311</x:v>
+      </x:c>
+      <x:c r="B29" s="6" t="s">
+        <x:v>312</x:v>
+      </x:c>
+      <x:c r="C29" s="6" t="s">
+        <x:v>313</x:v>
+      </x:c>
+      <x:c r="D29" s="6" t="s">
+        <x:v>314</x:v>
+      </x:c>
+      <x:c r="E29" s="6" t="s">
         <x:v>315</x:v>
       </x:c>
-      <x:c r="B29" s="6" t="s">
-        <x:v>316</x:v>
-      </x:c>
-      <x:c r="C29" s="6" t="s">
-        <x:v>317</x:v>
-      </x:c>
-      <x:c r="D29" s="6" t="s">
-        <x:v>318</x:v>
-      </x:c>
-      <x:c r="E29" s="6" t="s">
-        <x:v>319</x:v>
-      </x:c>
       <x:c r="F29" s="7" t="s">
-        <x:v>221</x:v>
+        <x:v>218</x:v>
       </x:c>
       <x:c r="G29" s="7" t="s">
-        <x:v>222</x:v>
+        <x:v>219</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="42" customHeight="1">
       <x:c r="A30" s="5" t="s">
+        <x:v>316</x:v>
+      </x:c>
+      <x:c r="B30" s="5" t="s">
+        <x:v>317</x:v>
+      </x:c>
+      <x:c r="C30" s="5" t="s">
+        <x:v>318</x:v>
+      </x:c>
+      <x:c r="D30" s="5" t="s">
+        <x:v>319</x:v>
+      </x:c>
+      <x:c r="E30" s="5" t="s">
         <x:v>320</x:v>
       </x:c>
-      <x:c r="B30" s="5" t="s">
-        <x:v>321</x:v>
-      </x:c>
-      <x:c r="C30" s="5" t="s">
-        <x:v>322</x:v>
-      </x:c>
-      <x:c r="D30" s="5" t="s">
-        <x:v>323</x:v>
-      </x:c>
-      <x:c r="E30" s="5" t="s">
-        <x:v>324</x:v>
-      </x:c>
       <x:c r="F30" s="7" t="s">
-        <x:v>221</x:v>
+        <x:v>218</x:v>
       </x:c>
       <x:c r="G30" s="7" t="s">
-        <x:v>222</x:v>
+        <x:v>219</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="42" customHeight="1">
       <x:c r="A31" s="6" t="s">
-        <x:v>325</x:v>
+        <x:v>321</x:v>
       </x:c>
       <x:c r="B31" s="6" t="s">
-        <x:v>326</x:v>
+        <x:v>322</x:v>
       </x:c>
       <x:c r="C31" s="6" t="s">
-        <x:v>327</x:v>
+        <x:v>323</x:v>
       </x:c>
       <x:c r="D31" s="6" t="s">
-        <x:v>328</x:v>
+        <x:v>324</x:v>
       </x:c>
       <x:c r="E31" s="6" t="s">
-        <x:v>276</x:v>
+        <x:v>273</x:v>
       </x:c>
       <x:c r="F31" s="7" t="s">
-        <x:v>221</x:v>
+        <x:v>218</x:v>
       </x:c>
       <x:c r="G31" s="7" t="s">
-        <x:v>222</x:v>
+        <x:v>219</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -4371,7 +4356,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Red3665f8452a41be"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2d67f2d6acb2410e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4404,7 +4389,7 @@
     </x:row>
     <x:row r="2" ht="21">
       <x:c r="A2" s="2" t="s">
-        <x:v>329</x:v>
+        <x:v>325</x:v>
       </x:c>
       <x:c r="B2" s="1"/>
       <x:c r="C2" s="1"/>
@@ -4417,7 +4402,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="3" t="s">
-        <x:v>330</x:v>
+        <x:v>326</x:v>
       </x:c>
       <x:c r="B3" s="1"/>
       <x:c r="C3" s="1"/>
@@ -4441,54 +4426,54 @@
     </x:row>
     <x:row r="5" ht="37.95000076293945" customHeight="1">
       <x:c r="A5" s="4" t="s">
+        <x:v>327</x:v>
+      </x:c>
+      <x:c r="B5" s="4" t="s">
+        <x:v>328</x:v>
+      </x:c>
+      <x:c r="C5" s="4" t="s">
+        <x:v>329</x:v>
+      </x:c>
+      <x:c r="D5" s="4" t="s">
+        <x:v>330</x:v>
+      </x:c>
+      <x:c r="E5" s="4" t="s">
         <x:v>331</x:v>
       </x:c>
-      <x:c r="B5" s="4" t="s">
+      <x:c r="F5" s="4" t="s">
         <x:v>332</x:v>
       </x:c>
-      <x:c r="C5" s="4" t="s">
+      <x:c r="G5" s="4" t="s">
         <x:v>333</x:v>
       </x:c>
-      <x:c r="D5" s="4" t="s">
+      <x:c r="H5" s="4" t="s">
         <x:v>334</x:v>
       </x:c>
-      <x:c r="E5" s="4" t="s">
+      <x:c r="I5" s="4" t="s">
         <x:v>335</x:v>
-      </x:c>
-      <x:c r="F5" s="4" t="s">
-        <x:v>336</x:v>
-      </x:c>
-      <x:c r="G5" s="4" t="s">
-        <x:v>337</x:v>
-      </x:c>
-      <x:c r="H5" s="4" t="s">
-        <x:v>338</x:v>
-      </x:c>
-      <x:c r="I5" s="4" t="s">
-        <x:v>339</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="85" customHeight="1">
       <x:c r="A6" s="5" t="s">
-        <x:v>127</x:v>
+        <x:v>124</x:v>
       </x:c>
       <x:c r="B6" s="5" t="s">
+        <x:v>336</x:v>
+      </x:c>
+      <x:c r="C6" s="5" t="s">
+        <x:v>337</x:v>
+      </x:c>
+      <x:c r="D6" s="5" t="s">
+        <x:v>338</x:v>
+      </x:c>
+      <x:c r="E6" s="5" t="s">
+        <x:v>339</x:v>
+      </x:c>
+      <x:c r="F6" s="5" t="s">
         <x:v>340</x:v>
       </x:c>
-      <x:c r="C6" s="5" t="s">
+      <x:c r="G6" s="5" t="s">
         <x:v>341</x:v>
-      </x:c>
-      <x:c r="D6" s="5" t="s">
-        <x:v>342</x:v>
-      </x:c>
-      <x:c r="E6" s="5" t="s">
-        <x:v>343</x:v>
-      </x:c>
-      <x:c r="F6" s="5" t="s">
-        <x:v>344</x:v>
-      </x:c>
-      <x:c r="G6" s="5" t="s">
-        <x:v>345</x:v>
       </x:c>
       <x:c r="H6" s="7" t="s">
         <x:v>31</x:v>
@@ -4499,25 +4484,25 @@
     </x:row>
     <x:row r="7" ht="110" customHeight="1">
       <x:c r="A7" s="6" t="s">
-        <x:v>132</x:v>
+        <x:v>129</x:v>
       </x:c>
       <x:c r="B7" s="6" t="s">
-        <x:v>346</x:v>
+        <x:v>342</x:v>
       </x:c>
       <x:c r="C7" s="6" t="str">
         <x:v>路径与域名已定；待确认权威DNS管理方、解析与变更权限、主站保留及切换回退方式。</x:v>
       </x:c>
       <x:c r="D7" s="6" t="s">
-        <x:v>347</x:v>
+        <x:v>343</x:v>
       </x:c>
       <x:c r="E7" s="6" t="s">
-        <x:v>348</x:v>
+        <x:v>344</x:v>
       </x:c>
       <x:c r="F7" s="6" t="s">
-        <x:v>344</x:v>
+        <x:v>340</x:v>
       </x:c>
       <x:c r="G7" s="6" t="s">
-        <x:v>345</x:v>
+        <x:v>341</x:v>
       </x:c>
       <x:c r="H7" s="7" t="s">
         <x:v>31</x:v>
@@ -4528,25 +4513,25 @@
     </x:row>
     <x:row r="8" ht="42" customHeight="1">
       <x:c r="A8" s="5" t="s">
-        <x:v>136</x:v>
+        <x:v>133</x:v>
       </x:c>
       <x:c r="B8" s="5" t="s">
+        <x:v>345</x:v>
+      </x:c>
+      <x:c r="C8" s="5" t="s">
+        <x:v>346</x:v>
+      </x:c>
+      <x:c r="D8" s="5" t="s">
+        <x:v>347</x:v>
+      </x:c>
+      <x:c r="E8" s="5" t="s">
+        <x:v>348</x:v>
+      </x:c>
+      <x:c r="F8" s="5" t="s">
+        <x:v>340</x:v>
+      </x:c>
+      <x:c r="G8" s="5" t="s">
         <x:v>349</x:v>
-      </x:c>
-      <x:c r="C8" s="5" t="s">
-        <x:v>350</x:v>
-      </x:c>
-      <x:c r="D8" s="5" t="s">
-        <x:v>351</x:v>
-      </x:c>
-      <x:c r="E8" s="5" t="s">
-        <x:v>352</x:v>
-      </x:c>
-      <x:c r="F8" s="5" t="s">
-        <x:v>344</x:v>
-      </x:c>
-      <x:c r="G8" s="5" t="s">
-        <x:v>353</x:v>
       </x:c>
       <x:c r="H8" s="7" t="s">
         <x:v>31</x:v>
@@ -4555,22 +4540,22 @@
     </x:row>
     <x:row r="9" ht="110" customHeight="1">
       <x:c r="A9" s="6" t="s">
-        <x:v>150</x:v>
+        <x:v>147</x:v>
       </x:c>
       <x:c r="B9" s="6" t="s">
-        <x:v>354</x:v>
+        <x:v>350</x:v>
       </x:c>
       <x:c r="C9" s="6" t="str">
         <x:v>在dev部署练习中比较并固定Node/npm及依赖版本，实际构建后验证产物再部署。</x:v>
       </x:c>
       <x:c r="D9" s="6" t="s">
-        <x:v>355</x:v>
+        <x:v>351</x:v>
       </x:c>
       <x:c r="E9" s="6" t="s">
-        <x:v>356</x:v>
+        <x:v>352</x:v>
       </x:c>
       <x:c r="F9" s="6" t="s">
-        <x:v>357</x:v>
+        <x:v>353</x:v>
       </x:c>
       <x:c r="G9" s="6" t="str">
         <x:v>dev部署练习中，部署前</x:v>
@@ -4582,54 +4567,56 @@
         <x:v>2026-10-08用户约定：版本选择与干净构建留至dev练习确认。npm流程已说明，3.6.3/3.0.1/3.5.2差异仍未解决。</x:v>
       </x:c>
     </x:row>
-    <x:row r="10" ht="42" customHeight="1">
+    <x:row r="10" ht="110" customHeight="1">
       <x:c r="A10" s="5" t="s">
-        <x:v>159</x:v>
+        <x:v>156</x:v>
       </x:c>
       <x:c r="B10" s="5" t="s">
-        <x:v>358</x:v>
-      </x:c>
-      <x:c r="C10" s="5" t="s">
-        <x:v>359</x:v>
+        <x:v>354</x:v>
+      </x:c>
+      <x:c r="C10" s="5" t="str">
+        <x:v>dev用用户私有副本，正式用开发者私有原仓库；分别确认来源、触发分支、连接授权、发布与失败处理。</x:v>
       </x:c>
       <x:c r="D10" s="5" t="s">
-        <x:v>360</x:v>
+        <x:v>355</x:v>
       </x:c>
       <x:c r="E10" s="5" t="s">
-        <x:v>361</x:v>
-      </x:c>
-      <x:c r="F10" s="5" t="s">
-        <x:v>344</x:v>
-      </x:c>
-      <x:c r="G10" s="5" t="s">
-        <x:v>345</x:v>
+        <x:v>356</x:v>
+      </x:c>
+      <x:c r="F10" s="5" t="str">
+        <x:v>用户与原开发者／待确认</x:v>
+      </x:c>
+      <x:c r="G10" s="5" t="str">
+        <x:v>dev基本设计前／正式发布前</x:v>
       </x:c>
       <x:c r="H10" s="7" t="s">
         <x:v>31</x:v>
       </x:c>
-      <x:c r="I10" s="7"/>
+      <x:c r="I10" s="7" t="str">
+        <x:v>2026-10-13：用户确认两阶段源码来源；正式仓库URL、分支、连接权限及与dev版本差异尚未核验。</x:v>
+      </x:c>
     </x:row>
     <x:row r="11" ht="42" customHeight="1">
       <x:c r="A11" s="6" t="s">
-        <x:v>179</x:v>
+        <x:v>176</x:v>
       </x:c>
       <x:c r="B11" s="6" t="s">
-        <x:v>362</x:v>
+        <x:v>357</x:v>
       </x:c>
       <x:c r="C11" s="6" t="s">
-        <x:v>363</x:v>
+        <x:v>358</x:v>
       </x:c>
       <x:c r="D11" s="6" t="s">
-        <x:v>364</x:v>
+        <x:v>359</x:v>
       </x:c>
       <x:c r="E11" s="6" t="s">
-        <x:v>176</x:v>
+        <x:v>173</x:v>
       </x:c>
       <x:c r="F11" s="6" t="s">
-        <x:v>344</x:v>
+        <x:v>340</x:v>
       </x:c>
       <x:c r="G11" s="6" t="s">
-        <x:v>353</x:v>
+        <x:v>349</x:v>
       </x:c>
       <x:c r="H11" s="7" t="s">
         <x:v>31</x:v>
@@ -4638,25 +4625,25 @@
     </x:row>
     <x:row r="12" ht="42" customHeight="1">
       <x:c r="A12" s="5" t="s">
-        <x:v>183</x:v>
+        <x:v>180</x:v>
       </x:c>
       <x:c r="B12" s="5" t="s">
-        <x:v>365</x:v>
+        <x:v>360</x:v>
       </x:c>
       <x:c r="C12" s="5" t="s">
-        <x:v>366</x:v>
+        <x:v>361</x:v>
       </x:c>
       <x:c r="D12" s="5" t="s">
-        <x:v>367</x:v>
+        <x:v>362</x:v>
       </x:c>
       <x:c r="E12" s="5" t="s">
-        <x:v>368</x:v>
+        <x:v>363</x:v>
       </x:c>
       <x:c r="F12" s="5" t="s">
-        <x:v>344</x:v>
+        <x:v>340</x:v>
       </x:c>
       <x:c r="G12" s="5" t="s">
-        <x:v>369</x:v>
+        <x:v>364</x:v>
       </x:c>
       <x:c r="H12" s="7" t="s">
         <x:v>31</x:v>
@@ -4665,25 +4652,25 @@
     </x:row>
     <x:row r="13" ht="42" customHeight="1">
       <x:c r="A13" s="6" t="s">
-        <x:v>370</x:v>
+        <x:v>365</x:v>
       </x:c>
       <x:c r="B13" s="6" t="s">
-        <x:v>371</x:v>
+        <x:v>366</x:v>
       </x:c>
       <x:c r="C13" s="6" t="s">
-        <x:v>372</x:v>
+        <x:v>367</x:v>
       </x:c>
       <x:c r="D13" s="6" t="s">
-        <x:v>373</x:v>
+        <x:v>368</x:v>
       </x:c>
       <x:c r="E13" s="6" t="s">
-        <x:v>374</x:v>
+        <x:v>369</x:v>
       </x:c>
       <x:c r="F13" s="6" t="s">
-        <x:v>344</x:v>
+        <x:v>340</x:v>
       </x:c>
       <x:c r="G13" s="6" t="s">
-        <x:v>345</x:v>
+        <x:v>341</x:v>
       </x:c>
       <x:c r="H13" s="7" t="s">
         <x:v>31</x:v>
@@ -4692,25 +4679,25 @@
     </x:row>
     <x:row r="14" ht="42" customHeight="1">
       <x:c r="A14" s="5" t="s">
-        <x:v>164</x:v>
+        <x:v>161</x:v>
       </x:c>
       <x:c r="B14" s="5" t="s">
-        <x:v>185</x:v>
+        <x:v>182</x:v>
       </x:c>
       <x:c r="C14" s="5" t="s">
-        <x:v>375</x:v>
+        <x:v>370</x:v>
       </x:c>
       <x:c r="D14" s="5" t="s">
-        <x:v>376</x:v>
+        <x:v>371</x:v>
       </x:c>
       <x:c r="E14" s="5" t="s">
-        <x:v>377</x:v>
+        <x:v>372</x:v>
       </x:c>
       <x:c r="F14" s="5" t="s">
-        <x:v>344</x:v>
+        <x:v>340</x:v>
       </x:c>
       <x:c r="G14" s="5" t="s">
-        <x:v>345</x:v>
+        <x:v>341</x:v>
       </x:c>
       <x:c r="H14" s="7" t="s">
         <x:v>31</x:v>
@@ -4719,25 +4706,25 @@
     </x:row>
     <x:row r="15" ht="110" customHeight="1">
       <x:c r="A15" s="6" t="s">
-        <x:v>378</x:v>
+        <x:v>373</x:v>
       </x:c>
       <x:c r="B15" s="6" t="s">
-        <x:v>379</x:v>
+        <x:v>374</x:v>
       </x:c>
       <x:c r="C15" s="6" t="str">
         <x:v>依赖已说明；待核验原站路由／响应头、完整网络请求及切换批准与窗口。</x:v>
       </x:c>
       <x:c r="D15" s="6" t="s">
-        <x:v>380</x:v>
+        <x:v>375</x:v>
       </x:c>
       <x:c r="E15" s="6" t="s">
-        <x:v>381</x:v>
+        <x:v>376</x:v>
       </x:c>
       <x:c r="F15" s="6" t="s">
-        <x:v>382</x:v>
+        <x:v>377</x:v>
       </x:c>
       <x:c r="G15" s="6" t="s">
-        <x:v>383</x:v>
+        <x:v>378</x:v>
       </x:c>
       <x:c r="H15" s="7" t="s">
         <x:v>31</x:v>
@@ -4748,25 +4735,25 @@
     </x:row>
     <x:row r="16" ht="42" customHeight="1">
       <x:c r="A16" s="5" t="s">
-        <x:v>206</x:v>
+        <x:v>203</x:v>
       </x:c>
       <x:c r="B16" s="5" t="s">
-        <x:v>384</x:v>
+        <x:v>379</x:v>
       </x:c>
       <x:c r="C16" s="5" t="s">
-        <x:v>385</x:v>
+        <x:v>380</x:v>
       </x:c>
       <x:c r="D16" s="5" t="s">
-        <x:v>386</x:v>
+        <x:v>381</x:v>
       </x:c>
       <x:c r="E16" s="5" t="s">
-        <x:v>203</x:v>
+        <x:v>200</x:v>
       </x:c>
       <x:c r="F16" s="5" t="s">
-        <x:v>344</x:v>
+        <x:v>340</x:v>
       </x:c>
       <x:c r="G16" s="5" t="s">
-        <x:v>353</x:v>
+        <x:v>349</x:v>
       </x:c>
       <x:c r="H16" s="7" t="s">
         <x:v>31</x:v>
@@ -4781,7 +4768,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1424a46a271c49bf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R349efe13f3c347f9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4812,7 +4799,7 @@
     </x:row>
     <x:row r="2" ht="21">
       <x:c r="A2" s="2" t="s">
-        <x:v>387</x:v>
+        <x:v>382</x:v>
       </x:c>
       <x:c r="B2" s="1"/>
       <x:c r="C2" s="1"/>
@@ -4824,7 +4811,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="3" t="s">
-        <x:v>388</x:v>
+        <x:v>383</x:v>
       </x:c>
       <x:c r="B3" s="1"/>
       <x:c r="C3" s="1"/>
@@ -4846,236 +4833,236 @@
     </x:row>
     <x:row r="5" ht="37.95000076293945" customHeight="1">
       <x:c r="A5" s="4" t="s">
+        <x:v>384</x:v>
+      </x:c>
+      <x:c r="B5" s="4" t="s">
+        <x:v>385</x:v>
+      </x:c>
+      <x:c r="C5" s="4" t="s">
+        <x:v>386</x:v>
+      </x:c>
+      <x:c r="D5" s="4" t="s">
+        <x:v>387</x:v>
+      </x:c>
+      <x:c r="E5" s="4" t="s">
+        <x:v>388</x:v>
+      </x:c>
+      <x:c r="F5" s="4" t="s">
         <x:v>389</x:v>
       </x:c>
-      <x:c r="B5" s="4" t="s">
+      <x:c r="G5" s="4" t="s">
         <x:v>390</x:v>
       </x:c>
-      <x:c r="C5" s="4" t="s">
-        <x:v>391</x:v>
-      </x:c>
-      <x:c r="D5" s="4" t="s">
-        <x:v>392</x:v>
-      </x:c>
-      <x:c r="E5" s="4" t="s">
-        <x:v>393</x:v>
-      </x:c>
-      <x:c r="F5" s="4" t="s">
-        <x:v>394</x:v>
-      </x:c>
-      <x:c r="G5" s="4" t="s">
-        <x:v>395</x:v>
-      </x:c>
       <x:c r="H5" s="4" t="s">
-        <x:v>120</x:v>
+        <x:v>117</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="42" customHeight="1">
       <x:c r="A6" s="5" t="s">
+        <x:v>391</x:v>
+      </x:c>
+      <x:c r="B6" s="5" t="s">
+        <x:v>392</x:v>
+      </x:c>
+      <x:c r="C6" s="5" t="s">
+        <x:v>393</x:v>
+      </x:c>
+      <x:c r="D6" s="5" t="s">
+        <x:v>394</x:v>
+      </x:c>
+      <x:c r="E6" s="5" t="s">
+        <x:v>395</x:v>
+      </x:c>
+      <x:c r="F6" s="5" t="s">
         <x:v>396</x:v>
       </x:c>
-      <x:c r="B6" s="5" t="s">
+      <x:c r="G6" s="5" t="s">
         <x:v>397</x:v>
       </x:c>
-      <x:c r="C6" s="5" t="s">
+      <x:c r="H6" s="7" t="s">
         <x:v>398</x:v>
-      </x:c>
-      <x:c r="D6" s="5" t="s">
-        <x:v>399</x:v>
-      </x:c>
-      <x:c r="E6" s="5" t="s">
-        <x:v>400</x:v>
-      </x:c>
-      <x:c r="F6" s="5" t="s">
-        <x:v>401</x:v>
-      </x:c>
-      <x:c r="G6" s="5" t="s">
-        <x:v>402</x:v>
-      </x:c>
-      <x:c r="H6" s="7" t="s">
-        <x:v>403</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="42" customHeight="1">
       <x:c r="A7" s="6" t="s">
+        <x:v>399</x:v>
+      </x:c>
+      <x:c r="B7" s="6" t="s">
+        <x:v>400</x:v>
+      </x:c>
+      <x:c r="C7" s="6" t="s">
+        <x:v>401</x:v>
+      </x:c>
+      <x:c r="D7" s="6" t="s">
+        <x:v>402</x:v>
+      </x:c>
+      <x:c r="E7" s="6" t="s">
+        <x:v>403</x:v>
+      </x:c>
+      <x:c r="F7" s="6" t="s">
         <x:v>404</x:v>
       </x:c>
-      <x:c r="B7" s="6" t="s">
+      <x:c r="G7" s="6" t="s">
         <x:v>405</x:v>
       </x:c>
-      <x:c r="C7" s="6" t="s">
-        <x:v>406</x:v>
-      </x:c>
-      <x:c r="D7" s="6" t="s">
-        <x:v>407</x:v>
-      </x:c>
-      <x:c r="E7" s="6" t="s">
-        <x:v>408</x:v>
-      </x:c>
-      <x:c r="F7" s="6" t="s">
-        <x:v>409</x:v>
-      </x:c>
-      <x:c r="G7" s="6" t="s">
-        <x:v>410</x:v>
-      </x:c>
       <x:c r="H7" s="7" t="s">
-        <x:v>403</x:v>
+        <x:v>398</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="42" customHeight="1">
       <x:c r="A8" s="5" t="s">
+        <x:v>406</x:v>
+      </x:c>
+      <x:c r="B8" s="5" t="s">
+        <x:v>407</x:v>
+      </x:c>
+      <x:c r="C8" s="5" t="s">
+        <x:v>408</x:v>
+      </x:c>
+      <x:c r="D8" s="5" t="s">
+        <x:v>409</x:v>
+      </x:c>
+      <x:c r="E8" s="5" t="s">
+        <x:v>410</x:v>
+      </x:c>
+      <x:c r="F8" s="5" t="s">
         <x:v>411</x:v>
       </x:c>
-      <x:c r="B8" s="5" t="s">
+      <x:c r="G8" s="5" t="s">
         <x:v>412</x:v>
       </x:c>
-      <x:c r="C8" s="5" t="s">
+      <x:c r="H8" s="7" t="s">
         <x:v>413</x:v>
-      </x:c>
-      <x:c r="D8" s="5" t="s">
-        <x:v>414</x:v>
-      </x:c>
-      <x:c r="E8" s="5" t="s">
-        <x:v>415</x:v>
-      </x:c>
-      <x:c r="F8" s="5" t="s">
-        <x:v>416</x:v>
-      </x:c>
-      <x:c r="G8" s="5" t="s">
-        <x:v>417</x:v>
-      </x:c>
-      <x:c r="H8" s="7" t="s">
-        <x:v>418</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="42" customHeight="1">
       <x:c r="A9" s="6" t="s">
+        <x:v>414</x:v>
+      </x:c>
+      <x:c r="B9" s="6" t="s">
+        <x:v>415</x:v>
+      </x:c>
+      <x:c r="C9" s="6" t="s">
+        <x:v>416</x:v>
+      </x:c>
+      <x:c r="D9" s="6" t="s">
+        <x:v>407</x:v>
+      </x:c>
+      <x:c r="E9" s="6" t="s">
+        <x:v>417</x:v>
+      </x:c>
+      <x:c r="F9" s="6" t="s">
+        <x:v>418</x:v>
+      </x:c>
+      <x:c r="G9" s="6" t="s">
         <x:v>419</x:v>
       </x:c>
-      <x:c r="B9" s="6" t="s">
-        <x:v>420</x:v>
-      </x:c>
-      <x:c r="C9" s="6" t="s">
-        <x:v>421</x:v>
-      </x:c>
-      <x:c r="D9" s="6" t="s">
-        <x:v>412</x:v>
-      </x:c>
-      <x:c r="E9" s="6" t="s">
-        <x:v>422</x:v>
-      </x:c>
-      <x:c r="F9" s="6" t="s">
-        <x:v>423</x:v>
-      </x:c>
-      <x:c r="G9" s="6" t="s">
-        <x:v>424</x:v>
-      </x:c>
       <x:c r="H9" s="7" t="s">
-        <x:v>418</x:v>
+        <x:v>413</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="42" customHeight="1">
       <x:c r="A10" s="5" t="s">
+        <x:v>420</x:v>
+      </x:c>
+      <x:c r="B10" s="5" t="s">
+        <x:v>144</x:v>
+      </x:c>
+      <x:c r="C10" s="5" t="s">
+        <x:v>421</x:v>
+      </x:c>
+      <x:c r="D10" s="5" t="s">
+        <x:v>422</x:v>
+      </x:c>
+      <x:c r="E10" s="5" t="s">
+        <x:v>423</x:v>
+      </x:c>
+      <x:c r="F10" s="5" t="s">
+        <x:v>424</x:v>
+      </x:c>
+      <x:c r="G10" s="5" t="s">
         <x:v>425</x:v>
       </x:c>
-      <x:c r="B10" s="5" t="s">
-        <x:v>147</x:v>
-      </x:c>
-      <x:c r="C10" s="5" t="s">
-        <x:v>426</x:v>
-      </x:c>
-      <x:c r="D10" s="5" t="s">
-        <x:v>427</x:v>
-      </x:c>
-      <x:c r="E10" s="5" t="s">
-        <x:v>428</x:v>
-      </x:c>
-      <x:c r="F10" s="5" t="s">
-        <x:v>429</x:v>
-      </x:c>
-      <x:c r="G10" s="5" t="s">
-        <x:v>430</x:v>
-      </x:c>
       <x:c r="H10" s="7" t="s">
-        <x:v>418</x:v>
+        <x:v>413</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="42" customHeight="1">
       <x:c r="A11" s="6" t="s">
+        <x:v>426</x:v>
+      </x:c>
+      <x:c r="B11" s="6" t="s">
+        <x:v>427</x:v>
+      </x:c>
+      <x:c r="C11" s="6" t="s">
+        <x:v>428</x:v>
+      </x:c>
+      <x:c r="D11" s="6" t="s">
+        <x:v>429</x:v>
+      </x:c>
+      <x:c r="E11" s="6" t="s">
+        <x:v>430</x:v>
+      </x:c>
+      <x:c r="F11" s="6" t="s">
         <x:v>431</x:v>
       </x:c>
-      <x:c r="B11" s="6" t="s">
+      <x:c r="G11" s="6" t="s">
         <x:v>432</x:v>
       </x:c>
-      <x:c r="C11" s="6" t="s">
-        <x:v>433</x:v>
-      </x:c>
-      <x:c r="D11" s="6" t="s">
-        <x:v>434</x:v>
-      </x:c>
-      <x:c r="E11" s="6" t="s">
-        <x:v>435</x:v>
-      </x:c>
-      <x:c r="F11" s="6" t="s">
-        <x:v>436</x:v>
-      </x:c>
-      <x:c r="G11" s="6" t="s">
-        <x:v>437</x:v>
-      </x:c>
       <x:c r="H11" s="7" t="s">
-        <x:v>418</x:v>
+        <x:v>413</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="42" customHeight="1">
       <x:c r="A12" s="5" t="s">
+        <x:v>433</x:v>
+      </x:c>
+      <x:c r="B12" s="5" t="s">
+        <x:v>434</x:v>
+      </x:c>
+      <x:c r="C12" s="5" t="s">
+        <x:v>435</x:v>
+      </x:c>
+      <x:c r="D12" s="5" t="s">
+        <x:v>436</x:v>
+      </x:c>
+      <x:c r="E12" s="5" t="s">
+        <x:v>437</x:v>
+      </x:c>
+      <x:c r="F12" s="5" t="s">
         <x:v>438</x:v>
       </x:c>
-      <x:c r="B12" s="5" t="s">
+      <x:c r="G12" s="5" t="s">
         <x:v>439</x:v>
       </x:c>
-      <x:c r="C12" s="5" t="s">
-        <x:v>440</x:v>
-      </x:c>
-      <x:c r="D12" s="5" t="s">
-        <x:v>441</x:v>
-      </x:c>
-      <x:c r="E12" s="5" t="s">
-        <x:v>442</x:v>
-      </x:c>
-      <x:c r="F12" s="5" t="s">
-        <x:v>443</x:v>
-      </x:c>
-      <x:c r="G12" s="5" t="s">
-        <x:v>444</x:v>
-      </x:c>
       <x:c r="H12" s="7" t="s">
-        <x:v>418</x:v>
+        <x:v>413</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="42" customHeight="1">
       <x:c r="A13" s="6" t="s">
+        <x:v>440</x:v>
+      </x:c>
+      <x:c r="B13" s="6" t="s">
+        <x:v>441</x:v>
+      </x:c>
+      <x:c r="C13" s="6" t="s">
+        <x:v>442</x:v>
+      </x:c>
+      <x:c r="D13" s="6" t="s">
+        <x:v>443</x:v>
+      </x:c>
+      <x:c r="E13" s="6" t="s">
+        <x:v>444</x:v>
+      </x:c>
+      <x:c r="F13" s="6" t="s">
         <x:v>445</x:v>
       </x:c>
-      <x:c r="B13" s="6" t="s">
+      <x:c r="G13" s="6" t="s">
         <x:v>446</x:v>
       </x:c>
-      <x:c r="C13" s="6" t="s">
-        <x:v>447</x:v>
-      </x:c>
-      <x:c r="D13" s="6" t="s">
-        <x:v>448</x:v>
-      </x:c>
-      <x:c r="E13" s="6" t="s">
-        <x:v>449</x:v>
-      </x:c>
-      <x:c r="F13" s="6" t="s">
-        <x:v>450</x:v>
-      </x:c>
-      <x:c r="G13" s="6" t="s">
-        <x:v>451</x:v>
-      </x:c>
       <x:c r="H13" s="7" t="s">
-        <x:v>418</x:v>
+        <x:v>413</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -5086,7 +5073,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R51026d9b917f4675"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4dcde4b134f24917"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5115,7 +5102,7 @@
     </x:row>
     <x:row r="2" ht="21">
       <x:c r="A2" s="2" t="s">
-        <x:v>452</x:v>
+        <x:v>447</x:v>
       </x:c>
       <x:c r="B2" s="1"/>
       <x:c r="C2" s="1"/>
@@ -5126,7 +5113,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="3" t="s">
-        <x:v>453</x:v>
+        <x:v>448</x:v>
       </x:c>
       <x:c r="B3" s="1"/>
       <x:c r="C3" s="1"/>
@@ -5146,1181 +5133,1181 @@
     </x:row>
     <x:row r="5" ht="37.95000076293945" customHeight="1">
       <x:c r="A5" s="4" t="s">
+        <x:v>449</x:v>
+      </x:c>
+      <x:c r="B5" s="4" t="s">
+        <x:v>450</x:v>
+      </x:c>
+      <x:c r="C5" s="4" t="s">
+        <x:v>451</x:v>
+      </x:c>
+      <x:c r="D5" s="4" t="s">
+        <x:v>452</x:v>
+      </x:c>
+      <x:c r="E5" s="4" t="s">
+        <x:v>453</x:v>
+      </x:c>
+      <x:c r="F5" s="4" t="s">
+        <x:v>331</x:v>
+      </x:c>
+      <x:c r="G5" s="4" t="s">
         <x:v>454</x:v>
-      </x:c>
-      <x:c r="B5" s="4" t="s">
-        <x:v>455</x:v>
-      </x:c>
-      <x:c r="C5" s="4" t="s">
-        <x:v>456</x:v>
-      </x:c>
-      <x:c r="D5" s="4" t="s">
-        <x:v>457</x:v>
-      </x:c>
-      <x:c r="E5" s="4" t="s">
-        <x:v>458</x:v>
-      </x:c>
-      <x:c r="F5" s="4" t="s">
-        <x:v>335</x:v>
-      </x:c>
-      <x:c r="G5" s="4" t="s">
-        <x:v>459</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="42" customHeight="1">
       <x:c r="A6" s="5" t="s">
+        <x:v>455</x:v>
+      </x:c>
+      <x:c r="B6" s="5" t="s">
+        <x:v>456</x:v>
+      </x:c>
+      <x:c r="C6" s="5" t="s">
+        <x:v>457</x:v>
+      </x:c>
+      <x:c r="D6" s="5" t="s">
+        <x:v>458</x:v>
+      </x:c>
+      <x:c r="E6" s="5" t="s">
+        <x:v>459</x:v>
+      </x:c>
+      <x:c r="F6" s="5" t="s">
         <x:v>460</x:v>
       </x:c>
-      <x:c r="B6" s="5" t="s">
+      <x:c r="G6" s="7" t="s">
         <x:v>461</x:v>
-      </x:c>
-      <x:c r="C6" s="5" t="s">
-        <x:v>462</x:v>
-      </x:c>
-      <x:c r="D6" s="5" t="s">
-        <x:v>463</x:v>
-      </x:c>
-      <x:c r="E6" s="5" t="s">
-        <x:v>464</x:v>
-      </x:c>
-      <x:c r="F6" s="5" t="s">
-        <x:v>465</x:v>
-      </x:c>
-      <x:c r="G6" s="7" t="s">
-        <x:v>466</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="42" customHeight="1">
       <x:c r="A7" s="6" t="s">
-        <x:v>467</x:v>
+        <x:v>462</x:v>
       </x:c>
       <x:c r="B7" s="6" t="s">
+        <x:v>456</x:v>
+      </x:c>
+      <x:c r="C7" s="6" t="s">
+        <x:v>463</x:v>
+      </x:c>
+      <x:c r="D7" s="6" t="s">
+        <x:v>464</x:v>
+      </x:c>
+      <x:c r="E7" s="6" t="s">
+        <x:v>459</x:v>
+      </x:c>
+      <x:c r="F7" s="6" t="s">
+        <x:v>460</x:v>
+      </x:c>
+      <x:c r="G7" s="7" t="s">
         <x:v>461</x:v>
-      </x:c>
-      <x:c r="C7" s="6" t="s">
-        <x:v>468</x:v>
-      </x:c>
-      <x:c r="D7" s="6" t="s">
-        <x:v>469</x:v>
-      </x:c>
-      <x:c r="E7" s="6" t="s">
-        <x:v>464</x:v>
-      </x:c>
-      <x:c r="F7" s="6" t="s">
-        <x:v>465</x:v>
-      </x:c>
-      <x:c r="G7" s="7" t="s">
-        <x:v>466</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="42" customHeight="1">
       <x:c r="A8" s="5" t="s">
-        <x:v>470</x:v>
+        <x:v>465</x:v>
       </x:c>
       <x:c r="B8" s="5" t="s">
+        <x:v>456</x:v>
+      </x:c>
+      <x:c r="C8" s="5" t="s">
+        <x:v>466</x:v>
+      </x:c>
+      <x:c r="D8" s="5" t="s">
+        <x:v>458</x:v>
+      </x:c>
+      <x:c r="E8" s="5" t="s">
+        <x:v>459</x:v>
+      </x:c>
+      <x:c r="F8" s="5" t="s">
+        <x:v>460</x:v>
+      </x:c>
+      <x:c r="G8" s="7" t="s">
         <x:v>461</x:v>
-      </x:c>
-      <x:c r="C8" s="5" t="s">
-        <x:v>471</x:v>
-      </x:c>
-      <x:c r="D8" s="5" t="s">
-        <x:v>463</x:v>
-      </x:c>
-      <x:c r="E8" s="5" t="s">
-        <x:v>464</x:v>
-      </x:c>
-      <x:c r="F8" s="5" t="s">
-        <x:v>465</x:v>
-      </x:c>
-      <x:c r="G8" s="7" t="s">
-        <x:v>466</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="42" customHeight="1">
       <x:c r="A9" s="6" t="s">
-        <x:v>472</x:v>
+        <x:v>467</x:v>
       </x:c>
       <x:c r="B9" s="6" t="s">
-        <x:v>473</x:v>
+        <x:v>468</x:v>
       </x:c>
       <x:c r="C9" s="6" t="s">
-        <x:v>474</x:v>
+        <x:v>469</x:v>
       </x:c>
       <x:c r="D9" s="6" t="s">
-        <x:v>463</x:v>
+        <x:v>458</x:v>
       </x:c>
       <x:c r="E9" s="6" t="s">
-        <x:v>464</x:v>
+        <x:v>459</x:v>
       </x:c>
       <x:c r="F9" s="6" t="s">
-        <x:v>465</x:v>
+        <x:v>460</x:v>
       </x:c>
       <x:c r="G9" s="7" t="s">
-        <x:v>466</x:v>
+        <x:v>461</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="42" customHeight="1">
       <x:c r="A10" s="5" t="s">
-        <x:v>475</x:v>
+        <x:v>470</x:v>
       </x:c>
       <x:c r="B10" s="5" t="s">
-        <x:v>473</x:v>
+        <x:v>468</x:v>
       </x:c>
       <x:c r="C10" s="5" t="s">
-        <x:v>476</x:v>
+        <x:v>471</x:v>
       </x:c>
       <x:c r="D10" s="5" t="s">
-        <x:v>469</x:v>
+        <x:v>464</x:v>
       </x:c>
       <x:c r="E10" s="5" t="s">
-        <x:v>464</x:v>
+        <x:v>459</x:v>
       </x:c>
       <x:c r="F10" s="5" t="s">
-        <x:v>465</x:v>
+        <x:v>460</x:v>
       </x:c>
       <x:c r="G10" s="7" t="s">
-        <x:v>466</x:v>
+        <x:v>461</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="42" customHeight="1">
       <x:c r="A11" s="6" t="s">
-        <x:v>477</x:v>
+        <x:v>472</x:v>
       </x:c>
       <x:c r="B11" s="6" t="s">
+        <x:v>456</x:v>
+      </x:c>
+      <x:c r="C11" s="6" t="s">
+        <x:v>473</x:v>
+      </x:c>
+      <x:c r="D11" s="6" t="s">
+        <x:v>458</x:v>
+      </x:c>
+      <x:c r="E11" s="6" t="s">
+        <x:v>459</x:v>
+      </x:c>
+      <x:c r="F11" s="6" t="s">
+        <x:v>460</x:v>
+      </x:c>
+      <x:c r="G11" s="7" t="s">
         <x:v>461</x:v>
-      </x:c>
-      <x:c r="C11" s="6" t="s">
-        <x:v>478</x:v>
-      </x:c>
-      <x:c r="D11" s="6" t="s">
-        <x:v>463</x:v>
-      </x:c>
-      <x:c r="E11" s="6" t="s">
-        <x:v>464</x:v>
-      </x:c>
-      <x:c r="F11" s="6" t="s">
-        <x:v>465</x:v>
-      </x:c>
-      <x:c r="G11" s="7" t="s">
-        <x:v>466</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="42" customHeight="1">
       <x:c r="A12" s="5" t="s">
-        <x:v>479</x:v>
+        <x:v>474</x:v>
       </x:c>
       <x:c r="B12" s="5" t="s">
+        <x:v>456</x:v>
+      </x:c>
+      <x:c r="C12" s="5" t="s">
+        <x:v>475</x:v>
+      </x:c>
+      <x:c r="D12" s="5" t="s">
+        <x:v>458</x:v>
+      </x:c>
+      <x:c r="E12" s="5" t="s">
+        <x:v>459</x:v>
+      </x:c>
+      <x:c r="F12" s="5" t="s">
+        <x:v>460</x:v>
+      </x:c>
+      <x:c r="G12" s="7" t="s">
         <x:v>461</x:v>
-      </x:c>
-      <x:c r="C12" s="5" t="s">
-        <x:v>480</x:v>
-      </x:c>
-      <x:c r="D12" s="5" t="s">
-        <x:v>463</x:v>
-      </x:c>
-      <x:c r="E12" s="5" t="s">
-        <x:v>464</x:v>
-      </x:c>
-      <x:c r="F12" s="5" t="s">
-        <x:v>465</x:v>
-      </x:c>
-      <x:c r="G12" s="7" t="s">
-        <x:v>466</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="42" customHeight="1">
       <x:c r="A13" s="6" t="s">
-        <x:v>481</x:v>
+        <x:v>476</x:v>
       </x:c>
       <x:c r="B13" s="6" t="s">
+        <x:v>456</x:v>
+      </x:c>
+      <x:c r="C13" s="6" t="s">
+        <x:v>477</x:v>
+      </x:c>
+      <x:c r="D13" s="6" t="s">
+        <x:v>458</x:v>
+      </x:c>
+      <x:c r="E13" s="6" t="s">
+        <x:v>459</x:v>
+      </x:c>
+      <x:c r="F13" s="6" t="s">
+        <x:v>460</x:v>
+      </x:c>
+      <x:c r="G13" s="7" t="s">
         <x:v>461</x:v>
-      </x:c>
-      <x:c r="C13" s="6" t="s">
-        <x:v>482</x:v>
-      </x:c>
-      <x:c r="D13" s="6" t="s">
-        <x:v>463</x:v>
-      </x:c>
-      <x:c r="E13" s="6" t="s">
-        <x:v>464</x:v>
-      </x:c>
-      <x:c r="F13" s="6" t="s">
-        <x:v>465</x:v>
-      </x:c>
-      <x:c r="G13" s="7" t="s">
-        <x:v>466</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="42" customHeight="1">
       <x:c r="A14" s="5" t="s">
-        <x:v>483</x:v>
+        <x:v>478</x:v>
       </x:c>
       <x:c r="B14" s="5" t="s">
-        <x:v>473</x:v>
+        <x:v>468</x:v>
       </x:c>
       <x:c r="C14" s="5" t="s">
-        <x:v>484</x:v>
+        <x:v>479</x:v>
       </x:c>
       <x:c r="D14" s="5" t="s">
-        <x:v>463</x:v>
+        <x:v>458</x:v>
       </x:c>
       <x:c r="E14" s="5" t="s">
-        <x:v>464</x:v>
+        <x:v>459</x:v>
       </x:c>
       <x:c r="F14" s="5" t="s">
-        <x:v>465</x:v>
+        <x:v>460</x:v>
       </x:c>
       <x:c r="G14" s="7" t="s">
-        <x:v>466</x:v>
+        <x:v>461</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="42" customHeight="1">
       <x:c r="A15" s="6" t="s">
-        <x:v>485</x:v>
+        <x:v>480</x:v>
       </x:c>
       <x:c r="B15" s="6" t="s">
-        <x:v>473</x:v>
+        <x:v>468</x:v>
       </x:c>
       <x:c r="C15" s="6" t="s">
-        <x:v>486</x:v>
+        <x:v>481</x:v>
       </x:c>
       <x:c r="D15" s="6" t="s">
-        <x:v>463</x:v>
+        <x:v>458</x:v>
       </x:c>
       <x:c r="E15" s="6" t="s">
-        <x:v>464</x:v>
+        <x:v>459</x:v>
       </x:c>
       <x:c r="F15" s="6" t="s">
-        <x:v>465</x:v>
+        <x:v>460</x:v>
       </x:c>
       <x:c r="G15" s="7" t="s">
-        <x:v>466</x:v>
+        <x:v>461</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="42" customHeight="1">
       <x:c r="A16" s="5" t="s">
-        <x:v>487</x:v>
+        <x:v>482</x:v>
       </x:c>
       <x:c r="B16" s="5" t="s">
-        <x:v>473</x:v>
+        <x:v>468</x:v>
       </x:c>
       <x:c r="C16" s="5" t="s">
-        <x:v>488</x:v>
+        <x:v>483</x:v>
       </x:c>
       <x:c r="D16" s="5" t="s">
-        <x:v>463</x:v>
+        <x:v>458</x:v>
       </x:c>
       <x:c r="E16" s="5" t="s">
-        <x:v>464</x:v>
+        <x:v>459</x:v>
       </x:c>
       <x:c r="F16" s="5" t="s">
-        <x:v>465</x:v>
+        <x:v>460</x:v>
       </x:c>
       <x:c r="G16" s="7" t="s">
-        <x:v>466</x:v>
+        <x:v>461</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="42" customHeight="1">
       <x:c r="A17" s="6" t="s">
-        <x:v>489</x:v>
+        <x:v>484</x:v>
       </x:c>
       <x:c r="B17" s="6" t="s">
-        <x:v>473</x:v>
+        <x:v>468</x:v>
       </x:c>
       <x:c r="C17" s="6" t="s">
-        <x:v>490</x:v>
+        <x:v>485</x:v>
       </x:c>
       <x:c r="D17" s="6" t="s">
-        <x:v>463</x:v>
+        <x:v>458</x:v>
       </x:c>
       <x:c r="E17" s="6" t="s">
-        <x:v>464</x:v>
+        <x:v>459</x:v>
       </x:c>
       <x:c r="F17" s="6" t="s">
-        <x:v>465</x:v>
+        <x:v>460</x:v>
       </x:c>
       <x:c r="G17" s="7" t="s">
-        <x:v>466</x:v>
+        <x:v>461</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="42" customHeight="1">
       <x:c r="A18" s="5" t="s">
-        <x:v>491</x:v>
+        <x:v>486</x:v>
       </x:c>
       <x:c r="B18" s="5" t="s">
+        <x:v>456</x:v>
+      </x:c>
+      <x:c r="C18" s="5" t="s">
+        <x:v>487</x:v>
+      </x:c>
+      <x:c r="D18" s="5" t="s">
+        <x:v>488</x:v>
+      </x:c>
+      <x:c r="E18" s="5" t="s">
+        <x:v>459</x:v>
+      </x:c>
+      <x:c r="F18" s="5" t="s">
+        <x:v>460</x:v>
+      </x:c>
+      <x:c r="G18" s="7" t="s">
         <x:v>461</x:v>
-      </x:c>
-      <x:c r="C18" s="5" t="s">
-        <x:v>492</x:v>
-      </x:c>
-      <x:c r="D18" s="5" t="s">
-        <x:v>493</x:v>
-      </x:c>
-      <x:c r="E18" s="5" t="s">
-        <x:v>464</x:v>
-      </x:c>
-      <x:c r="F18" s="5" t="s">
-        <x:v>465</x:v>
-      </x:c>
-      <x:c r="G18" s="7" t="s">
-        <x:v>466</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="42" customHeight="1">
       <x:c r="A19" s="6" t="s">
-        <x:v>494</x:v>
+        <x:v>489</x:v>
       </x:c>
       <x:c r="B19" s="6" t="s">
+        <x:v>456</x:v>
+      </x:c>
+      <x:c r="C19" s="6" t="s">
+        <x:v>490</x:v>
+      </x:c>
+      <x:c r="D19" s="6" t="s">
+        <x:v>488</x:v>
+      </x:c>
+      <x:c r="E19" s="6" t="s">
+        <x:v>459</x:v>
+      </x:c>
+      <x:c r="F19" s="6" t="s">
+        <x:v>460</x:v>
+      </x:c>
+      <x:c r="G19" s="7" t="s">
         <x:v>461</x:v>
-      </x:c>
-      <x:c r="C19" s="6" t="s">
-        <x:v>495</x:v>
-      </x:c>
-      <x:c r="D19" s="6" t="s">
-        <x:v>493</x:v>
-      </x:c>
-      <x:c r="E19" s="6" t="s">
-        <x:v>464</x:v>
-      </x:c>
-      <x:c r="F19" s="6" t="s">
-        <x:v>465</x:v>
-      </x:c>
-      <x:c r="G19" s="7" t="s">
-        <x:v>466</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="42" customHeight="1">
       <x:c r="A20" s="5" t="s">
-        <x:v>496</x:v>
+        <x:v>491</x:v>
       </x:c>
       <x:c r="B20" s="5" t="s">
+        <x:v>456</x:v>
+      </x:c>
+      <x:c r="C20" s="5" t="s">
+        <x:v>492</x:v>
+      </x:c>
+      <x:c r="D20" s="5" t="s">
+        <x:v>488</x:v>
+      </x:c>
+      <x:c r="E20" s="5" t="s">
+        <x:v>459</x:v>
+      </x:c>
+      <x:c r="F20" s="5" t="s">
+        <x:v>460</x:v>
+      </x:c>
+      <x:c r="G20" s="7" t="s">
         <x:v>461</x:v>
-      </x:c>
-      <x:c r="C20" s="5" t="s">
-        <x:v>497</x:v>
-      </x:c>
-      <x:c r="D20" s="5" t="s">
-        <x:v>493</x:v>
-      </x:c>
-      <x:c r="E20" s="5" t="s">
-        <x:v>464</x:v>
-      </x:c>
-      <x:c r="F20" s="5" t="s">
-        <x:v>465</x:v>
-      </x:c>
-      <x:c r="G20" s="7" t="s">
-        <x:v>466</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="42" customHeight="1">
       <x:c r="A21" s="6" t="s">
-        <x:v>498</x:v>
+        <x:v>493</x:v>
       </x:c>
       <x:c r="B21" s="6" t="s">
+        <x:v>456</x:v>
+      </x:c>
+      <x:c r="C21" s="6" t="s">
+        <x:v>494</x:v>
+      </x:c>
+      <x:c r="D21" s="6" t="s">
+        <x:v>488</x:v>
+      </x:c>
+      <x:c r="E21" s="6" t="s">
+        <x:v>459</x:v>
+      </x:c>
+      <x:c r="F21" s="6" t="s">
+        <x:v>460</x:v>
+      </x:c>
+      <x:c r="G21" s="7" t="s">
         <x:v>461</x:v>
-      </x:c>
-      <x:c r="C21" s="6" t="s">
-        <x:v>499</x:v>
-      </x:c>
-      <x:c r="D21" s="6" t="s">
-        <x:v>493</x:v>
-      </x:c>
-      <x:c r="E21" s="6" t="s">
-        <x:v>464</x:v>
-      </x:c>
-      <x:c r="F21" s="6" t="s">
-        <x:v>465</x:v>
-      </x:c>
-      <x:c r="G21" s="7" t="s">
-        <x:v>466</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="42" customHeight="1">
       <x:c r="A22" s="5" t="s">
-        <x:v>500</x:v>
+        <x:v>495</x:v>
       </x:c>
       <x:c r="B22" s="5" t="s">
+        <x:v>456</x:v>
+      </x:c>
+      <x:c r="C22" s="5" t="s">
+        <x:v>496</x:v>
+      </x:c>
+      <x:c r="D22" s="5" t="s">
+        <x:v>488</x:v>
+      </x:c>
+      <x:c r="E22" s="5" t="s">
+        <x:v>459</x:v>
+      </x:c>
+      <x:c r="F22" s="5" t="s">
+        <x:v>460</x:v>
+      </x:c>
+      <x:c r="G22" s="7" t="s">
         <x:v>461</x:v>
-      </x:c>
-      <x:c r="C22" s="5" t="s">
-        <x:v>501</x:v>
-      </x:c>
-      <x:c r="D22" s="5" t="s">
-        <x:v>493</x:v>
-      </x:c>
-      <x:c r="E22" s="5" t="s">
-        <x:v>464</x:v>
-      </x:c>
-      <x:c r="F22" s="5" t="s">
-        <x:v>465</x:v>
-      </x:c>
-      <x:c r="G22" s="7" t="s">
-        <x:v>466</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="42" customHeight="1">
       <x:c r="A23" s="6" t="s">
-        <x:v>502</x:v>
+        <x:v>497</x:v>
       </x:c>
       <x:c r="B23" s="6" t="s">
+        <x:v>456</x:v>
+      </x:c>
+      <x:c r="C23" s="6" t="s">
+        <x:v>498</x:v>
+      </x:c>
+      <x:c r="D23" s="6" t="s">
+        <x:v>488</x:v>
+      </x:c>
+      <x:c r="E23" s="6" t="s">
+        <x:v>459</x:v>
+      </x:c>
+      <x:c r="F23" s="6" t="s">
+        <x:v>460</x:v>
+      </x:c>
+      <x:c r="G23" s="7" t="s">
         <x:v>461</x:v>
-      </x:c>
-      <x:c r="C23" s="6" t="s">
-        <x:v>503</x:v>
-      </x:c>
-      <x:c r="D23" s="6" t="s">
-        <x:v>493</x:v>
-      </x:c>
-      <x:c r="E23" s="6" t="s">
-        <x:v>464</x:v>
-      </x:c>
-      <x:c r="F23" s="6" t="s">
-        <x:v>465</x:v>
-      </x:c>
-      <x:c r="G23" s="7" t="s">
-        <x:v>466</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="42" customHeight="1">
       <x:c r="A24" s="5" t="s">
-        <x:v>504</x:v>
+        <x:v>499</x:v>
       </x:c>
       <x:c r="B24" s="5" t="s">
+        <x:v>456</x:v>
+      </x:c>
+      <x:c r="C24" s="5" t="s">
+        <x:v>500</x:v>
+      </x:c>
+      <x:c r="D24" s="5" t="s">
+        <x:v>488</x:v>
+      </x:c>
+      <x:c r="E24" s="5" t="s">
+        <x:v>459</x:v>
+      </x:c>
+      <x:c r="F24" s="5" t="s">
+        <x:v>460</x:v>
+      </x:c>
+      <x:c r="G24" s="7" t="s">
         <x:v>461</x:v>
-      </x:c>
-      <x:c r="C24" s="5" t="s">
-        <x:v>505</x:v>
-      </x:c>
-      <x:c r="D24" s="5" t="s">
-        <x:v>493</x:v>
-      </x:c>
-      <x:c r="E24" s="5" t="s">
-        <x:v>464</x:v>
-      </x:c>
-      <x:c r="F24" s="5" t="s">
-        <x:v>465</x:v>
-      </x:c>
-      <x:c r="G24" s="7" t="s">
-        <x:v>466</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="42" customHeight="1">
       <x:c r="A25" s="6" t="s">
-        <x:v>506</x:v>
+        <x:v>501</x:v>
       </x:c>
       <x:c r="B25" s="6" t="s">
+        <x:v>456</x:v>
+      </x:c>
+      <x:c r="C25" s="6" t="s">
+        <x:v>502</x:v>
+      </x:c>
+      <x:c r="D25" s="6" t="s">
+        <x:v>488</x:v>
+      </x:c>
+      <x:c r="E25" s="6" t="s">
+        <x:v>459</x:v>
+      </x:c>
+      <x:c r="F25" s="6" t="s">
+        <x:v>460</x:v>
+      </x:c>
+      <x:c r="G25" s="7" t="s">
         <x:v>461</x:v>
-      </x:c>
-      <x:c r="C25" s="6" t="s">
-        <x:v>507</x:v>
-      </x:c>
-      <x:c r="D25" s="6" t="s">
-        <x:v>493</x:v>
-      </x:c>
-      <x:c r="E25" s="6" t="s">
-        <x:v>464</x:v>
-      </x:c>
-      <x:c r="F25" s="6" t="s">
-        <x:v>465</x:v>
-      </x:c>
-      <x:c r="G25" s="7" t="s">
-        <x:v>466</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="42" customHeight="1">
       <x:c r="A26" s="5" t="s">
-        <x:v>508</x:v>
+        <x:v>503</x:v>
       </x:c>
       <x:c r="B26" s="5" t="s">
+        <x:v>456</x:v>
+      </x:c>
+      <x:c r="C26" s="5" t="s">
+        <x:v>504</x:v>
+      </x:c>
+      <x:c r="D26" s="5" t="s">
+        <x:v>488</x:v>
+      </x:c>
+      <x:c r="E26" s="5" t="s">
+        <x:v>459</x:v>
+      </x:c>
+      <x:c r="F26" s="5" t="s">
+        <x:v>460</x:v>
+      </x:c>
+      <x:c r="G26" s="7" t="s">
         <x:v>461</x:v>
-      </x:c>
-      <x:c r="C26" s="5" t="s">
-        <x:v>509</x:v>
-      </x:c>
-      <x:c r="D26" s="5" t="s">
-        <x:v>493</x:v>
-      </x:c>
-      <x:c r="E26" s="5" t="s">
-        <x:v>464</x:v>
-      </x:c>
-      <x:c r="F26" s="5" t="s">
-        <x:v>465</x:v>
-      </x:c>
-      <x:c r="G26" s="7" t="s">
-        <x:v>466</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="42" customHeight="1">
       <x:c r="A27" s="6" t="s">
-        <x:v>510</x:v>
+        <x:v>505</x:v>
       </x:c>
       <x:c r="B27" s="6" t="s">
+        <x:v>456</x:v>
+      </x:c>
+      <x:c r="C27" s="6" t="s">
+        <x:v>506</x:v>
+      </x:c>
+      <x:c r="D27" s="6" t="s">
+        <x:v>488</x:v>
+      </x:c>
+      <x:c r="E27" s="6" t="s">
+        <x:v>459</x:v>
+      </x:c>
+      <x:c r="F27" s="6" t="s">
+        <x:v>460</x:v>
+      </x:c>
+      <x:c r="G27" s="7" t="s">
         <x:v>461</x:v>
-      </x:c>
-      <x:c r="C27" s="6" t="s">
-        <x:v>511</x:v>
-      </x:c>
-      <x:c r="D27" s="6" t="s">
-        <x:v>493</x:v>
-      </x:c>
-      <x:c r="E27" s="6" t="s">
-        <x:v>464</x:v>
-      </x:c>
-      <x:c r="F27" s="6" t="s">
-        <x:v>465</x:v>
-      </x:c>
-      <x:c r="G27" s="7" t="s">
-        <x:v>466</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="42" customHeight="1">
       <x:c r="A28" s="5" t="s">
-        <x:v>512</x:v>
+        <x:v>507</x:v>
       </x:c>
       <x:c r="B28" s="5" t="s">
+        <x:v>456</x:v>
+      </x:c>
+      <x:c r="C28" s="5" t="s">
+        <x:v>508</x:v>
+      </x:c>
+      <x:c r="D28" s="5" t="s">
+        <x:v>488</x:v>
+      </x:c>
+      <x:c r="E28" s="5" t="s">
+        <x:v>459</x:v>
+      </x:c>
+      <x:c r="F28" s="5" t="s">
+        <x:v>460</x:v>
+      </x:c>
+      <x:c r="G28" s="7" t="s">
         <x:v>461</x:v>
-      </x:c>
-      <x:c r="C28" s="5" t="s">
-        <x:v>513</x:v>
-      </x:c>
-      <x:c r="D28" s="5" t="s">
-        <x:v>493</x:v>
-      </x:c>
-      <x:c r="E28" s="5" t="s">
-        <x:v>464</x:v>
-      </x:c>
-      <x:c r="F28" s="5" t="s">
-        <x:v>465</x:v>
-      </x:c>
-      <x:c r="G28" s="7" t="s">
-        <x:v>466</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="42" customHeight="1">
       <x:c r="A29" s="6" t="s">
-        <x:v>514</x:v>
+        <x:v>509</x:v>
       </x:c>
       <x:c r="B29" s="6" t="s">
+        <x:v>456</x:v>
+      </x:c>
+      <x:c r="C29" s="6" t="s">
+        <x:v>510</x:v>
+      </x:c>
+      <x:c r="D29" s="6" t="s">
+        <x:v>488</x:v>
+      </x:c>
+      <x:c r="E29" s="6" t="s">
+        <x:v>459</x:v>
+      </x:c>
+      <x:c r="F29" s="6" t="s">
+        <x:v>460</x:v>
+      </x:c>
+      <x:c r="G29" s="7" t="s">
         <x:v>461</x:v>
-      </x:c>
-      <x:c r="C29" s="6" t="s">
-        <x:v>515</x:v>
-      </x:c>
-      <x:c r="D29" s="6" t="s">
-        <x:v>493</x:v>
-      </x:c>
-      <x:c r="E29" s="6" t="s">
-        <x:v>464</x:v>
-      </x:c>
-      <x:c r="F29" s="6" t="s">
-        <x:v>465</x:v>
-      </x:c>
-      <x:c r="G29" s="7" t="s">
-        <x:v>466</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="42" customHeight="1">
       <x:c r="A30" s="5" t="s">
-        <x:v>516</x:v>
+        <x:v>511</x:v>
       </x:c>
       <x:c r="B30" s="5" t="s">
+        <x:v>456</x:v>
+      </x:c>
+      <x:c r="C30" s="5" t="s">
+        <x:v>512</x:v>
+      </x:c>
+      <x:c r="D30" s="5" t="s">
+        <x:v>488</x:v>
+      </x:c>
+      <x:c r="E30" s="5" t="s">
+        <x:v>459</x:v>
+      </x:c>
+      <x:c r="F30" s="5" t="s">
+        <x:v>460</x:v>
+      </x:c>
+      <x:c r="G30" s="7" t="s">
         <x:v>461</x:v>
-      </x:c>
-      <x:c r="C30" s="5" t="s">
-        <x:v>517</x:v>
-      </x:c>
-      <x:c r="D30" s="5" t="s">
-        <x:v>493</x:v>
-      </x:c>
-      <x:c r="E30" s="5" t="s">
-        <x:v>464</x:v>
-      </x:c>
-      <x:c r="F30" s="5" t="s">
-        <x:v>465</x:v>
-      </x:c>
-      <x:c r="G30" s="7" t="s">
-        <x:v>466</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="42" customHeight="1">
       <x:c r="A31" s="6" t="s">
-        <x:v>518</x:v>
+        <x:v>513</x:v>
       </x:c>
       <x:c r="B31" s="6" t="s">
+        <x:v>456</x:v>
+      </x:c>
+      <x:c r="C31" s="6" t="s">
+        <x:v>514</x:v>
+      </x:c>
+      <x:c r="D31" s="6" t="s">
+        <x:v>488</x:v>
+      </x:c>
+      <x:c r="E31" s="6" t="s">
+        <x:v>459</x:v>
+      </x:c>
+      <x:c r="F31" s="6" t="s">
+        <x:v>460</x:v>
+      </x:c>
+      <x:c r="G31" s="7" t="s">
         <x:v>461</x:v>
-      </x:c>
-      <x:c r="C31" s="6" t="s">
-        <x:v>519</x:v>
-      </x:c>
-      <x:c r="D31" s="6" t="s">
-        <x:v>493</x:v>
-      </x:c>
-      <x:c r="E31" s="6" t="s">
-        <x:v>464</x:v>
-      </x:c>
-      <x:c r="F31" s="6" t="s">
-        <x:v>465</x:v>
-      </x:c>
-      <x:c r="G31" s="7" t="s">
-        <x:v>466</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="42" customHeight="1">
       <x:c r="A32" s="5" t="s">
-        <x:v>520</x:v>
+        <x:v>515</x:v>
       </x:c>
       <x:c r="B32" s="5" t="s">
+        <x:v>456</x:v>
+      </x:c>
+      <x:c r="C32" s="5" t="s">
+        <x:v>516</x:v>
+      </x:c>
+      <x:c r="D32" s="5" t="s">
+        <x:v>488</x:v>
+      </x:c>
+      <x:c r="E32" s="5" t="s">
+        <x:v>459</x:v>
+      </x:c>
+      <x:c r="F32" s="5" t="s">
+        <x:v>460</x:v>
+      </x:c>
+      <x:c r="G32" s="7" t="s">
         <x:v>461</x:v>
-      </x:c>
-      <x:c r="C32" s="5" t="s">
-        <x:v>521</x:v>
-      </x:c>
-      <x:c r="D32" s="5" t="s">
-        <x:v>493</x:v>
-      </x:c>
-      <x:c r="E32" s="5" t="s">
-        <x:v>464</x:v>
-      </x:c>
-      <x:c r="F32" s="5" t="s">
-        <x:v>465</x:v>
-      </x:c>
-      <x:c r="G32" s="7" t="s">
-        <x:v>466</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="42" customHeight="1">
       <x:c r="A33" s="6" t="s">
-        <x:v>522</x:v>
+        <x:v>517</x:v>
       </x:c>
       <x:c r="B33" s="6" t="s">
+        <x:v>456</x:v>
+      </x:c>
+      <x:c r="C33" s="6" t="s">
+        <x:v>518</x:v>
+      </x:c>
+      <x:c r="D33" s="6" t="s">
+        <x:v>488</x:v>
+      </x:c>
+      <x:c r="E33" s="6" t="s">
+        <x:v>459</x:v>
+      </x:c>
+      <x:c r="F33" s="6" t="s">
+        <x:v>460</x:v>
+      </x:c>
+      <x:c r="G33" s="7" t="s">
         <x:v>461</x:v>
-      </x:c>
-      <x:c r="C33" s="6" t="s">
-        <x:v>523</x:v>
-      </x:c>
-      <x:c r="D33" s="6" t="s">
-        <x:v>493</x:v>
-      </x:c>
-      <x:c r="E33" s="6" t="s">
-        <x:v>464</x:v>
-      </x:c>
-      <x:c r="F33" s="6" t="s">
-        <x:v>465</x:v>
-      </x:c>
-      <x:c r="G33" s="7" t="s">
-        <x:v>466</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="42" customHeight="1">
       <x:c r="A34" s="5" t="s">
-        <x:v>524</x:v>
+        <x:v>519</x:v>
       </x:c>
       <x:c r="B34" s="5" t="s">
+        <x:v>456</x:v>
+      </x:c>
+      <x:c r="C34" s="5" t="s">
+        <x:v>520</x:v>
+      </x:c>
+      <x:c r="D34" s="5" t="s">
+        <x:v>488</x:v>
+      </x:c>
+      <x:c r="E34" s="5" t="s">
+        <x:v>459</x:v>
+      </x:c>
+      <x:c r="F34" s="5" t="s">
+        <x:v>460</x:v>
+      </x:c>
+      <x:c r="G34" s="7" t="s">
         <x:v>461</x:v>
-      </x:c>
-      <x:c r="C34" s="5" t="s">
-        <x:v>525</x:v>
-      </x:c>
-      <x:c r="D34" s="5" t="s">
-        <x:v>493</x:v>
-      </x:c>
-      <x:c r="E34" s="5" t="s">
-        <x:v>464</x:v>
-      </x:c>
-      <x:c r="F34" s="5" t="s">
-        <x:v>465</x:v>
-      </x:c>
-      <x:c r="G34" s="7" t="s">
-        <x:v>466</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="42" customHeight="1">
       <x:c r="A35" s="6" t="s">
-        <x:v>526</x:v>
+        <x:v>521</x:v>
       </x:c>
       <x:c r="B35" s="6" t="s">
+        <x:v>456</x:v>
+      </x:c>
+      <x:c r="C35" s="6" t="s">
+        <x:v>522</x:v>
+      </x:c>
+      <x:c r="D35" s="6" t="s">
+        <x:v>488</x:v>
+      </x:c>
+      <x:c r="E35" s="6" t="s">
+        <x:v>459</x:v>
+      </x:c>
+      <x:c r="F35" s="6" t="s">
+        <x:v>460</x:v>
+      </x:c>
+      <x:c r="G35" s="7" t="s">
         <x:v>461</x:v>
-      </x:c>
-      <x:c r="C35" s="6" t="s">
-        <x:v>527</x:v>
-      </x:c>
-      <x:c r="D35" s="6" t="s">
-        <x:v>493</x:v>
-      </x:c>
-      <x:c r="E35" s="6" t="s">
-        <x:v>464</x:v>
-      </x:c>
-      <x:c r="F35" s="6" t="s">
-        <x:v>465</x:v>
-      </x:c>
-      <x:c r="G35" s="7" t="s">
-        <x:v>466</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="42" customHeight="1">
       <x:c r="A36" s="5" t="s">
-        <x:v>528</x:v>
+        <x:v>523</x:v>
       </x:c>
       <x:c r="B36" s="5" t="s">
+        <x:v>456</x:v>
+      </x:c>
+      <x:c r="C36" s="5" t="s">
+        <x:v>524</x:v>
+      </x:c>
+      <x:c r="D36" s="5" t="s">
+        <x:v>488</x:v>
+      </x:c>
+      <x:c r="E36" s="5" t="s">
+        <x:v>459</x:v>
+      </x:c>
+      <x:c r="F36" s="5" t="s">
+        <x:v>460</x:v>
+      </x:c>
+      <x:c r="G36" s="7" t="s">
         <x:v>461</x:v>
-      </x:c>
-      <x:c r="C36" s="5" t="s">
-        <x:v>529</x:v>
-      </x:c>
-      <x:c r="D36" s="5" t="s">
-        <x:v>493</x:v>
-      </x:c>
-      <x:c r="E36" s="5" t="s">
-        <x:v>464</x:v>
-      </x:c>
-      <x:c r="F36" s="5" t="s">
-        <x:v>465</x:v>
-      </x:c>
-      <x:c r="G36" s="7" t="s">
-        <x:v>466</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="42" customHeight="1">
       <x:c r="A37" s="6" t="s">
-        <x:v>530</x:v>
+        <x:v>525</x:v>
       </x:c>
       <x:c r="B37" s="6" t="s">
-        <x:v>473</x:v>
+        <x:v>468</x:v>
       </x:c>
       <x:c r="C37" s="6" t="s">
-        <x:v>531</x:v>
+        <x:v>526</x:v>
       </x:c>
       <x:c r="D37" s="6" t="s">
-        <x:v>493</x:v>
+        <x:v>488</x:v>
       </x:c>
       <x:c r="E37" s="6" t="s">
-        <x:v>464</x:v>
+        <x:v>459</x:v>
       </x:c>
       <x:c r="F37" s="6" t="s">
-        <x:v>465</x:v>
+        <x:v>460</x:v>
       </x:c>
       <x:c r="G37" s="7" t="s">
-        <x:v>466</x:v>
+        <x:v>461</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="42" customHeight="1">
       <x:c r="A38" s="5" t="s">
-        <x:v>532</x:v>
+        <x:v>527</x:v>
       </x:c>
       <x:c r="B38" s="5" t="s">
-        <x:v>473</x:v>
+        <x:v>468</x:v>
       </x:c>
       <x:c r="C38" s="5" t="s">
-        <x:v>533</x:v>
+        <x:v>528</x:v>
       </x:c>
       <x:c r="D38" s="5" t="s">
-        <x:v>493</x:v>
+        <x:v>488</x:v>
       </x:c>
       <x:c r="E38" s="5" t="s">
-        <x:v>464</x:v>
+        <x:v>459</x:v>
       </x:c>
       <x:c r="F38" s="5" t="s">
-        <x:v>465</x:v>
+        <x:v>460</x:v>
       </x:c>
       <x:c r="G38" s="7" t="s">
-        <x:v>466</x:v>
+        <x:v>461</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="42" customHeight="1">
       <x:c r="A39" s="6" t="s">
-        <x:v>534</x:v>
+        <x:v>529</x:v>
       </x:c>
       <x:c r="B39" s="6" t="s">
-        <x:v>473</x:v>
+        <x:v>468</x:v>
       </x:c>
       <x:c r="C39" s="6" t="s">
-        <x:v>535</x:v>
+        <x:v>530</x:v>
       </x:c>
       <x:c r="D39" s="6" t="s">
-        <x:v>493</x:v>
+        <x:v>488</x:v>
       </x:c>
       <x:c r="E39" s="6" t="s">
-        <x:v>464</x:v>
+        <x:v>459</x:v>
       </x:c>
       <x:c r="F39" s="6" t="s">
-        <x:v>465</x:v>
+        <x:v>460</x:v>
       </x:c>
       <x:c r="G39" s="7" t="s">
-        <x:v>466</x:v>
+        <x:v>461</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="42" customHeight="1">
       <x:c r="A40" s="5" t="s">
-        <x:v>536</x:v>
+        <x:v>531</x:v>
       </x:c>
       <x:c r="B40" s="5" t="s">
-        <x:v>473</x:v>
+        <x:v>468</x:v>
       </x:c>
       <x:c r="C40" s="5" t="s">
-        <x:v>537</x:v>
+        <x:v>532</x:v>
       </x:c>
       <x:c r="D40" s="5" t="s">
-        <x:v>493</x:v>
+        <x:v>488</x:v>
       </x:c>
       <x:c r="E40" s="5" t="s">
-        <x:v>464</x:v>
+        <x:v>459</x:v>
       </x:c>
       <x:c r="F40" s="5" t="s">
-        <x:v>465</x:v>
+        <x:v>460</x:v>
       </x:c>
       <x:c r="G40" s="7" t="s">
-        <x:v>466</x:v>
+        <x:v>461</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="42" customHeight="1">
       <x:c r="A41" s="6" t="s">
-        <x:v>538</x:v>
+        <x:v>533</x:v>
       </x:c>
       <x:c r="B41" s="6" t="s">
-        <x:v>473</x:v>
+        <x:v>468</x:v>
       </x:c>
       <x:c r="C41" s="6" t="s">
-        <x:v>539</x:v>
+        <x:v>534</x:v>
       </x:c>
       <x:c r="D41" s="6" t="s">
-        <x:v>493</x:v>
+        <x:v>488</x:v>
       </x:c>
       <x:c r="E41" s="6" t="s">
-        <x:v>464</x:v>
+        <x:v>459</x:v>
       </x:c>
       <x:c r="F41" s="6" t="s">
-        <x:v>465</x:v>
+        <x:v>460</x:v>
       </x:c>
       <x:c r="G41" s="7" t="s">
-        <x:v>466</x:v>
+        <x:v>461</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="42" customHeight="1">
       <x:c r="A42" s="5" t="s">
-        <x:v>540</x:v>
+        <x:v>535</x:v>
       </x:c>
       <x:c r="B42" s="5" t="s">
-        <x:v>473</x:v>
+        <x:v>468</x:v>
       </x:c>
       <x:c r="C42" s="5" t="s">
-        <x:v>541</x:v>
+        <x:v>536</x:v>
       </x:c>
       <x:c r="D42" s="5" t="s">
-        <x:v>493</x:v>
+        <x:v>488</x:v>
       </x:c>
       <x:c r="E42" s="5" t="s">
-        <x:v>464</x:v>
+        <x:v>459</x:v>
       </x:c>
       <x:c r="F42" s="5" t="s">
-        <x:v>465</x:v>
+        <x:v>460</x:v>
       </x:c>
       <x:c r="G42" s="7" t="s">
-        <x:v>466</x:v>
+        <x:v>461</x:v>
       </x:c>
     </x:row>
     <x:row r="43" ht="42" customHeight="1">
       <x:c r="A43" s="6" t="s">
-        <x:v>542</x:v>
+        <x:v>537</x:v>
       </x:c>
       <x:c r="B43" s="6" t="s">
-        <x:v>473</x:v>
+        <x:v>468</x:v>
       </x:c>
       <x:c r="C43" s="6" t="s">
-        <x:v>543</x:v>
+        <x:v>538</x:v>
       </x:c>
       <x:c r="D43" s="6" t="s">
-        <x:v>493</x:v>
+        <x:v>488</x:v>
       </x:c>
       <x:c r="E43" s="6" t="s">
-        <x:v>464</x:v>
+        <x:v>459</x:v>
       </x:c>
       <x:c r="F43" s="6" t="s">
-        <x:v>465</x:v>
+        <x:v>460</x:v>
       </x:c>
       <x:c r="G43" s="7" t="s">
-        <x:v>466</x:v>
+        <x:v>461</x:v>
       </x:c>
     </x:row>
     <x:row r="44" ht="42" customHeight="1">
       <x:c r="A44" s="5" t="s">
-        <x:v>544</x:v>
+        <x:v>539</x:v>
       </x:c>
       <x:c r="B44" s="5" t="s">
-        <x:v>473</x:v>
+        <x:v>468</x:v>
       </x:c>
       <x:c r="C44" s="5" t="s">
-        <x:v>545</x:v>
+        <x:v>540</x:v>
       </x:c>
       <x:c r="D44" s="5" t="s">
-        <x:v>493</x:v>
+        <x:v>488</x:v>
       </x:c>
       <x:c r="E44" s="5" t="s">
-        <x:v>464</x:v>
+        <x:v>459</x:v>
       </x:c>
       <x:c r="F44" s="5" t="s">
-        <x:v>465</x:v>
+        <x:v>460</x:v>
       </x:c>
       <x:c r="G44" s="7" t="s">
-        <x:v>466</x:v>
+        <x:v>461</x:v>
       </x:c>
     </x:row>
     <x:row r="45" ht="42" customHeight="1">
       <x:c r="A45" s="6" t="s">
-        <x:v>546</x:v>
+        <x:v>541</x:v>
       </x:c>
       <x:c r="B45" s="6" t="s">
-        <x:v>473</x:v>
+        <x:v>468</x:v>
       </x:c>
       <x:c r="C45" s="6" t="s">
-        <x:v>547</x:v>
+        <x:v>542</x:v>
       </x:c>
       <x:c r="D45" s="6" t="s">
-        <x:v>493</x:v>
+        <x:v>488</x:v>
       </x:c>
       <x:c r="E45" s="6" t="s">
-        <x:v>464</x:v>
+        <x:v>459</x:v>
       </x:c>
       <x:c r="F45" s="6" t="s">
-        <x:v>465</x:v>
+        <x:v>460</x:v>
       </x:c>
       <x:c r="G45" s="7" t="s">
-        <x:v>466</x:v>
+        <x:v>461</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="42" customHeight="1">
       <x:c r="A46" s="5" t="s">
-        <x:v>548</x:v>
+        <x:v>543</x:v>
       </x:c>
       <x:c r="B46" s="5" t="s">
-        <x:v>473</x:v>
+        <x:v>468</x:v>
       </x:c>
       <x:c r="C46" s="5" t="s">
-        <x:v>549</x:v>
+        <x:v>544</x:v>
       </x:c>
       <x:c r="D46" s="5" t="s">
-        <x:v>493</x:v>
+        <x:v>488</x:v>
       </x:c>
       <x:c r="E46" s="5" t="s">
-        <x:v>464</x:v>
+        <x:v>459</x:v>
       </x:c>
       <x:c r="F46" s="5" t="s">
-        <x:v>465</x:v>
+        <x:v>460</x:v>
       </x:c>
       <x:c r="G46" s="7" t="s">
-        <x:v>466</x:v>
+        <x:v>461</x:v>
       </x:c>
     </x:row>
     <x:row r="47" ht="42" customHeight="1">
       <x:c r="A47" s="6" t="s">
-        <x:v>550</x:v>
+        <x:v>545</x:v>
       </x:c>
       <x:c r="B47" s="6" t="s">
-        <x:v>473</x:v>
+        <x:v>468</x:v>
       </x:c>
       <x:c r="C47" s="6" t="s">
-        <x:v>551</x:v>
+        <x:v>546</x:v>
       </x:c>
       <x:c r="D47" s="6" t="s">
-        <x:v>493</x:v>
+        <x:v>488</x:v>
       </x:c>
       <x:c r="E47" s="6" t="s">
-        <x:v>464</x:v>
+        <x:v>459</x:v>
       </x:c>
       <x:c r="F47" s="6" t="s">
-        <x:v>465</x:v>
+        <x:v>460</x:v>
       </x:c>
       <x:c r="G47" s="7" t="s">
-        <x:v>466</x:v>
+        <x:v>461</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="42" customHeight="1">
       <x:c r="A48" s="5" t="s">
-        <x:v>552</x:v>
+        <x:v>547</x:v>
       </x:c>
       <x:c r="B48" s="5" t="s">
-        <x:v>473</x:v>
+        <x:v>468</x:v>
       </x:c>
       <x:c r="C48" s="5" t="s">
-        <x:v>553</x:v>
+        <x:v>548</x:v>
       </x:c>
       <x:c r="D48" s="5" t="s">
-        <x:v>493</x:v>
+        <x:v>488</x:v>
       </x:c>
       <x:c r="E48" s="5" t="s">
-        <x:v>464</x:v>
+        <x:v>459</x:v>
       </x:c>
       <x:c r="F48" s="5" t="s">
-        <x:v>465</x:v>
+        <x:v>460</x:v>
       </x:c>
       <x:c r="G48" s="7" t="s">
-        <x:v>466</x:v>
+        <x:v>461</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="42" customHeight="1">
       <x:c r="A49" s="6" t="s">
-        <x:v>554</x:v>
+        <x:v>549</x:v>
       </x:c>
       <x:c r="B49" s="6" t="s">
-        <x:v>473</x:v>
+        <x:v>468</x:v>
       </x:c>
       <x:c r="C49" s="6" t="s">
-        <x:v>555</x:v>
+        <x:v>550</x:v>
       </x:c>
       <x:c r="D49" s="6" t="s">
-        <x:v>493</x:v>
+        <x:v>488</x:v>
       </x:c>
       <x:c r="E49" s="6" t="s">
-        <x:v>464</x:v>
+        <x:v>459</x:v>
       </x:c>
       <x:c r="F49" s="6" t="s">
-        <x:v>465</x:v>
+        <x:v>460</x:v>
       </x:c>
       <x:c r="G49" s="7" t="s">
-        <x:v>466</x:v>
+        <x:v>461</x:v>
       </x:c>
     </x:row>
     <x:row r="50" ht="42" customHeight="1">
       <x:c r="A50" s="5" t="s">
-        <x:v>556</x:v>
+        <x:v>551</x:v>
       </x:c>
       <x:c r="B50" s="5" t="s">
-        <x:v>473</x:v>
+        <x:v>468</x:v>
       </x:c>
       <x:c r="C50" s="5" t="s">
-        <x:v>557</x:v>
+        <x:v>552</x:v>
       </x:c>
       <x:c r="D50" s="5" t="s">
-        <x:v>493</x:v>
+        <x:v>488</x:v>
       </x:c>
       <x:c r="E50" s="5" t="s">
-        <x:v>464</x:v>
+        <x:v>459</x:v>
       </x:c>
       <x:c r="F50" s="5" t="s">
-        <x:v>465</x:v>
+        <x:v>460</x:v>
       </x:c>
       <x:c r="G50" s="7" t="s">
-        <x:v>466</x:v>
+        <x:v>461</x:v>
       </x:c>
     </x:row>
     <x:row r="51" ht="42" customHeight="1">
       <x:c r="A51" s="6" t="s">
-        <x:v>558</x:v>
+        <x:v>553</x:v>
       </x:c>
       <x:c r="B51" s="6" t="s">
-        <x:v>473</x:v>
+        <x:v>468</x:v>
       </x:c>
       <x:c r="C51" s="6" t="s">
-        <x:v>559</x:v>
+        <x:v>554</x:v>
       </x:c>
       <x:c r="D51" s="6" t="s">
-        <x:v>493</x:v>
+        <x:v>488</x:v>
       </x:c>
       <x:c r="E51" s="6" t="s">
-        <x:v>464</x:v>
+        <x:v>459</x:v>
       </x:c>
       <x:c r="F51" s="6" t="s">
-        <x:v>465</x:v>
+        <x:v>460</x:v>
       </x:c>
       <x:c r="G51" s="7" t="s">
-        <x:v>466</x:v>
+        <x:v>461</x:v>
       </x:c>
     </x:row>
     <x:row r="52" ht="42" customHeight="1">
       <x:c r="A52" s="5" t="s">
-        <x:v>560</x:v>
+        <x:v>555</x:v>
       </x:c>
       <x:c r="B52" s="5" t="s">
-        <x:v>473</x:v>
+        <x:v>468</x:v>
       </x:c>
       <x:c r="C52" s="5" t="s">
-        <x:v>561</x:v>
+        <x:v>556</x:v>
       </x:c>
       <x:c r="D52" s="5" t="s">
-        <x:v>493</x:v>
+        <x:v>488</x:v>
       </x:c>
       <x:c r="E52" s="5" t="s">
-        <x:v>464</x:v>
+        <x:v>459</x:v>
       </x:c>
       <x:c r="F52" s="5" t="s">
-        <x:v>465</x:v>
+        <x:v>460</x:v>
       </x:c>
       <x:c r="G52" s="7" t="s">
-        <x:v>466</x:v>
+        <x:v>461</x:v>
       </x:c>
     </x:row>
     <x:row r="53" ht="42" customHeight="1">
       <x:c r="A53" s="6" t="s">
-        <x:v>562</x:v>
+        <x:v>557</x:v>
       </x:c>
       <x:c r="B53" s="6" t="s">
-        <x:v>473</x:v>
+        <x:v>468</x:v>
       </x:c>
       <x:c r="C53" s="6" t="s">
-        <x:v>563</x:v>
+        <x:v>558</x:v>
       </x:c>
       <x:c r="D53" s="6" t="s">
-        <x:v>493</x:v>
+        <x:v>488</x:v>
       </x:c>
       <x:c r="E53" s="6" t="s">
-        <x:v>464</x:v>
+        <x:v>459</x:v>
       </x:c>
       <x:c r="F53" s="6" t="s">
-        <x:v>465</x:v>
+        <x:v>460</x:v>
       </x:c>
       <x:c r="G53" s="7" t="s">
-        <x:v>466</x:v>
+        <x:v>461</x:v>
       </x:c>
     </x:row>
     <x:row r="54" ht="42" customHeight="1">
       <x:c r="A54" s="5" t="s">
-        <x:v>564</x:v>
+        <x:v>559</x:v>
       </x:c>
       <x:c r="B54" s="5" t="s">
-        <x:v>473</x:v>
+        <x:v>468</x:v>
       </x:c>
       <x:c r="C54" s="5" t="s">
-        <x:v>565</x:v>
+        <x:v>560</x:v>
       </x:c>
       <x:c r="D54" s="5" t="s">
-        <x:v>493</x:v>
+        <x:v>488</x:v>
       </x:c>
       <x:c r="E54" s="5" t="s">
-        <x:v>464</x:v>
+        <x:v>459</x:v>
       </x:c>
       <x:c r="F54" s="5" t="s">
-        <x:v>465</x:v>
+        <x:v>460</x:v>
       </x:c>
       <x:c r="G54" s="7" t="s">
-        <x:v>466</x:v>
+        <x:v>461</x:v>
       </x:c>
     </x:row>
     <x:row r="55" ht="42" customHeight="1">
       <x:c r="A55" s="6" t="s">
-        <x:v>566</x:v>
+        <x:v>561</x:v>
       </x:c>
       <x:c r="B55" s="6" t="s">
-        <x:v>473</x:v>
+        <x:v>468</x:v>
       </x:c>
       <x:c r="C55" s="6" t="s">
-        <x:v>567</x:v>
+        <x:v>562</x:v>
       </x:c>
       <x:c r="D55" s="6" t="s">
-        <x:v>493</x:v>
+        <x:v>488</x:v>
       </x:c>
       <x:c r="E55" s="6" t="s">
-        <x:v>464</x:v>
+        <x:v>459</x:v>
       </x:c>
       <x:c r="F55" s="6" t="s">
-        <x:v>465</x:v>
+        <x:v>460</x:v>
       </x:c>
       <x:c r="G55" s="7" t="s">
-        <x:v>466</x:v>
+        <x:v>461</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R70dc1d4ea3f74ee5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R82e9f932a39d44ca"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Clarify build artifact differences and website acceptance
</commit_message>
<xml_diff>
--- a/01_要件定義/outputs/requirements-v01/PhotonCam_AWS_要件定義_v0.1.xlsx
+++ b/01_要件定義/outputs/requirements-v01/PhotonCam_AWS_要件定義_v0.1.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_概要" sheetId="1" r:id="Rb880a7089ffa4e70"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_范围" sheetId="2" r:id="R7d507f3a29344388"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_现状依据" sheetId="3" r:id="R0cda765281f64896"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_要件清单" sheetId="4" r:id="R039dd51158bb4e92"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_验收条件" sheetId="5" r:id="R25b80ccfb539499d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_待确认" sheetId="6" r:id="R1e2dd30bf396471d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_阶段评审" sheetId="7" r:id="R2950eabd305b4dd4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_页面基线" sheetId="8" r:id="R6f71628a7b6b4fdf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_概要" sheetId="1" r:id="R4ce8f4b2a7414fcf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_范围" sheetId="2" r:id="Rc407dd36ccc84396"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_现状依据" sheetId="3" r:id="R10b59b8629584ce2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_要件清单" sheetId="4" r:id="R37f010ef8bae402a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_验收条件" sheetId="5" r:id="R05b0431665f441a1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_待确认" sheetId="6" r:id="Rfa32959397fd46cd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_阶段评审" sheetId="7" r:id="Rdcc5e849c44f45b8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_页面基线" sheetId="8" r:id="Rbb426468a2ba47b0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -332,9 +332,6 @@
     <x:t xml:space="preserve">源码与发布包构建调查.md</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">不是源码与线上全部内容一致的证明</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">S09</x:t>
   </x:si>
   <x:si>
@@ -464,9 +461,6 @@
     <x:t xml:space="preserve">R09</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">以源码构建出的 build 静态产物进行 dev 部署演练。</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">S01,S04</x:t>
   </x:si>
   <x:si>
@@ -752,9 +746,6 @@
     <x:t xml:space="preserve">Q04 已决策</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">解决清单和锁文件冲突；两次干净构建均成功；记录版本与差异原因。</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">安装与构建日志、版本清单</x:t>
   </x:si>
   <x:si>
@@ -765,12 +756,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">R08 完成</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">构建输出含中英文 HTML、JS、CSS、图片；关键页面对照基线通过。</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">产物清单、哈希、页面核对</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">A10 / R10</x:t>
@@ -2384,7 +2369,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R153778ef704a4ffb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3ed34d9043f749f0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2620,7 +2605,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R852f621e560e403c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb03a456f10f84dc0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2833,7 +2818,7 @@
         <x:v>dev提交572c5a1311151acd45a361aa718f59070bfde32d；未核对正式原仓库，不证明两库同版</x:v>
       </x:c>
     </x:row>
-    <x:row r="13" ht="42" customHeight="1">
+    <x:row r="13" ht="95" customHeight="1">
       <x:c r="A13" s="6" t="s">
         <x:v>102</x:v>
       </x:c>
@@ -2849,33 +2834,33 @@
       <x:c r="E13" s="6" t="s">
         <x:v>104</x:v>
       </x:c>
-      <x:c r="F13" s="6" t="s">
-        <x:v>105</x:v>
+      <x:c r="F13" s="6" t="str">
+        <x:v>94个static文件一致，不证明全部构建产物一致；生成文件可有差异，须解释并验证内容与功能</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="42" customHeight="1">
       <x:c r="A14" s="5" t="s">
-        <x:v>106</x:v>
+        <x:v>105</x:v>
       </x:c>
       <x:c r="B14" s="5" t="s">
         <x:v>79</x:v>
       </x:c>
       <x:c r="C14" s="5" t="s">
-        <x:v>107</x:v>
+        <x:v>106</x:v>
       </x:c>
       <x:c r="D14" s="5" t="s">
         <x:v>90</x:v>
       </x:c>
       <x:c r="E14" s="5" t="s">
+        <x:v>107</x:v>
+      </x:c>
+      <x:c r="F14" s="5" t="s">
         <x:v>108</x:v>
-      </x:c>
-      <x:c r="F14" s="5" t="s">
-        <x:v>109</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="42" customHeight="1">
       <x:c r="A15" s="6" t="s">
-        <x:v>110</x:v>
+        <x:v>109</x:v>
       </x:c>
       <x:c r="B15" s="6" t="str">
         <x:v>开发者说明与调查</x:v>
@@ -2976,7 +2961,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R20a091d018994d41"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R92c29469456e4dfe"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3005,7 +2990,7 @@
     </x:row>
     <x:row r="2" ht="21">
       <x:c r="A2" s="2" t="s">
-        <x:v>111</x:v>
+        <x:v>110</x:v>
       </x:c>
       <x:c r="B2" s="1"/>
       <x:c r="C2" s="1"/>
@@ -3016,7 +3001,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="3" t="s">
-        <x:v>112</x:v>
+        <x:v>111</x:v>
       </x:c>
       <x:c r="B3" s="1"/>
       <x:c r="C3" s="1"/>
@@ -3036,148 +3021,148 @@
     </x:row>
     <x:row r="5" ht="37.95000076293945" customHeight="1">
       <x:c r="A5" s="4" t="s">
+        <x:v>112</x:v>
+      </x:c>
+      <x:c r="B5" s="4" t="s">
         <x:v>113</x:v>
       </x:c>
-      <x:c r="B5" s="4" t="s">
+      <x:c r="C5" s="4" t="s">
         <x:v>114</x:v>
-      </x:c>
-      <x:c r="C5" s="4" t="s">
-        <x:v>115</x:v>
       </x:c>
       <x:c r="D5" s="4" t="s">
         <x:v>68</x:v>
       </x:c>
       <x:c r="E5" s="4" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="F5" s="4" t="s">
         <x:v>116</x:v>
       </x:c>
-      <x:c r="F5" s="4" t="s">
+      <x:c r="G5" s="4" t="s">
         <x:v>117</x:v>
-      </x:c>
-      <x:c r="G5" s="4" t="s">
-        <x:v>118</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="42" customHeight="1">
       <x:c r="A6" s="5" t="s">
+        <x:v>118</x:v>
+      </x:c>
+      <x:c r="B6" s="5" t="s">
         <x:v>119</x:v>
       </x:c>
-      <x:c r="B6" s="5" t="s">
+      <x:c r="C6" s="5" t="s">
         <x:v>120</x:v>
-      </x:c>
-      <x:c r="C6" s="5" t="s">
-        <x:v>121</x:v>
       </x:c>
       <x:c r="D6" s="5" t="s">
         <x:v>46</x:v>
       </x:c>
       <x:c r="E6" s="7" t="s">
+        <x:v>121</x:v>
+      </x:c>
+      <x:c r="F6" s="7" t="s">
         <x:v>122</x:v>
       </x:c>
-      <x:c r="F6" s="7" t="s">
+      <x:c r="G6" s="5" t="s">
         <x:v>123</x:v>
-      </x:c>
-      <x:c r="G6" s="5" t="s">
-        <x:v>124</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="42" customHeight="1">
       <x:c r="A7" s="6" t="s">
+        <x:v>124</x:v>
+      </x:c>
+      <x:c r="B7" s="6" t="s">
         <x:v>125</x:v>
       </x:c>
-      <x:c r="B7" s="6" t="s">
+      <x:c r="C7" s="6" t="s">
         <x:v>126</x:v>
       </x:c>
-      <x:c r="C7" s="6" t="s">
+      <x:c r="D7" s="6" t="s">
         <x:v>127</x:v>
       </x:c>
-      <x:c r="D7" s="6" t="s">
+      <x:c r="E7" s="7" t="s">
+        <x:v>121</x:v>
+      </x:c>
+      <x:c r="F7" s="7" t="s">
+        <x:v>122</x:v>
+      </x:c>
+      <x:c r="G7" s="6" t="s">
         <x:v>128</x:v>
-      </x:c>
-      <x:c r="E7" s="7" t="s">
-        <x:v>122</x:v>
-      </x:c>
-      <x:c r="F7" s="7" t="s">
-        <x:v>123</x:v>
-      </x:c>
-      <x:c r="G7" s="6" t="s">
-        <x:v>129</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="42" customHeight="1">
       <x:c r="A8" s="5" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="B8" s="5" t="s">
+        <x:v>125</x:v>
+      </x:c>
+      <x:c r="C8" s="5" t="s">
         <x:v>130</x:v>
-      </x:c>
-      <x:c r="B8" s="5" t="s">
-        <x:v>126</x:v>
-      </x:c>
-      <x:c r="C8" s="5" t="s">
-        <x:v>131</x:v>
       </x:c>
       <x:c r="D8" s="5" t="s">
         <x:v>84</x:v>
       </x:c>
       <x:c r="E8" s="7" t="s">
+        <x:v>131</x:v>
+      </x:c>
+      <x:c r="F8" s="7" t="s">
+        <x:v>122</x:v>
+      </x:c>
+      <x:c r="G8" s="5" t="s">
         <x:v>132</x:v>
-      </x:c>
-      <x:c r="F8" s="7" t="s">
-        <x:v>123</x:v>
-      </x:c>
-      <x:c r="G8" s="5" t="s">
-        <x:v>133</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="42" customHeight="1">
       <x:c r="A9" s="6" t="s">
+        <x:v>133</x:v>
+      </x:c>
+      <x:c r="B9" s="6" t="s">
+        <x:v>125</x:v>
+      </x:c>
+      <x:c r="C9" s="6" t="s">
         <x:v>134</x:v>
-      </x:c>
-      <x:c r="B9" s="6" t="s">
-        <x:v>126</x:v>
-      </x:c>
-      <x:c r="C9" s="6" t="s">
-        <x:v>135</x:v>
       </x:c>
       <x:c r="D9" s="6" t="s">
         <x:v>84</x:v>
       </x:c>
       <x:c r="E9" s="7" t="s">
-        <x:v>132</x:v>
+        <x:v>131</x:v>
       </x:c>
       <x:c r="F9" s="7" t="s">
-        <x:v>123</x:v>
+        <x:v>122</x:v>
       </x:c>
       <x:c r="G9" s="6" t="s">
-        <x:v>136</x:v>
+        <x:v>135</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="42" customHeight="1">
       <x:c r="A10" s="5" t="s">
+        <x:v>136</x:v>
+      </x:c>
+      <x:c r="B10" s="5" t="s">
+        <x:v>125</x:v>
+      </x:c>
+      <x:c r="C10" s="5" t="s">
         <x:v>137</x:v>
       </x:c>
-      <x:c r="B10" s="5" t="s">
-        <x:v>126</x:v>
-      </x:c>
-      <x:c r="C10" s="5" t="s">
-        <x:v>138</x:v>
-      </x:c>
       <x:c r="D10" s="5" t="s">
-        <x:v>128</x:v>
+        <x:v>127</x:v>
       </x:c>
       <x:c r="E10" s="7" t="s">
+        <x:v>131</x:v>
+      </x:c>
+      <x:c r="F10" s="7" t="s">
+        <x:v>122</x:v>
+      </x:c>
+      <x:c r="G10" s="5" t="s">
         <x:v>132</x:v>
-      </x:c>
-      <x:c r="F10" s="7" t="s">
-        <x:v>123</x:v>
-      </x:c>
-      <x:c r="G10" s="5" t="s">
-        <x:v>133</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="42" customHeight="1">
       <x:c r="A11" s="6" t="s">
-        <x:v>139</x:v>
+        <x:v>138</x:v>
       </x:c>
       <x:c r="B11" s="6" t="s">
-        <x:v>126</x:v>
+        <x:v>125</x:v>
       </x:c>
       <x:c r="C11" s="6" t="str">
         <x:v>正式环境续用 juniperphoton.dev/photoncam/，深层链接、刷新和资源路径正常；dev地址另定。</x:v>
@@ -3186,366 +3171,366 @@
         <x:v>S02,S04,S11</x:v>
       </x:c>
       <x:c r="E11" s="7" t="s">
+        <x:v>121</x:v>
+      </x:c>
+      <x:c r="F11" s="7" t="s">
         <x:v>122</x:v>
       </x:c>
-      <x:c r="F11" s="7" t="s">
-        <x:v>123</x:v>
-      </x:c>
       <x:c r="G11" s="6" t="s">
-        <x:v>129</x:v>
+        <x:v>128</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="42" customHeight="1">
       <x:c r="A12" s="5" t="s">
+        <x:v>139</x:v>
+      </x:c>
+      <x:c r="B12" s="5" t="s">
+        <x:v>125</x:v>
+      </x:c>
+      <x:c r="C12" s="5" t="s">
         <x:v>140</x:v>
       </x:c>
-      <x:c r="B12" s="5" t="s">
-        <x:v>126</x:v>
-      </x:c>
-      <x:c r="C12" s="5" t="s">
+      <x:c r="D12" s="5" t="s">
         <x:v>141</x:v>
       </x:c>
-      <x:c r="D12" s="5" t="s">
-        <x:v>142</x:v>
-      </x:c>
       <x:c r="E12" s="7" t="s">
-        <x:v>132</x:v>
+        <x:v>131</x:v>
       </x:c>
       <x:c r="F12" s="7" t="s">
-        <x:v>123</x:v>
+        <x:v>122</x:v>
       </x:c>
       <x:c r="G12" s="5" t="s">
-        <x:v>129</x:v>
+        <x:v>128</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="42" customHeight="1">
       <x:c r="A13" s="6" t="s">
+        <x:v>142</x:v>
+      </x:c>
+      <x:c r="B13" s="6" t="s">
         <x:v>143</x:v>
       </x:c>
-      <x:c r="B13" s="6" t="s">
+      <x:c r="C13" s="6" t="s">
         <x:v>144</x:v>
       </x:c>
-      <x:c r="C13" s="6" t="s">
+      <x:c r="D13" s="6" t="s">
         <x:v>145</x:v>
       </x:c>
-      <x:c r="D13" s="6" t="s">
+      <x:c r="E13" s="7" t="s">
+        <x:v>121</x:v>
+      </x:c>
+      <x:c r="F13" s="7" t="s">
+        <x:v>122</x:v>
+      </x:c>
+      <x:c r="G13" s="6" t="s">
         <x:v>146</x:v>
       </x:c>
-      <x:c r="E13" s="7" t="s">
+    </x:row>
+    <x:row r="14" ht="85" customHeight="1">
+      <x:c r="A14" s="5" t="s">
+        <x:v>147</x:v>
+      </x:c>
+      <x:c r="B14" s="5" t="s">
+        <x:v>143</x:v>
+      </x:c>
+      <x:c r="C14" s="5" t="str">
+        <x:v>以源码生成的静态产物进行dev部署；生成文件可与旧ZIP不同，但差异须可解释，页面内容和功能须符合约定。</x:v>
+      </x:c>
+      <x:c r="D14" s="5" t="s">
+        <x:v>148</x:v>
+      </x:c>
+      <x:c r="E14" s="7" t="s">
+        <x:v>121</x:v>
+      </x:c>
+      <x:c r="F14" s="7" t="s">
         <x:v>122</x:v>
       </x:c>
-      <x:c r="F13" s="7" t="s">
-        <x:v>123</x:v>
-      </x:c>
-      <x:c r="G13" s="6" t="s">
-        <x:v>147</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14" ht="42" customHeight="1">
-      <x:c r="A14" s="5" t="s">
-        <x:v>148</x:v>
-      </x:c>
-      <x:c r="B14" s="5" t="s">
-        <x:v>144</x:v>
-      </x:c>
-      <x:c r="C14" s="5" t="s">
-        <x:v>149</x:v>
-      </x:c>
-      <x:c r="D14" s="5" t="s">
-        <x:v>150</x:v>
-      </x:c>
-      <x:c r="E14" s="7" t="s">
-        <x:v>122</x:v>
-      </x:c>
-      <x:c r="F14" s="7" t="s">
-        <x:v>123</x:v>
-      </x:c>
       <x:c r="G14" s="5" t="s">
-        <x:v>147</x:v>
+        <x:v>146</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="42" customHeight="1">
       <x:c r="A15" s="6" t="s">
+        <x:v>149</x:v>
+      </x:c>
+      <x:c r="B15" s="6" t="s">
+        <x:v>150</x:v>
+      </x:c>
+      <x:c r="C15" s="6" t="s">
         <x:v>151</x:v>
-      </x:c>
-      <x:c r="B15" s="6" t="s">
-        <x:v>152</x:v>
-      </x:c>
-      <x:c r="C15" s="6" t="s">
-        <x:v>153</x:v>
       </x:c>
       <x:c r="D15" s="6" t="s">
         <x:v>51</x:v>
       </x:c>
       <x:c r="E15" s="7" t="s">
+        <x:v>121</x:v>
+      </x:c>
+      <x:c r="F15" s="7" t="s">
         <x:v>122</x:v>
       </x:c>
-      <x:c r="F15" s="7" t="s">
-        <x:v>123</x:v>
-      </x:c>
       <x:c r="G15" s="6" t="s">
-        <x:v>147</x:v>
+        <x:v>146</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="42" customHeight="1">
       <x:c r="A16" s="5" t="s">
-        <x:v>154</x:v>
+        <x:v>152</x:v>
       </x:c>
       <x:c r="B16" s="5" t="s">
-        <x:v>152</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="C16" s="5" t="s">
-        <x:v>155</x:v>
+        <x:v>153</x:v>
       </x:c>
       <x:c r="D16" s="5" t="str">
         <x:v>S01,S06,S07</x:v>
       </x:c>
       <x:c r="E16" s="7" t="s">
+        <x:v>121</x:v>
+      </x:c>
+      <x:c r="F16" s="7" t="s">
         <x:v>122</x:v>
       </x:c>
-      <x:c r="F16" s="7" t="s">
-        <x:v>123</x:v>
-      </x:c>
       <x:c r="G16" s="5" t="s">
-        <x:v>156</x:v>
+        <x:v>154</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="42" customHeight="1">
       <x:c r="A17" s="6" t="s">
-        <x:v>157</x:v>
+        <x:v>155</x:v>
       </x:c>
       <x:c r="B17" s="6" t="s">
-        <x:v>152</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="C17" s="6" t="s">
-        <x:v>158</x:v>
+        <x:v>156</x:v>
       </x:c>
       <x:c r="D17" s="6" t="s">
-        <x:v>142</x:v>
+        <x:v>141</x:v>
       </x:c>
       <x:c r="E17" s="7" t="s">
-        <x:v>132</x:v>
+        <x:v>131</x:v>
       </x:c>
       <x:c r="F17" s="7" t="s">
-        <x:v>123</x:v>
+        <x:v>122</x:v>
       </x:c>
       <x:c r="G17" s="6" t="s">
-        <x:v>156</x:v>
+        <x:v>154</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="42" customHeight="1">
       <x:c r="A18" s="5" t="s">
+        <x:v>157</x:v>
+      </x:c>
+      <x:c r="B18" s="5" t="s">
+        <x:v>150</x:v>
+      </x:c>
+      <x:c r="C18" s="5" t="s">
+        <x:v>158</x:v>
+      </x:c>
+      <x:c r="D18" s="5" t="s">
+        <x:v>141</x:v>
+      </x:c>
+      <x:c r="E18" s="7" t="s">
+        <x:v>131</x:v>
+      </x:c>
+      <x:c r="F18" s="7" t="s">
+        <x:v>122</x:v>
+      </x:c>
+      <x:c r="G18" s="5" t="s">
         <x:v>159</x:v>
-      </x:c>
-      <x:c r="B18" s="5" t="s">
-        <x:v>152</x:v>
-      </x:c>
-      <x:c r="C18" s="5" t="s">
-        <x:v>160</x:v>
-      </x:c>
-      <x:c r="D18" s="5" t="s">
-        <x:v>142</x:v>
-      </x:c>
-      <x:c r="E18" s="7" t="s">
-        <x:v>132</x:v>
-      </x:c>
-      <x:c r="F18" s="7" t="s">
-        <x:v>123</x:v>
-      </x:c>
-      <x:c r="G18" s="5" t="s">
-        <x:v>161</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="42" customHeight="1">
       <x:c r="A19" s="6" t="s">
+        <x:v>160</x:v>
+      </x:c>
+      <x:c r="B19" s="6" t="s">
+        <x:v>161</x:v>
+      </x:c>
+      <x:c r="C19" s="6" t="s">
         <x:v>162</x:v>
-      </x:c>
-      <x:c r="B19" s="6" t="s">
-        <x:v>163</x:v>
-      </x:c>
-      <x:c r="C19" s="6" t="s">
-        <x:v>164</x:v>
       </x:c>
       <x:c r="D19" s="6" t="s">
         <x:v>46</x:v>
       </x:c>
       <x:c r="E19" s="7" t="s">
+        <x:v>121</x:v>
+      </x:c>
+      <x:c r="F19" s="7" t="s">
         <x:v>122</x:v>
       </x:c>
-      <x:c r="F19" s="7" t="s">
-        <x:v>123</x:v>
-      </x:c>
       <x:c r="G19" s="6" t="s">
-        <x:v>136</x:v>
+        <x:v>135</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="42" customHeight="1">
       <x:c r="A20" s="5" t="s">
+        <x:v>163</x:v>
+      </x:c>
+      <x:c r="B20" s="5" t="s">
+        <x:v>161</x:v>
+      </x:c>
+      <x:c r="C20" s="5" t="s">
+        <x:v>164</x:v>
+      </x:c>
+      <x:c r="D20" s="5" t="s">
         <x:v>165</x:v>
       </x:c>
-      <x:c r="B20" s="5" t="s">
-        <x:v>163</x:v>
-      </x:c>
-      <x:c r="C20" s="5" t="s">
-        <x:v>166</x:v>
-      </x:c>
-      <x:c r="D20" s="5" t="s">
-        <x:v>167</x:v>
-      </x:c>
       <x:c r="E20" s="7" t="s">
+        <x:v>121</x:v>
+      </x:c>
+      <x:c r="F20" s="7" t="s">
         <x:v>122</x:v>
       </x:c>
-      <x:c r="F20" s="7" t="s">
+      <x:c r="G20" s="5" t="s">
         <x:v>123</x:v>
-      </x:c>
-      <x:c r="G20" s="5" t="s">
-        <x:v>124</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="42" customHeight="1">
       <x:c r="A21" s="6" t="s">
-        <x:v>168</x:v>
+        <x:v>166</x:v>
       </x:c>
       <x:c r="B21" s="6" t="s">
-        <x:v>163</x:v>
+        <x:v>161</x:v>
       </x:c>
       <x:c r="C21" s="6" t="s">
-        <x:v>169</x:v>
+        <x:v>167</x:v>
       </x:c>
       <x:c r="D21" s="6" t="s">
-        <x:v>142</x:v>
+        <x:v>141</x:v>
       </x:c>
       <x:c r="E21" s="7" t="s">
-        <x:v>132</x:v>
+        <x:v>131</x:v>
       </x:c>
       <x:c r="F21" s="7" t="s">
+        <x:v>122</x:v>
+      </x:c>
+      <x:c r="G21" s="6" t="s">
         <x:v>123</x:v>
-      </x:c>
-      <x:c r="G21" s="6" t="s">
-        <x:v>124</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="42" customHeight="1">
       <x:c r="A22" s="5" t="s">
+        <x:v>168</x:v>
+      </x:c>
+      <x:c r="B22" s="5" t="s">
+        <x:v>169</x:v>
+      </x:c>
+      <x:c r="C22" s="5" t="s">
         <x:v>170</x:v>
       </x:c>
-      <x:c r="B22" s="5" t="s">
-        <x:v>171</x:v>
-      </x:c>
-      <x:c r="C22" s="5" t="s">
-        <x:v>172</x:v>
-      </x:c>
       <x:c r="D22" s="5" t="s">
-        <x:v>142</x:v>
+        <x:v>141</x:v>
       </x:c>
       <x:c r="E22" s="7" t="s">
+        <x:v>131</x:v>
+      </x:c>
+      <x:c r="F22" s="7" t="s">
+        <x:v>122</x:v>
+      </x:c>
+      <x:c r="G22" s="5" t="s">
         <x:v>132</x:v>
-      </x:c>
-      <x:c r="F22" s="7" t="s">
-        <x:v>123</x:v>
-      </x:c>
-      <x:c r="G22" s="5" t="s">
-        <x:v>133</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="42" customHeight="1">
       <x:c r="A23" s="6" t="s">
-        <x:v>173</x:v>
+        <x:v>171</x:v>
       </x:c>
       <x:c r="B23" s="6" t="s">
-        <x:v>171</x:v>
+        <x:v>169</x:v>
       </x:c>
       <x:c r="C23" s="6" t="s">
-        <x:v>174</x:v>
+        <x:v>172</x:v>
       </x:c>
       <x:c r="D23" s="6" t="s">
         <x:v>31</x:v>
       </x:c>
       <x:c r="E23" s="7" t="s">
-        <x:v>175</x:v>
+        <x:v>173</x:v>
       </x:c>
       <x:c r="F23" s="7" t="s">
-        <x:v>123</x:v>
+        <x:v>122</x:v>
       </x:c>
       <x:c r="G23" s="6" t="s">
-        <x:v>176</x:v>
+        <x:v>174</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="42" customHeight="1">
       <x:c r="A24" s="5" t="s">
+        <x:v>175</x:v>
+      </x:c>
+      <x:c r="B24" s="5" t="s">
+        <x:v>169</x:v>
+      </x:c>
+      <x:c r="C24" s="5" t="s">
+        <x:v>176</x:v>
+      </x:c>
+      <x:c r="D24" s="5" t="s">
         <x:v>177</x:v>
       </x:c>
-      <x:c r="B24" s="5" t="s">
-        <x:v>171</x:v>
-      </x:c>
-      <x:c r="C24" s="5" t="s">
+      <x:c r="E24" s="7" t="s">
+        <x:v>121</x:v>
+      </x:c>
+      <x:c r="F24" s="7" t="s">
+        <x:v>122</x:v>
+      </x:c>
+      <x:c r="G24" s="5" t="s">
         <x:v>178</x:v>
-      </x:c>
-      <x:c r="D24" s="5" t="s">
-        <x:v>179</x:v>
-      </x:c>
-      <x:c r="E24" s="7" t="s">
-        <x:v>122</x:v>
-      </x:c>
-      <x:c r="F24" s="7" t="s">
-        <x:v>123</x:v>
-      </x:c>
-      <x:c r="G24" s="5" t="s">
-        <x:v>180</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="42" customHeight="1">
       <x:c r="A25" s="6" t="s">
+        <x:v>179</x:v>
+      </x:c>
+      <x:c r="B25" s="6" t="s">
+        <x:v>180</x:v>
+      </x:c>
+      <x:c r="C25" s="6" t="s">
         <x:v>181</x:v>
-      </x:c>
-      <x:c r="B25" s="6" t="s">
-        <x:v>182</x:v>
-      </x:c>
-      <x:c r="C25" s="6" t="s">
-        <x:v>183</x:v>
       </x:c>
       <x:c r="D25" s="6" t="s">
         <x:v>31</x:v>
       </x:c>
       <x:c r="E25" s="7" t="s">
-        <x:v>175</x:v>
+        <x:v>173</x:v>
       </x:c>
       <x:c r="F25" s="7" t="s">
-        <x:v>123</x:v>
+        <x:v>122</x:v>
       </x:c>
       <x:c r="G25" s="6" t="s">
-        <x:v>184</x:v>
+        <x:v>182</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="42" customHeight="1">
       <x:c r="A26" s="5" t="s">
+        <x:v>183</x:v>
+      </x:c>
+      <x:c r="B26" s="5" t="s">
+        <x:v>184</x:v>
+      </x:c>
+      <x:c r="C26" s="5" t="s">
         <x:v>185</x:v>
       </x:c>
-      <x:c r="B26" s="5" t="s">
+      <x:c r="D26" s="5" t="s">
+        <x:v>165</x:v>
+      </x:c>
+      <x:c r="E26" s="7" t="s">
+        <x:v>121</x:v>
+      </x:c>
+      <x:c r="F26" s="7" t="s">
+        <x:v>122</x:v>
+      </x:c>
+      <x:c r="G26" s="5" t="s">
         <x:v>186</x:v>
-      </x:c>
-      <x:c r="C26" s="5" t="s">
-        <x:v>187</x:v>
-      </x:c>
-      <x:c r="D26" s="5" t="s">
-        <x:v>167</x:v>
-      </x:c>
-      <x:c r="E26" s="7" t="s">
-        <x:v>122</x:v>
-      </x:c>
-      <x:c r="F26" s="7" t="s">
-        <x:v>123</x:v>
-      </x:c>
-      <x:c r="G26" s="5" t="s">
-        <x:v>188</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="85" customHeight="1">
       <x:c r="A27" s="6" t="s">
-        <x:v>189</x:v>
+        <x:v>187</x:v>
       </x:c>
       <x:c r="B27" s="6" t="s">
-        <x:v>186</x:v>
+        <x:v>184</x:v>
       </x:c>
       <x:c r="C27" s="6" t="str">
         <x:v>仅迁移 /photoncam/ 并保留根首页、主站资源与其他产品入口；正式前确认DNS权限、切换窗口、回退与负责人。</x:v>
@@ -3554,105 +3539,105 @@
         <x:v>S01,S11,S12</x:v>
       </x:c>
       <x:c r="E27" s="7" t="s">
+        <x:v>121</x:v>
+      </x:c>
+      <x:c r="F27" s="7" t="s">
         <x:v>122</x:v>
       </x:c>
-      <x:c r="F27" s="7" t="s">
-        <x:v>123</x:v>
-      </x:c>
       <x:c r="G27" s="6" t="s">
-        <x:v>190</x:v>
+        <x:v>188</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="42" customHeight="1">
       <x:c r="A28" s="5" t="s">
+        <x:v>189</x:v>
+      </x:c>
+      <x:c r="B28" s="5" t="s">
+        <x:v>190</x:v>
+      </x:c>
+      <x:c r="C28" s="5" t="s">
         <x:v>191</x:v>
-      </x:c>
-      <x:c r="B28" s="5" t="s">
-        <x:v>192</x:v>
-      </x:c>
-      <x:c r="C28" s="5" t="s">
-        <x:v>193</x:v>
       </x:c>
       <x:c r="D28" s="5" t="s">
         <x:v>46</x:v>
       </x:c>
       <x:c r="E28" s="7" t="s">
+        <x:v>121</x:v>
+      </x:c>
+      <x:c r="F28" s="7" t="s">
         <x:v>122</x:v>
       </x:c>
-      <x:c r="F28" s="7" t="s">
-        <x:v>123</x:v>
-      </x:c>
       <x:c r="G28" s="5" t="s">
-        <x:v>136</x:v>
+        <x:v>135</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="42" customHeight="1">
       <x:c r="A29" s="6" t="s">
-        <x:v>194</x:v>
+        <x:v>192</x:v>
       </x:c>
       <x:c r="B29" s="6" t="s">
-        <x:v>192</x:v>
+        <x:v>190</x:v>
       </x:c>
       <x:c r="C29" s="6" t="s">
-        <x:v>195</x:v>
+        <x:v>193</x:v>
       </x:c>
       <x:c r="D29" s="6" t="s">
         <x:v>46</x:v>
       </x:c>
       <x:c r="E29" s="7" t="s">
+        <x:v>121</x:v>
+      </x:c>
+      <x:c r="F29" s="7" t="s">
         <x:v>122</x:v>
       </x:c>
-      <x:c r="F29" s="7" t="s">
-        <x:v>123</x:v>
-      </x:c>
       <x:c r="G29" s="6" t="s">
-        <x:v>196</x:v>
+        <x:v>194</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="42" customHeight="1">
       <x:c r="A30" s="5" t="s">
+        <x:v>195</x:v>
+      </x:c>
+      <x:c r="B30" s="5" t="s">
+        <x:v>196</x:v>
+      </x:c>
+      <x:c r="C30" s="5" t="s">
         <x:v>197</x:v>
-      </x:c>
-      <x:c r="B30" s="5" t="s">
-        <x:v>198</x:v>
-      </x:c>
-      <x:c r="C30" s="5" t="s">
-        <x:v>199</x:v>
       </x:c>
       <x:c r="D30" s="5" t="s">
         <x:v>46</x:v>
       </x:c>
       <x:c r="E30" s="7" t="s">
+        <x:v>121</x:v>
+      </x:c>
+      <x:c r="F30" s="7" t="s">
         <x:v>122</x:v>
       </x:c>
-      <x:c r="F30" s="7" t="s">
-        <x:v>123</x:v>
-      </x:c>
       <x:c r="G30" s="5" t="s">
-        <x:v>136</x:v>
+        <x:v>135</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="42" customHeight="1">
       <x:c r="A31" s="6" t="s">
+        <x:v>198</x:v>
+      </x:c>
+      <x:c r="B31" s="6" t="s">
+        <x:v>199</x:v>
+      </x:c>
+      <x:c r="C31" s="6" t="s">
         <x:v>200</x:v>
-      </x:c>
-      <x:c r="B31" s="6" t="s">
-        <x:v>201</x:v>
-      </x:c>
-      <x:c r="C31" s="6" t="s">
-        <x:v>202</x:v>
       </x:c>
       <x:c r="D31" s="6" t="s">
         <x:v>46</x:v>
       </x:c>
       <x:c r="E31" s="7" t="s">
+        <x:v>121</x:v>
+      </x:c>
+      <x:c r="F31" s="7" t="s">
         <x:v>122</x:v>
       </x:c>
-      <x:c r="F31" s="7" t="s">
-        <x:v>123</x:v>
-      </x:c>
       <x:c r="G31" s="6" t="s">
-        <x:v>203</x:v>
+        <x:v>201</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -3669,7 +3654,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R04146f0ed12842bf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2eeeb53c52b14585"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3698,7 +3683,7 @@
     </x:row>
     <x:row r="2" ht="21">
       <x:c r="A2" s="2" t="s">
-        <x:v>204</x:v>
+        <x:v>202</x:v>
       </x:c>
       <x:c r="B2" s="1"/>
       <x:c r="C2" s="1"/>
@@ -3709,7 +3694,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="3" t="s">
-        <x:v>205</x:v>
+        <x:v>203</x:v>
       </x:c>
       <x:c r="B3" s="1"/>
       <x:c r="C3" s="1"/>
@@ -3729,145 +3714,145 @@
     </x:row>
     <x:row r="5" ht="37.95000076293945" customHeight="1">
       <x:c r="A5" s="4" t="s">
+        <x:v>204</x:v>
+      </x:c>
+      <x:c r="B5" s="4" t="s">
+        <x:v>205</x:v>
+      </x:c>
+      <x:c r="C5" s="4" t="s">
         <x:v>206</x:v>
       </x:c>
-      <x:c r="B5" s="4" t="s">
+      <x:c r="D5" s="4" t="s">
         <x:v>207</x:v>
       </x:c>
-      <x:c r="C5" s="4" t="s">
+      <x:c r="E5" s="4" t="s">
         <x:v>208</x:v>
       </x:c>
-      <x:c r="D5" s="4" t="s">
+      <x:c r="F5" s="4" t="s">
         <x:v>209</x:v>
       </x:c>
-      <x:c r="E5" s="4" t="s">
+      <x:c r="G5" s="4" t="s">
         <x:v>210</x:v>
-      </x:c>
-      <x:c r="F5" s="4" t="s">
-        <x:v>211</x:v>
-      </x:c>
-      <x:c r="G5" s="4" t="s">
-        <x:v>212</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="42" customHeight="1">
       <x:c r="A6" s="5" t="s">
+        <x:v>211</x:v>
+      </x:c>
+      <x:c r="B6" s="5" t="s">
+        <x:v>212</x:v>
+      </x:c>
+      <x:c r="C6" s="5" t="s">
         <x:v>213</x:v>
       </x:c>
-      <x:c r="B6" s="5" t="s">
+      <x:c r="D6" s="5" t="s">
         <x:v>214</x:v>
       </x:c>
-      <x:c r="C6" s="5" t="s">
+      <x:c r="E6" s="5" t="s">
         <x:v>215</x:v>
       </x:c>
-      <x:c r="D6" s="5" t="s">
+      <x:c r="F6" s="7" t="s">
         <x:v>216</x:v>
       </x:c>
-      <x:c r="E6" s="5" t="s">
+      <x:c r="G6" s="7" t="s">
         <x:v>217</x:v>
-      </x:c>
-      <x:c r="F6" s="7" t="s">
-        <x:v>218</x:v>
-      </x:c>
-      <x:c r="G6" s="7" t="s">
-        <x:v>219</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="42" customHeight="1">
       <x:c r="A7" s="6" t="s">
+        <x:v>218</x:v>
+      </x:c>
+      <x:c r="B7" s="6" t="s">
+        <x:v>219</x:v>
+      </x:c>
+      <x:c r="C7" s="6" t="s">
         <x:v>220</x:v>
       </x:c>
-      <x:c r="B7" s="6" t="s">
+      <x:c r="D7" s="6" t="s">
         <x:v>221</x:v>
       </x:c>
-      <x:c r="C7" s="6" t="s">
+      <x:c r="E7" s="6" t="s">
         <x:v>222</x:v>
       </x:c>
-      <x:c r="D7" s="6" t="s">
-        <x:v>223</x:v>
-      </x:c>
-      <x:c r="E7" s="6" t="s">
-        <x:v>224</x:v>
-      </x:c>
       <x:c r="F7" s="7" t="s">
-        <x:v>218</x:v>
+        <x:v>216</x:v>
       </x:c>
       <x:c r="G7" s="7" t="s">
-        <x:v>219</x:v>
+        <x:v>217</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="42" customHeight="1">
       <x:c r="A8" s="5" t="s">
+        <x:v>223</x:v>
+      </x:c>
+      <x:c r="B8" s="5" t="s">
+        <x:v>224</x:v>
+      </x:c>
+      <x:c r="C8" s="5" t="s">
         <x:v>225</x:v>
       </x:c>
-      <x:c r="B8" s="5" t="s">
+      <x:c r="D8" s="5" t="s">
         <x:v>226</x:v>
       </x:c>
-      <x:c r="C8" s="5" t="s">
-        <x:v>227</x:v>
-      </x:c>
-      <x:c r="D8" s="5" t="s">
-        <x:v>228</x:v>
-      </x:c>
       <x:c r="E8" s="5" t="s">
-        <x:v>224</x:v>
+        <x:v>222</x:v>
       </x:c>
       <x:c r="F8" s="7" t="s">
-        <x:v>218</x:v>
+        <x:v>216</x:v>
       </x:c>
       <x:c r="G8" s="7" t="s">
-        <x:v>219</x:v>
+        <x:v>217</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="42" customHeight="1">
       <x:c r="A9" s="6" t="s">
+        <x:v>227</x:v>
+      </x:c>
+      <x:c r="B9" s="6" t="s">
+        <x:v>228</x:v>
+      </x:c>
+      <x:c r="C9" s="6" t="s">
         <x:v>229</x:v>
       </x:c>
-      <x:c r="B9" s="6" t="s">
+      <x:c r="D9" s="6" t="s">
         <x:v>230</x:v>
       </x:c>
-      <x:c r="C9" s="6" t="s">
-        <x:v>231</x:v>
-      </x:c>
-      <x:c r="D9" s="6" t="s">
-        <x:v>232</x:v>
-      </x:c>
       <x:c r="E9" s="6" t="s">
-        <x:v>224</x:v>
+        <x:v>222</x:v>
       </x:c>
       <x:c r="F9" s="7" t="s">
-        <x:v>218</x:v>
+        <x:v>216</x:v>
       </x:c>
       <x:c r="G9" s="7" t="s">
-        <x:v>219</x:v>
+        <x:v>217</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="42" customHeight="1">
       <x:c r="A10" s="5" t="s">
+        <x:v>231</x:v>
+      </x:c>
+      <x:c r="B10" s="5" t="s">
+        <x:v>232</x:v>
+      </x:c>
+      <x:c r="C10" s="5" t="s">
         <x:v>233</x:v>
       </x:c>
-      <x:c r="B10" s="5" t="s">
+      <x:c r="D10" s="5" t="s">
         <x:v>234</x:v>
       </x:c>
-      <x:c r="C10" s="5" t="s">
-        <x:v>235</x:v>
-      </x:c>
-      <x:c r="D10" s="5" t="s">
-        <x:v>236</x:v>
-      </x:c>
       <x:c r="E10" s="5" t="s">
-        <x:v>224</x:v>
+        <x:v>222</x:v>
       </x:c>
       <x:c r="F10" s="7" t="s">
-        <x:v>218</x:v>
+        <x:v>216</x:v>
       </x:c>
       <x:c r="G10" s="7" t="s">
-        <x:v>219</x:v>
+        <x:v>217</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="85" customHeight="1">
       <x:c r="A11" s="6" t="s">
-        <x:v>237</x:v>
+        <x:v>235</x:v>
       </x:c>
       <x:c r="B11" s="6" t="str">
         <x:v>dev地址／正式切换方案已定</x:v>
@@ -3876,366 +3861,366 @@
         <x:v>正式URL保持 juniperphoton.dev/photoncam/；中英深层页面直接访问及刷新成功，资源无迁移引入的404。</x:v>
       </x:c>
       <x:c r="D11" s="6" t="s">
-        <x:v>238</x:v>
+        <x:v>236</x:v>
       </x:c>
       <x:c r="E11" s="6" t="s">
-        <x:v>224</x:v>
+        <x:v>222</x:v>
       </x:c>
       <x:c r="F11" s="7" t="s">
-        <x:v>218</x:v>
+        <x:v>216</x:v>
       </x:c>
       <x:c r="G11" s="7" t="s">
-        <x:v>219</x:v>
+        <x:v>217</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="42" customHeight="1">
       <x:c r="A12" s="5" t="s">
+        <x:v>237</x:v>
+      </x:c>
+      <x:c r="B12" s="5" t="s">
+        <x:v>238</x:v>
+      </x:c>
+      <x:c r="C12" s="5" t="s">
         <x:v>239</x:v>
       </x:c>
-      <x:c r="B12" s="5" t="s">
+      <x:c r="D12" s="5" t="s">
         <x:v>240</x:v>
       </x:c>
-      <x:c r="C12" s="5" t="s">
+      <x:c r="E12" s="5" t="s">
+        <x:v>222</x:v>
+      </x:c>
+      <x:c r="F12" s="7" t="s">
+        <x:v>216</x:v>
+      </x:c>
+      <x:c r="G12" s="7" t="s">
+        <x:v>217</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="120" customHeight="1">
+      <x:c r="A13" s="6" t="s">
         <x:v>241</x:v>
       </x:c>
-      <x:c r="D12" s="5" t="s">
+      <x:c r="B13" s="6" t="s">
         <x:v>242</x:v>
       </x:c>
-      <x:c r="E12" s="5" t="s">
-        <x:v>224</x:v>
-      </x:c>
-      <x:c r="F12" s="7" t="s">
-        <x:v>218</x:v>
-      </x:c>
-      <x:c r="G12" s="7" t="s">
-        <x:v>219</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13" ht="42" customHeight="1">
-      <x:c r="A13" s="6" t="s">
+      <x:c r="C13" s="6" t="str">
+        <x:v>统一依赖清单与锁文件，固定提交、环境及配置；两次干净构建成功，记录版本与差异原因。</x:v>
+      </x:c>
+      <x:c r="D13" s="6" t="s">
         <x:v>243</x:v>
       </x:c>
-      <x:c r="B13" s="6" t="s">
+      <x:c r="E13" s="6" t="s">
         <x:v>244</x:v>
       </x:c>
-      <x:c r="C13" s="6" t="s">
+      <x:c r="F13" s="7" t="s">
+        <x:v>216</x:v>
+      </x:c>
+      <x:c r="G13" s="7" t="s">
+        <x:v>217</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="120" customHeight="1">
+      <x:c r="A14" s="5" t="s">
         <x:v>245</x:v>
       </x:c>
-      <x:c r="D13" s="6" t="s">
+      <x:c r="B14" s="5" t="s">
         <x:v>246</x:v>
       </x:c>
-      <x:c r="E13" s="6" t="s">
-        <x:v>247</x:v>
-      </x:c>
-      <x:c r="F13" s="7" t="s">
-        <x:v>218</x:v>
-      </x:c>
-      <x:c r="G13" s="7" t="s">
-        <x:v>219</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14" ht="42" customHeight="1">
-      <x:c r="A14" s="5" t="s">
-        <x:v>248</x:v>
-      </x:c>
-      <x:c r="B14" s="5" t="s">
-        <x:v>249</x:v>
-      </x:c>
-      <x:c r="C14" s="5" t="s">
-        <x:v>250</x:v>
-      </x:c>
-      <x:c r="D14" s="5" t="s">
-        <x:v>251</x:v>
+      <x:c r="C14" s="5" t="str">
+        <x:v>产物含中英文HTML、JS、CSS和图片；记录文件差异原因，按基线验证内容、路径、图片和操作，不要求全部生成文件与旧ZIP哈希相同。</x:v>
+      </x:c>
+      <x:c r="D14" s="5" t="str">
+        <x:v>产物清单、哈希与差异说明、页面及操作记录</x:v>
       </x:c>
       <x:c r="E14" s="5" t="s">
-        <x:v>247</x:v>
+        <x:v>244</x:v>
       </x:c>
       <x:c r="F14" s="7" t="s">
-        <x:v>218</x:v>
+        <x:v>216</x:v>
       </x:c>
       <x:c r="G14" s="7" t="s">
-        <x:v>219</x:v>
+        <x:v>217</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="42" customHeight="1">
       <x:c r="A15" s="6" t="s">
-        <x:v>252</x:v>
+        <x:v>247</x:v>
       </x:c>
       <x:c r="B15" s="6" t="s">
-        <x:v>253</x:v>
+        <x:v>248</x:v>
       </x:c>
       <x:c r="C15" s="6" t="s">
-        <x:v>254</x:v>
+        <x:v>249</x:v>
       </x:c>
       <x:c r="D15" s="6" t="s">
-        <x:v>255</x:v>
+        <x:v>250</x:v>
       </x:c>
       <x:c r="E15" s="6" t="s">
-        <x:v>256</x:v>
+        <x:v>251</x:v>
       </x:c>
       <x:c r="F15" s="7" t="s">
-        <x:v>218</x:v>
+        <x:v>216</x:v>
       </x:c>
       <x:c r="G15" s="7" t="s">
-        <x:v>219</x:v>
+        <x:v>217</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="42" customHeight="1">
       <x:c r="A16" s="5" t="s">
-        <x:v>257</x:v>
+        <x:v>252</x:v>
       </x:c>
       <x:c r="B16" s="5" t="s">
-        <x:v>258</x:v>
+        <x:v>253</x:v>
       </x:c>
       <x:c r="C16" s="5" t="s">
-        <x:v>259</x:v>
+        <x:v>254</x:v>
       </x:c>
       <x:c r="D16" s="5" t="s">
-        <x:v>260</x:v>
+        <x:v>255</x:v>
       </x:c>
       <x:c r="E16" s="5" t="s">
-        <x:v>256</x:v>
+        <x:v>251</x:v>
       </x:c>
       <x:c r="F16" s="7" t="s">
-        <x:v>218</x:v>
+        <x:v>216</x:v>
       </x:c>
       <x:c r="G16" s="7" t="s">
-        <x:v>219</x:v>
+        <x:v>217</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="42" customHeight="1">
       <x:c r="A17" s="6" t="s">
-        <x:v>261</x:v>
+        <x:v>256</x:v>
       </x:c>
       <x:c r="B17" s="6" t="s">
-        <x:v>262</x:v>
+        <x:v>257</x:v>
       </x:c>
       <x:c r="C17" s="6" t="s">
-        <x:v>263</x:v>
+        <x:v>258</x:v>
       </x:c>
       <x:c r="D17" s="6" t="s">
-        <x:v>264</x:v>
+        <x:v>259</x:v>
       </x:c>
       <x:c r="E17" s="6" t="s">
-        <x:v>256</x:v>
+        <x:v>251</x:v>
       </x:c>
       <x:c r="F17" s="7" t="s">
-        <x:v>218</x:v>
+        <x:v>216</x:v>
       </x:c>
       <x:c r="G17" s="7" t="s">
-        <x:v>219</x:v>
+        <x:v>217</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="42" customHeight="1">
       <x:c r="A18" s="5" t="s">
-        <x:v>265</x:v>
+        <x:v>260</x:v>
       </x:c>
       <x:c r="B18" s="5" t="s">
-        <x:v>266</x:v>
+        <x:v>261</x:v>
       </x:c>
       <x:c r="C18" s="5" t="s">
-        <x:v>267</x:v>
+        <x:v>262</x:v>
       </x:c>
       <x:c r="D18" s="5" t="s">
-        <x:v>268</x:v>
+        <x:v>263</x:v>
       </x:c>
       <x:c r="E18" s="5" t="s">
-        <x:v>256</x:v>
+        <x:v>251</x:v>
       </x:c>
       <x:c r="F18" s="7" t="s">
-        <x:v>218</x:v>
+        <x:v>216</x:v>
       </x:c>
       <x:c r="G18" s="7" t="s">
-        <x:v>219</x:v>
+        <x:v>217</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="42" customHeight="1">
       <x:c r="A19" s="6" t="s">
-        <x:v>269</x:v>
+        <x:v>264</x:v>
       </x:c>
       <x:c r="B19" s="6" t="s">
-        <x:v>270</x:v>
+        <x:v>265</x:v>
       </x:c>
       <x:c r="C19" s="6" t="s">
-        <x:v>271</x:v>
+        <x:v>266</x:v>
       </x:c>
       <x:c r="D19" s="6" t="s">
-        <x:v>272</x:v>
+        <x:v>267</x:v>
       </x:c>
       <x:c r="E19" s="6" t="s">
-        <x:v>273</x:v>
+        <x:v>268</x:v>
       </x:c>
       <x:c r="F19" s="7" t="s">
-        <x:v>218</x:v>
+        <x:v>216</x:v>
       </x:c>
       <x:c r="G19" s="7" t="s">
-        <x:v>219</x:v>
+        <x:v>217</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="42" customHeight="1">
       <x:c r="A20" s="5" t="s">
-        <x:v>274</x:v>
+        <x:v>269</x:v>
       </x:c>
       <x:c r="B20" s="5" t="s">
-        <x:v>275</x:v>
+        <x:v>270</x:v>
       </x:c>
       <x:c r="C20" s="5" t="s">
-        <x:v>276</x:v>
+        <x:v>271</x:v>
       </x:c>
       <x:c r="D20" s="5" t="s">
-        <x:v>277</x:v>
+        <x:v>272</x:v>
       </x:c>
       <x:c r="E20" s="5" t="s">
-        <x:v>278</x:v>
+        <x:v>273</x:v>
       </x:c>
       <x:c r="F20" s="7" t="s">
-        <x:v>218</x:v>
+        <x:v>216</x:v>
       </x:c>
       <x:c r="G20" s="7" t="s">
-        <x:v>219</x:v>
+        <x:v>217</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="42" customHeight="1">
       <x:c r="A21" s="6" t="s">
-        <x:v>279</x:v>
+        <x:v>274</x:v>
       </x:c>
       <x:c r="B21" s="6" t="s">
-        <x:v>280</x:v>
+        <x:v>275</x:v>
       </x:c>
       <x:c r="C21" s="6" t="s">
-        <x:v>281</x:v>
+        <x:v>276</x:v>
       </x:c>
       <x:c r="D21" s="6" t="s">
-        <x:v>282</x:v>
+        <x:v>277</x:v>
       </x:c>
       <x:c r="E21" s="6" t="s">
-        <x:v>224</x:v>
+        <x:v>222</x:v>
       </x:c>
       <x:c r="F21" s="7" t="s">
-        <x:v>218</x:v>
+        <x:v>216</x:v>
       </x:c>
       <x:c r="G21" s="7" t="s">
-        <x:v>219</x:v>
+        <x:v>217</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="42" customHeight="1">
       <x:c r="A22" s="5" t="s">
-        <x:v>283</x:v>
+        <x:v>278</x:v>
       </x:c>
       <x:c r="B22" s="5" t="s">
-        <x:v>284</x:v>
+        <x:v>279</x:v>
       </x:c>
       <x:c r="C22" s="5" t="s">
-        <x:v>285</x:v>
+        <x:v>280</x:v>
       </x:c>
       <x:c r="D22" s="5" t="s">
-        <x:v>286</x:v>
+        <x:v>281</x:v>
       </x:c>
       <x:c r="E22" s="5" t="s">
-        <x:v>224</x:v>
+        <x:v>222</x:v>
       </x:c>
       <x:c r="F22" s="7" t="s">
-        <x:v>218</x:v>
+        <x:v>216</x:v>
       </x:c>
       <x:c r="G22" s="7" t="s">
-        <x:v>219</x:v>
+        <x:v>217</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="42" customHeight="1">
       <x:c r="A23" s="6" t="s">
-        <x:v>287</x:v>
+        <x:v>282</x:v>
       </x:c>
       <x:c r="B23" s="6" t="s">
-        <x:v>288</x:v>
+        <x:v>283</x:v>
       </x:c>
       <x:c r="C23" s="6" t="s">
-        <x:v>289</x:v>
+        <x:v>284</x:v>
       </x:c>
       <x:c r="D23" s="6" t="s">
-        <x:v>290</x:v>
+        <x:v>285</x:v>
       </x:c>
       <x:c r="E23" s="6" t="s">
+        <x:v>215</x:v>
+      </x:c>
+      <x:c r="F23" s="7" t="s">
+        <x:v>216</x:v>
+      </x:c>
+      <x:c r="G23" s="7" t="s">
         <x:v>217</x:v>
-      </x:c>
-      <x:c r="F23" s="7" t="s">
-        <x:v>218</x:v>
-      </x:c>
-      <x:c r="G23" s="7" t="s">
-        <x:v>219</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="42" customHeight="1">
       <x:c r="A24" s="5" t="s">
-        <x:v>291</x:v>
+        <x:v>286</x:v>
       </x:c>
       <x:c r="B24" s="5" t="s">
-        <x:v>292</x:v>
+        <x:v>287</x:v>
       </x:c>
       <x:c r="C24" s="5" t="s">
-        <x:v>293</x:v>
+        <x:v>288</x:v>
       </x:c>
       <x:c r="D24" s="5" t="s">
-        <x:v>294</x:v>
+        <x:v>289</x:v>
       </x:c>
       <x:c r="E24" s="5" t="s">
-        <x:v>295</x:v>
+        <x:v>290</x:v>
       </x:c>
       <x:c r="F24" s="7" t="s">
-        <x:v>218</x:v>
+        <x:v>216</x:v>
       </x:c>
       <x:c r="G24" s="7" t="s">
-        <x:v>219</x:v>
+        <x:v>217</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="42" customHeight="1">
       <x:c r="A25" s="6" t="s">
-        <x:v>296</x:v>
+        <x:v>291</x:v>
       </x:c>
       <x:c r="B25" s="6" t="s">
-        <x:v>297</x:v>
+        <x:v>292</x:v>
       </x:c>
       <x:c r="C25" s="6" t="s">
-        <x:v>298</x:v>
+        <x:v>293</x:v>
       </x:c>
       <x:c r="D25" s="6" t="s">
-        <x:v>299</x:v>
+        <x:v>294</x:v>
       </x:c>
       <x:c r="E25" s="6" t="s">
+        <x:v>215</x:v>
+      </x:c>
+      <x:c r="F25" s="7" t="s">
+        <x:v>216</x:v>
+      </x:c>
+      <x:c r="G25" s="7" t="s">
         <x:v>217</x:v>
-      </x:c>
-      <x:c r="F25" s="7" t="s">
-        <x:v>218</x:v>
-      </x:c>
-      <x:c r="G25" s="7" t="s">
-        <x:v>219</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="42" customHeight="1">
       <x:c r="A26" s="5" t="s">
-        <x:v>300</x:v>
+        <x:v>295</x:v>
       </x:c>
       <x:c r="B26" s="5" t="s">
-        <x:v>301</x:v>
+        <x:v>296</x:v>
       </x:c>
       <x:c r="C26" s="5" t="s">
-        <x:v>302</x:v>
+        <x:v>297</x:v>
       </x:c>
       <x:c r="D26" s="5" t="s">
-        <x:v>303</x:v>
+        <x:v>298</x:v>
       </x:c>
       <x:c r="E26" s="5" t="s">
-        <x:v>224</x:v>
+        <x:v>222</x:v>
       </x:c>
       <x:c r="F26" s="7" t="s">
-        <x:v>218</x:v>
+        <x:v>216</x:v>
       </x:c>
       <x:c r="G26" s="7" t="s">
-        <x:v>219</x:v>
+        <x:v>217</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="95" customHeight="1">
       <x:c r="A27" s="6" t="s">
-        <x:v>304</x:v>
+        <x:v>299</x:v>
       </x:c>
       <x:c r="B27" s="6" t="str">
         <x:v>dev验收及正式源码仓库、分支与授权确认完成</x:v>
@@ -4247,105 +4232,105 @@
         <x:v>迁移计划、DNS记录、演练与主站回归记录</x:v>
       </x:c>
       <x:c r="E27" s="6" t="s">
-        <x:v>305</x:v>
+        <x:v>300</x:v>
       </x:c>
       <x:c r="F27" s="7" t="s">
-        <x:v>218</x:v>
+        <x:v>216</x:v>
       </x:c>
       <x:c r="G27" s="7" t="s">
-        <x:v>219</x:v>
+        <x:v>217</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="42" customHeight="1">
       <x:c r="A28" s="5" t="s">
-        <x:v>306</x:v>
+        <x:v>301</x:v>
       </x:c>
       <x:c r="B28" s="5" t="s">
-        <x:v>307</x:v>
+        <x:v>302</x:v>
       </x:c>
       <x:c r="C28" s="5" t="s">
-        <x:v>308</x:v>
+        <x:v>303</x:v>
       </x:c>
       <x:c r="D28" s="5" t="s">
-        <x:v>309</x:v>
+        <x:v>304</x:v>
       </x:c>
       <x:c r="E28" s="5" t="s">
-        <x:v>310</x:v>
+        <x:v>305</x:v>
       </x:c>
       <x:c r="F28" s="7" t="s">
-        <x:v>218</x:v>
+        <x:v>216</x:v>
       </x:c>
       <x:c r="G28" s="7" t="s">
-        <x:v>219</x:v>
+        <x:v>217</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="42" customHeight="1">
       <x:c r="A29" s="6" t="s">
-        <x:v>311</x:v>
+        <x:v>306</x:v>
       </x:c>
       <x:c r="B29" s="6" t="s">
-        <x:v>312</x:v>
+        <x:v>307</x:v>
       </x:c>
       <x:c r="C29" s="6" t="s">
-        <x:v>313</x:v>
+        <x:v>308</x:v>
       </x:c>
       <x:c r="D29" s="6" t="s">
-        <x:v>314</x:v>
+        <x:v>309</x:v>
       </x:c>
       <x:c r="E29" s="6" t="s">
-        <x:v>315</x:v>
+        <x:v>310</x:v>
       </x:c>
       <x:c r="F29" s="7" t="s">
-        <x:v>218</x:v>
+        <x:v>216</x:v>
       </x:c>
       <x:c r="G29" s="7" t="s">
-        <x:v>219</x:v>
+        <x:v>217</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="42" customHeight="1">
       <x:c r="A30" s="5" t="s">
-        <x:v>316</x:v>
+        <x:v>311</x:v>
       </x:c>
       <x:c r="B30" s="5" t="s">
-        <x:v>317</x:v>
+        <x:v>312</x:v>
       </x:c>
       <x:c r="C30" s="5" t="s">
-        <x:v>318</x:v>
+        <x:v>313</x:v>
       </x:c>
       <x:c r="D30" s="5" t="s">
-        <x:v>319</x:v>
+        <x:v>314</x:v>
       </x:c>
       <x:c r="E30" s="5" t="s">
-        <x:v>320</x:v>
+        <x:v>315</x:v>
       </x:c>
       <x:c r="F30" s="7" t="s">
-        <x:v>218</x:v>
+        <x:v>216</x:v>
       </x:c>
       <x:c r="G30" s="7" t="s">
-        <x:v>219</x:v>
+        <x:v>217</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="42" customHeight="1">
       <x:c r="A31" s="6" t="s">
-        <x:v>321</x:v>
+        <x:v>316</x:v>
       </x:c>
       <x:c r="B31" s="6" t="s">
-        <x:v>322</x:v>
+        <x:v>317</x:v>
       </x:c>
       <x:c r="C31" s="6" t="s">
-        <x:v>323</x:v>
+        <x:v>318</x:v>
       </x:c>
       <x:c r="D31" s="6" t="s">
-        <x:v>324</x:v>
+        <x:v>319</x:v>
       </x:c>
       <x:c r="E31" s="6" t="s">
-        <x:v>273</x:v>
+        <x:v>268</x:v>
       </x:c>
       <x:c r="F31" s="7" t="s">
-        <x:v>218</x:v>
+        <x:v>216</x:v>
       </x:c>
       <x:c r="G31" s="7" t="s">
-        <x:v>219</x:v>
+        <x:v>217</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -4356,7 +4341,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2d67f2d6acb2410e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R77cfc0fe72e34fb8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4389,7 +4374,7 @@
     </x:row>
     <x:row r="2" ht="21">
       <x:c r="A2" s="2" t="s">
-        <x:v>325</x:v>
+        <x:v>320</x:v>
       </x:c>
       <x:c r="B2" s="1"/>
       <x:c r="C2" s="1"/>
@@ -4402,7 +4387,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="3" t="s">
-        <x:v>326</x:v>
+        <x:v>321</x:v>
       </x:c>
       <x:c r="B3" s="1"/>
       <x:c r="C3" s="1"/>
@@ -4426,54 +4411,54 @@
     </x:row>
     <x:row r="5" ht="37.95000076293945" customHeight="1">
       <x:c r="A5" s="4" t="s">
+        <x:v>322</x:v>
+      </x:c>
+      <x:c r="B5" s="4" t="s">
+        <x:v>323</x:v>
+      </x:c>
+      <x:c r="C5" s="4" t="s">
+        <x:v>324</x:v>
+      </x:c>
+      <x:c r="D5" s="4" t="s">
+        <x:v>325</x:v>
+      </x:c>
+      <x:c r="E5" s="4" t="s">
+        <x:v>326</x:v>
+      </x:c>
+      <x:c r="F5" s="4" t="s">
         <x:v>327</x:v>
       </x:c>
-      <x:c r="B5" s="4" t="s">
+      <x:c r="G5" s="4" t="s">
         <x:v>328</x:v>
       </x:c>
-      <x:c r="C5" s="4" t="s">
+      <x:c r="H5" s="4" t="s">
         <x:v>329</x:v>
       </x:c>
-      <x:c r="D5" s="4" t="s">
+      <x:c r="I5" s="4" t="s">
         <x:v>330</x:v>
-      </x:c>
-      <x:c r="E5" s="4" t="s">
-        <x:v>331</x:v>
-      </x:c>
-      <x:c r="F5" s="4" t="s">
-        <x:v>332</x:v>
-      </x:c>
-      <x:c r="G5" s="4" t="s">
-        <x:v>333</x:v>
-      </x:c>
-      <x:c r="H5" s="4" t="s">
-        <x:v>334</x:v>
-      </x:c>
-      <x:c r="I5" s="4" t="s">
-        <x:v>335</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="85" customHeight="1">
       <x:c r="A6" s="5" t="s">
-        <x:v>124</x:v>
+        <x:v>123</x:v>
       </x:c>
       <x:c r="B6" s="5" t="s">
+        <x:v>331</x:v>
+      </x:c>
+      <x:c r="C6" s="5" t="s">
+        <x:v>332</x:v>
+      </x:c>
+      <x:c r="D6" s="5" t="s">
+        <x:v>333</x:v>
+      </x:c>
+      <x:c r="E6" s="5" t="s">
+        <x:v>334</x:v>
+      </x:c>
+      <x:c r="F6" s="5" t="s">
+        <x:v>335</x:v>
+      </x:c>
+      <x:c r="G6" s="5" t="s">
         <x:v>336</x:v>
-      </x:c>
-      <x:c r="C6" s="5" t="s">
-        <x:v>337</x:v>
-      </x:c>
-      <x:c r="D6" s="5" t="s">
-        <x:v>338</x:v>
-      </x:c>
-      <x:c r="E6" s="5" t="s">
-        <x:v>339</x:v>
-      </x:c>
-      <x:c r="F6" s="5" t="s">
-        <x:v>340</x:v>
-      </x:c>
-      <x:c r="G6" s="5" t="s">
-        <x:v>341</x:v>
       </x:c>
       <x:c r="H6" s="7" t="s">
         <x:v>31</x:v>
@@ -4484,25 +4469,25 @@
     </x:row>
     <x:row r="7" ht="110" customHeight="1">
       <x:c r="A7" s="6" t="s">
-        <x:v>129</x:v>
+        <x:v>128</x:v>
       </x:c>
       <x:c r="B7" s="6" t="s">
-        <x:v>342</x:v>
+        <x:v>337</x:v>
       </x:c>
       <x:c r="C7" s="6" t="str">
         <x:v>路径与域名已定；待确认权威DNS管理方、解析与变更权限、主站保留及切换回退方式。</x:v>
       </x:c>
       <x:c r="D7" s="6" t="s">
-        <x:v>343</x:v>
+        <x:v>338</x:v>
       </x:c>
       <x:c r="E7" s="6" t="s">
-        <x:v>344</x:v>
+        <x:v>339</x:v>
       </x:c>
       <x:c r="F7" s="6" t="s">
-        <x:v>340</x:v>
+        <x:v>335</x:v>
       </x:c>
       <x:c r="G7" s="6" t="s">
-        <x:v>341</x:v>
+        <x:v>336</x:v>
       </x:c>
       <x:c r="H7" s="7" t="s">
         <x:v>31</x:v>
@@ -4513,25 +4498,25 @@
     </x:row>
     <x:row r="8" ht="42" customHeight="1">
       <x:c r="A8" s="5" t="s">
-        <x:v>133</x:v>
+        <x:v>132</x:v>
       </x:c>
       <x:c r="B8" s="5" t="s">
-        <x:v>345</x:v>
+        <x:v>340</x:v>
       </x:c>
       <x:c r="C8" s="5" t="s">
-        <x:v>346</x:v>
+        <x:v>341</x:v>
       </x:c>
       <x:c r="D8" s="5" t="s">
-        <x:v>347</x:v>
+        <x:v>342</x:v>
       </x:c>
       <x:c r="E8" s="5" t="s">
-        <x:v>348</x:v>
+        <x:v>343</x:v>
       </x:c>
       <x:c r="F8" s="5" t="s">
-        <x:v>340</x:v>
+        <x:v>335</x:v>
       </x:c>
       <x:c r="G8" s="5" t="s">
-        <x:v>349</x:v>
+        <x:v>344</x:v>
       </x:c>
       <x:c r="H8" s="7" t="s">
         <x:v>31</x:v>
@@ -4540,22 +4525,22 @@
     </x:row>
     <x:row r="9" ht="110" customHeight="1">
       <x:c r="A9" s="6" t="s">
-        <x:v>147</x:v>
+        <x:v>146</x:v>
       </x:c>
       <x:c r="B9" s="6" t="s">
-        <x:v>350</x:v>
+        <x:v>345</x:v>
       </x:c>
       <x:c r="C9" s="6" t="str">
         <x:v>在dev部署练习中比较并固定Node/npm及依赖版本，实际构建后验证产物再部署。</x:v>
       </x:c>
       <x:c r="D9" s="6" t="s">
-        <x:v>351</x:v>
+        <x:v>346</x:v>
       </x:c>
       <x:c r="E9" s="6" t="s">
-        <x:v>352</x:v>
+        <x:v>347</x:v>
       </x:c>
       <x:c r="F9" s="6" t="s">
-        <x:v>353</x:v>
+        <x:v>348</x:v>
       </x:c>
       <x:c r="G9" s="6" t="str">
         <x:v>dev部署练习中，部署前</x:v>
@@ -4569,19 +4554,19 @@
     </x:row>
     <x:row r="10" ht="110" customHeight="1">
       <x:c r="A10" s="5" t="s">
-        <x:v>156</x:v>
+        <x:v>154</x:v>
       </x:c>
       <x:c r="B10" s="5" t="s">
-        <x:v>354</x:v>
+        <x:v>349</x:v>
       </x:c>
       <x:c r="C10" s="5" t="str">
         <x:v>dev用用户私有副本，正式用开发者私有原仓库；分别确认来源、触发分支、连接授权、发布与失败处理。</x:v>
       </x:c>
       <x:c r="D10" s="5" t="s">
-        <x:v>355</x:v>
+        <x:v>350</x:v>
       </x:c>
       <x:c r="E10" s="5" t="s">
-        <x:v>356</x:v>
+        <x:v>351</x:v>
       </x:c>
       <x:c r="F10" s="5" t="str">
         <x:v>用户与原开发者／待确认</x:v>
@@ -4598,25 +4583,25 @@
     </x:row>
     <x:row r="11" ht="42" customHeight="1">
       <x:c r="A11" s="6" t="s">
-        <x:v>176</x:v>
+        <x:v>174</x:v>
       </x:c>
       <x:c r="B11" s="6" t="s">
-        <x:v>357</x:v>
+        <x:v>352</x:v>
       </x:c>
       <x:c r="C11" s="6" t="s">
-        <x:v>358</x:v>
+        <x:v>353</x:v>
       </x:c>
       <x:c r="D11" s="6" t="s">
-        <x:v>359</x:v>
+        <x:v>354</x:v>
       </x:c>
       <x:c r="E11" s="6" t="s">
-        <x:v>173</x:v>
+        <x:v>171</x:v>
       </x:c>
       <x:c r="F11" s="6" t="s">
-        <x:v>340</x:v>
+        <x:v>335</x:v>
       </x:c>
       <x:c r="G11" s="6" t="s">
-        <x:v>349</x:v>
+        <x:v>344</x:v>
       </x:c>
       <x:c r="H11" s="7" t="s">
         <x:v>31</x:v>
@@ -4625,25 +4610,25 @@
     </x:row>
     <x:row r="12" ht="42" customHeight="1">
       <x:c r="A12" s="5" t="s">
-        <x:v>180</x:v>
+        <x:v>178</x:v>
       </x:c>
       <x:c r="B12" s="5" t="s">
-        <x:v>360</x:v>
+        <x:v>355</x:v>
       </x:c>
       <x:c r="C12" s="5" t="s">
-        <x:v>361</x:v>
+        <x:v>356</x:v>
       </x:c>
       <x:c r="D12" s="5" t="s">
-        <x:v>362</x:v>
+        <x:v>357</x:v>
       </x:c>
       <x:c r="E12" s="5" t="s">
-        <x:v>363</x:v>
+        <x:v>358</x:v>
       </x:c>
       <x:c r="F12" s="5" t="s">
-        <x:v>340</x:v>
+        <x:v>335</x:v>
       </x:c>
       <x:c r="G12" s="5" t="s">
-        <x:v>364</x:v>
+        <x:v>359</x:v>
       </x:c>
       <x:c r="H12" s="7" t="s">
         <x:v>31</x:v>
@@ -4652,25 +4637,25 @@
     </x:row>
     <x:row r="13" ht="42" customHeight="1">
       <x:c r="A13" s="6" t="s">
-        <x:v>365</x:v>
+        <x:v>360</x:v>
       </x:c>
       <x:c r="B13" s="6" t="s">
-        <x:v>366</x:v>
+        <x:v>361</x:v>
       </x:c>
       <x:c r="C13" s="6" t="s">
-        <x:v>367</x:v>
+        <x:v>362</x:v>
       </x:c>
       <x:c r="D13" s="6" t="s">
-        <x:v>368</x:v>
+        <x:v>363</x:v>
       </x:c>
       <x:c r="E13" s="6" t="s">
-        <x:v>369</x:v>
+        <x:v>364</x:v>
       </x:c>
       <x:c r="F13" s="6" t="s">
-        <x:v>340</x:v>
+        <x:v>335</x:v>
       </x:c>
       <x:c r="G13" s="6" t="s">
-        <x:v>341</x:v>
+        <x:v>336</x:v>
       </x:c>
       <x:c r="H13" s="7" t="s">
         <x:v>31</x:v>
@@ -4679,25 +4664,25 @@
     </x:row>
     <x:row r="14" ht="42" customHeight="1">
       <x:c r="A14" s="5" t="s">
-        <x:v>161</x:v>
+        <x:v>159</x:v>
       </x:c>
       <x:c r="B14" s="5" t="s">
-        <x:v>182</x:v>
+        <x:v>180</x:v>
       </x:c>
       <x:c r="C14" s="5" t="s">
-        <x:v>370</x:v>
+        <x:v>365</x:v>
       </x:c>
       <x:c r="D14" s="5" t="s">
-        <x:v>371</x:v>
+        <x:v>366</x:v>
       </x:c>
       <x:c r="E14" s="5" t="s">
-        <x:v>372</x:v>
+        <x:v>367</x:v>
       </x:c>
       <x:c r="F14" s="5" t="s">
-        <x:v>340</x:v>
+        <x:v>335</x:v>
       </x:c>
       <x:c r="G14" s="5" t="s">
-        <x:v>341</x:v>
+        <x:v>336</x:v>
       </x:c>
       <x:c r="H14" s="7" t="s">
         <x:v>31</x:v>
@@ -4706,25 +4691,25 @@
     </x:row>
     <x:row r="15" ht="110" customHeight="1">
       <x:c r="A15" s="6" t="s">
-        <x:v>373</x:v>
+        <x:v>368</x:v>
       </x:c>
       <x:c r="B15" s="6" t="s">
-        <x:v>374</x:v>
+        <x:v>369</x:v>
       </x:c>
       <x:c r="C15" s="6" t="str">
         <x:v>依赖已说明；待核验原站路由／响应头、完整网络请求及切换批准与窗口。</x:v>
       </x:c>
       <x:c r="D15" s="6" t="s">
-        <x:v>375</x:v>
+        <x:v>370</x:v>
       </x:c>
       <x:c r="E15" s="6" t="s">
-        <x:v>376</x:v>
+        <x:v>371</x:v>
       </x:c>
       <x:c r="F15" s="6" t="s">
-        <x:v>377</x:v>
+        <x:v>372</x:v>
       </x:c>
       <x:c r="G15" s="6" t="s">
-        <x:v>378</x:v>
+        <x:v>373</x:v>
       </x:c>
       <x:c r="H15" s="7" t="s">
         <x:v>31</x:v>
@@ -4735,25 +4720,25 @@
     </x:row>
     <x:row r="16" ht="42" customHeight="1">
       <x:c r="A16" s="5" t="s">
-        <x:v>203</x:v>
+        <x:v>201</x:v>
       </x:c>
       <x:c r="B16" s="5" t="s">
-        <x:v>379</x:v>
+        <x:v>374</x:v>
       </x:c>
       <x:c r="C16" s="5" t="s">
-        <x:v>380</x:v>
+        <x:v>375</x:v>
       </x:c>
       <x:c r="D16" s="5" t="s">
-        <x:v>381</x:v>
+        <x:v>376</x:v>
       </x:c>
       <x:c r="E16" s="5" t="s">
-        <x:v>200</x:v>
+        <x:v>198</x:v>
       </x:c>
       <x:c r="F16" s="5" t="s">
-        <x:v>340</x:v>
+        <x:v>335</x:v>
       </x:c>
       <x:c r="G16" s="5" t="s">
-        <x:v>349</x:v>
+        <x:v>344</x:v>
       </x:c>
       <x:c r="H16" s="7" t="s">
         <x:v>31</x:v>
@@ -4768,7 +4753,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R349efe13f3c347f9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdddbc3dd8db8460b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4799,7 +4784,7 @@
     </x:row>
     <x:row r="2" ht="21">
       <x:c r="A2" s="2" t="s">
-        <x:v>382</x:v>
+        <x:v>377</x:v>
       </x:c>
       <x:c r="B2" s="1"/>
       <x:c r="C2" s="1"/>
@@ -4811,7 +4796,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="3" t="s">
-        <x:v>383</x:v>
+        <x:v>378</x:v>
       </x:c>
       <x:c r="B3" s="1"/>
       <x:c r="C3" s="1"/>
@@ -4833,236 +4818,236 @@
     </x:row>
     <x:row r="5" ht="37.95000076293945" customHeight="1">
       <x:c r="A5" s="4" t="s">
+        <x:v>379</x:v>
+      </x:c>
+      <x:c r="B5" s="4" t="s">
+        <x:v>380</x:v>
+      </x:c>
+      <x:c r="C5" s="4" t="s">
+        <x:v>381</x:v>
+      </x:c>
+      <x:c r="D5" s="4" t="s">
+        <x:v>382</x:v>
+      </x:c>
+      <x:c r="E5" s="4" t="s">
+        <x:v>383</x:v>
+      </x:c>
+      <x:c r="F5" s="4" t="s">
         <x:v>384</x:v>
       </x:c>
-      <x:c r="B5" s="4" t="s">
+      <x:c r="G5" s="4" t="s">
         <x:v>385</x:v>
       </x:c>
-      <x:c r="C5" s="4" t="s">
-        <x:v>386</x:v>
-      </x:c>
-      <x:c r="D5" s="4" t="s">
-        <x:v>387</x:v>
-      </x:c>
-      <x:c r="E5" s="4" t="s">
-        <x:v>388</x:v>
-      </x:c>
-      <x:c r="F5" s="4" t="s">
-        <x:v>389</x:v>
-      </x:c>
-      <x:c r="G5" s="4" t="s">
-        <x:v>390</x:v>
-      </x:c>
       <x:c r="H5" s="4" t="s">
-        <x:v>117</x:v>
+        <x:v>116</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="42" customHeight="1">
       <x:c r="A6" s="5" t="s">
+        <x:v>386</x:v>
+      </x:c>
+      <x:c r="B6" s="5" t="s">
+        <x:v>387</x:v>
+      </x:c>
+      <x:c r="C6" s="5" t="s">
+        <x:v>388</x:v>
+      </x:c>
+      <x:c r="D6" s="5" t="s">
+        <x:v>389</x:v>
+      </x:c>
+      <x:c r="E6" s="5" t="s">
+        <x:v>390</x:v>
+      </x:c>
+      <x:c r="F6" s="5" t="s">
         <x:v>391</x:v>
       </x:c>
-      <x:c r="B6" s="5" t="s">
+      <x:c r="G6" s="5" t="s">
         <x:v>392</x:v>
       </x:c>
-      <x:c r="C6" s="5" t="s">
+      <x:c r="H6" s="7" t="s">
         <x:v>393</x:v>
-      </x:c>
-      <x:c r="D6" s="5" t="s">
-        <x:v>394</x:v>
-      </x:c>
-      <x:c r="E6" s="5" t="s">
-        <x:v>395</x:v>
-      </x:c>
-      <x:c r="F6" s="5" t="s">
-        <x:v>396</x:v>
-      </x:c>
-      <x:c r="G6" s="5" t="s">
-        <x:v>397</x:v>
-      </x:c>
-      <x:c r="H6" s="7" t="s">
-        <x:v>398</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="42" customHeight="1">
       <x:c r="A7" s="6" t="s">
+        <x:v>394</x:v>
+      </x:c>
+      <x:c r="B7" s="6" t="s">
+        <x:v>395</x:v>
+      </x:c>
+      <x:c r="C7" s="6" t="s">
+        <x:v>396</x:v>
+      </x:c>
+      <x:c r="D7" s="6" t="s">
+        <x:v>397</x:v>
+      </x:c>
+      <x:c r="E7" s="6" t="s">
+        <x:v>398</x:v>
+      </x:c>
+      <x:c r="F7" s="6" t="s">
         <x:v>399</x:v>
       </x:c>
-      <x:c r="B7" s="6" t="s">
+      <x:c r="G7" s="6" t="s">
         <x:v>400</x:v>
       </x:c>
-      <x:c r="C7" s="6" t="s">
-        <x:v>401</x:v>
-      </x:c>
-      <x:c r="D7" s="6" t="s">
-        <x:v>402</x:v>
-      </x:c>
-      <x:c r="E7" s="6" t="s">
-        <x:v>403</x:v>
-      </x:c>
-      <x:c r="F7" s="6" t="s">
-        <x:v>404</x:v>
-      </x:c>
-      <x:c r="G7" s="6" t="s">
-        <x:v>405</x:v>
-      </x:c>
       <x:c r="H7" s="7" t="s">
-        <x:v>398</x:v>
+        <x:v>393</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="42" customHeight="1">
       <x:c r="A8" s="5" t="s">
+        <x:v>401</x:v>
+      </x:c>
+      <x:c r="B8" s="5" t="s">
+        <x:v>402</x:v>
+      </x:c>
+      <x:c r="C8" s="5" t="s">
+        <x:v>403</x:v>
+      </x:c>
+      <x:c r="D8" s="5" t="s">
+        <x:v>404</x:v>
+      </x:c>
+      <x:c r="E8" s="5" t="s">
+        <x:v>405</x:v>
+      </x:c>
+      <x:c r="F8" s="5" t="s">
         <x:v>406</x:v>
       </x:c>
-      <x:c r="B8" s="5" t="s">
+      <x:c r="G8" s="5" t="s">
         <x:v>407</x:v>
       </x:c>
-      <x:c r="C8" s="5" t="s">
+      <x:c r="H8" s="7" t="s">
         <x:v>408</x:v>
-      </x:c>
-      <x:c r="D8" s="5" t="s">
-        <x:v>409</x:v>
-      </x:c>
-      <x:c r="E8" s="5" t="s">
-        <x:v>410</x:v>
-      </x:c>
-      <x:c r="F8" s="5" t="s">
-        <x:v>411</x:v>
-      </x:c>
-      <x:c r="G8" s="5" t="s">
-        <x:v>412</x:v>
-      </x:c>
-      <x:c r="H8" s="7" t="s">
-        <x:v>413</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="42" customHeight="1">
       <x:c r="A9" s="6" t="s">
+        <x:v>409</x:v>
+      </x:c>
+      <x:c r="B9" s="6" t="s">
+        <x:v>410</x:v>
+      </x:c>
+      <x:c r="C9" s="6" t="s">
+        <x:v>411</x:v>
+      </x:c>
+      <x:c r="D9" s="6" t="s">
+        <x:v>402</x:v>
+      </x:c>
+      <x:c r="E9" s="6" t="s">
+        <x:v>412</x:v>
+      </x:c>
+      <x:c r="F9" s="6" t="s">
+        <x:v>413</x:v>
+      </x:c>
+      <x:c r="G9" s="6" t="s">
         <x:v>414</x:v>
       </x:c>
-      <x:c r="B9" s="6" t="s">
-        <x:v>415</x:v>
-      </x:c>
-      <x:c r="C9" s="6" t="s">
-        <x:v>416</x:v>
-      </x:c>
-      <x:c r="D9" s="6" t="s">
-        <x:v>407</x:v>
-      </x:c>
-      <x:c r="E9" s="6" t="s">
-        <x:v>417</x:v>
-      </x:c>
-      <x:c r="F9" s="6" t="s">
-        <x:v>418</x:v>
-      </x:c>
-      <x:c r="G9" s="6" t="s">
-        <x:v>419</x:v>
-      </x:c>
       <x:c r="H9" s="7" t="s">
-        <x:v>413</x:v>
+        <x:v>408</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="42" customHeight="1">
       <x:c r="A10" s="5" t="s">
+        <x:v>415</x:v>
+      </x:c>
+      <x:c r="B10" s="5" t="s">
+        <x:v>143</x:v>
+      </x:c>
+      <x:c r="C10" s="5" t="s">
+        <x:v>416</x:v>
+      </x:c>
+      <x:c r="D10" s="5" t="s">
+        <x:v>417</x:v>
+      </x:c>
+      <x:c r="E10" s="5" t="s">
+        <x:v>418</x:v>
+      </x:c>
+      <x:c r="F10" s="5" t="s">
+        <x:v>419</x:v>
+      </x:c>
+      <x:c r="G10" s="5" t="s">
         <x:v>420</x:v>
       </x:c>
-      <x:c r="B10" s="5" t="s">
-        <x:v>144</x:v>
-      </x:c>
-      <x:c r="C10" s="5" t="s">
-        <x:v>421</x:v>
-      </x:c>
-      <x:c r="D10" s="5" t="s">
-        <x:v>422</x:v>
-      </x:c>
-      <x:c r="E10" s="5" t="s">
-        <x:v>423</x:v>
-      </x:c>
-      <x:c r="F10" s="5" t="s">
-        <x:v>424</x:v>
-      </x:c>
-      <x:c r="G10" s="5" t="s">
-        <x:v>425</x:v>
-      </x:c>
       <x:c r="H10" s="7" t="s">
-        <x:v>413</x:v>
+        <x:v>408</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="42" customHeight="1">
       <x:c r="A11" s="6" t="s">
+        <x:v>421</x:v>
+      </x:c>
+      <x:c r="B11" s="6" t="s">
+        <x:v>422</x:v>
+      </x:c>
+      <x:c r="C11" s="6" t="s">
+        <x:v>423</x:v>
+      </x:c>
+      <x:c r="D11" s="6" t="s">
+        <x:v>424</x:v>
+      </x:c>
+      <x:c r="E11" s="6" t="s">
+        <x:v>425</x:v>
+      </x:c>
+      <x:c r="F11" s="6" t="s">
         <x:v>426</x:v>
       </x:c>
-      <x:c r="B11" s="6" t="s">
+      <x:c r="G11" s="6" t="s">
         <x:v>427</x:v>
       </x:c>
-      <x:c r="C11" s="6" t="s">
-        <x:v>428</x:v>
-      </x:c>
-      <x:c r="D11" s="6" t="s">
-        <x:v>429</x:v>
-      </x:c>
-      <x:c r="E11" s="6" t="s">
-        <x:v>430</x:v>
-      </x:c>
-      <x:c r="F11" s="6" t="s">
-        <x:v>431</x:v>
-      </x:c>
-      <x:c r="G11" s="6" t="s">
-        <x:v>432</x:v>
-      </x:c>
       <x:c r="H11" s="7" t="s">
-        <x:v>413</x:v>
+        <x:v>408</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="42" customHeight="1">
       <x:c r="A12" s="5" t="s">
+        <x:v>428</x:v>
+      </x:c>
+      <x:c r="B12" s="5" t="s">
+        <x:v>429</x:v>
+      </x:c>
+      <x:c r="C12" s="5" t="s">
+        <x:v>430</x:v>
+      </x:c>
+      <x:c r="D12" s="5" t="s">
+        <x:v>431</x:v>
+      </x:c>
+      <x:c r="E12" s="5" t="s">
+        <x:v>432</x:v>
+      </x:c>
+      <x:c r="F12" s="5" t="s">
         <x:v>433</x:v>
       </x:c>
-      <x:c r="B12" s="5" t="s">
+      <x:c r="G12" s="5" t="s">
         <x:v>434</x:v>
       </x:c>
-      <x:c r="C12" s="5" t="s">
-        <x:v>435</x:v>
-      </x:c>
-      <x:c r="D12" s="5" t="s">
-        <x:v>436</x:v>
-      </x:c>
-      <x:c r="E12" s="5" t="s">
-        <x:v>437</x:v>
-      </x:c>
-      <x:c r="F12" s="5" t="s">
-        <x:v>438</x:v>
-      </x:c>
-      <x:c r="G12" s="5" t="s">
-        <x:v>439</x:v>
-      </x:c>
       <x:c r="H12" s="7" t="s">
-        <x:v>413</x:v>
+        <x:v>408</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="42" customHeight="1">
       <x:c r="A13" s="6" t="s">
+        <x:v>435</x:v>
+      </x:c>
+      <x:c r="B13" s="6" t="s">
+        <x:v>436</x:v>
+      </x:c>
+      <x:c r="C13" s="6" t="s">
+        <x:v>437</x:v>
+      </x:c>
+      <x:c r="D13" s="6" t="s">
+        <x:v>438</x:v>
+      </x:c>
+      <x:c r="E13" s="6" t="s">
+        <x:v>439</x:v>
+      </x:c>
+      <x:c r="F13" s="6" t="s">
         <x:v>440</x:v>
       </x:c>
-      <x:c r="B13" s="6" t="s">
+      <x:c r="G13" s="6" t="s">
         <x:v>441</x:v>
       </x:c>
-      <x:c r="C13" s="6" t="s">
-        <x:v>442</x:v>
-      </x:c>
-      <x:c r="D13" s="6" t="s">
-        <x:v>443</x:v>
-      </x:c>
-      <x:c r="E13" s="6" t="s">
-        <x:v>444</x:v>
-      </x:c>
-      <x:c r="F13" s="6" t="s">
-        <x:v>445</x:v>
-      </x:c>
-      <x:c r="G13" s="6" t="s">
-        <x:v>446</x:v>
-      </x:c>
       <x:c r="H13" s="7" t="s">
-        <x:v>413</x:v>
+        <x:v>408</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -5073,7 +5058,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4dcde4b134f24917"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1c25241aa4284f6d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5102,7 +5087,7 @@
     </x:row>
     <x:row r="2" ht="21">
       <x:c r="A2" s="2" t="s">
-        <x:v>447</x:v>
+        <x:v>442</x:v>
       </x:c>
       <x:c r="B2" s="1"/>
       <x:c r="C2" s="1"/>
@@ -5113,7 +5098,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="3" t="s">
-        <x:v>448</x:v>
+        <x:v>443</x:v>
       </x:c>
       <x:c r="B3" s="1"/>
       <x:c r="C3" s="1"/>
@@ -5133,1181 +5118,1181 @@
     </x:row>
     <x:row r="5" ht="37.95000076293945" customHeight="1">
       <x:c r="A5" s="4" t="s">
+        <x:v>444</x:v>
+      </x:c>
+      <x:c r="B5" s="4" t="s">
+        <x:v>445</x:v>
+      </x:c>
+      <x:c r="C5" s="4" t="s">
+        <x:v>446</x:v>
+      </x:c>
+      <x:c r="D5" s="4" t="s">
+        <x:v>447</x:v>
+      </x:c>
+      <x:c r="E5" s="4" t="s">
+        <x:v>448</x:v>
+      </x:c>
+      <x:c r="F5" s="4" t="s">
+        <x:v>326</x:v>
+      </x:c>
+      <x:c r="G5" s="4" t="s">
         <x:v>449</x:v>
-      </x:c>
-      <x:c r="B5" s="4" t="s">
-        <x:v>450</x:v>
-      </x:c>
-      <x:c r="C5" s="4" t="s">
-        <x:v>451</x:v>
-      </x:c>
-      <x:c r="D5" s="4" t="s">
-        <x:v>452</x:v>
-      </x:c>
-      <x:c r="E5" s="4" t="s">
-        <x:v>453</x:v>
-      </x:c>
-      <x:c r="F5" s="4" t="s">
-        <x:v>331</x:v>
-      </x:c>
-      <x:c r="G5" s="4" t="s">
-        <x:v>454</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="42" customHeight="1">
       <x:c r="A6" s="5" t="s">
+        <x:v>450</x:v>
+      </x:c>
+      <x:c r="B6" s="5" t="s">
+        <x:v>451</x:v>
+      </x:c>
+      <x:c r="C6" s="5" t="s">
+        <x:v>452</x:v>
+      </x:c>
+      <x:c r="D6" s="5" t="s">
+        <x:v>453</x:v>
+      </x:c>
+      <x:c r="E6" s="5" t="s">
+        <x:v>454</x:v>
+      </x:c>
+      <x:c r="F6" s="5" t="s">
         <x:v>455</x:v>
       </x:c>
-      <x:c r="B6" s="5" t="s">
+      <x:c r="G6" s="7" t="s">
         <x:v>456</x:v>
-      </x:c>
-      <x:c r="C6" s="5" t="s">
-        <x:v>457</x:v>
-      </x:c>
-      <x:c r="D6" s="5" t="s">
-        <x:v>458</x:v>
-      </x:c>
-      <x:c r="E6" s="5" t="s">
-        <x:v>459</x:v>
-      </x:c>
-      <x:c r="F6" s="5" t="s">
-        <x:v>460</x:v>
-      </x:c>
-      <x:c r="G6" s="7" t="s">
-        <x:v>461</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="42" customHeight="1">
       <x:c r="A7" s="6" t="s">
-        <x:v>462</x:v>
+        <x:v>457</x:v>
       </x:c>
       <x:c r="B7" s="6" t="s">
+        <x:v>451</x:v>
+      </x:c>
+      <x:c r="C7" s="6" t="s">
+        <x:v>458</x:v>
+      </x:c>
+      <x:c r="D7" s="6" t="s">
+        <x:v>459</x:v>
+      </x:c>
+      <x:c r="E7" s="6" t="s">
+        <x:v>454</x:v>
+      </x:c>
+      <x:c r="F7" s="6" t="s">
+        <x:v>455</x:v>
+      </x:c>
+      <x:c r="G7" s="7" t="s">
         <x:v>456</x:v>
-      </x:c>
-      <x:c r="C7" s="6" t="s">
-        <x:v>463</x:v>
-      </x:c>
-      <x:c r="D7" s="6" t="s">
-        <x:v>464</x:v>
-      </x:c>
-      <x:c r="E7" s="6" t="s">
-        <x:v>459</x:v>
-      </x:c>
-      <x:c r="F7" s="6" t="s">
-        <x:v>460</x:v>
-      </x:c>
-      <x:c r="G7" s="7" t="s">
-        <x:v>461</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="42" customHeight="1">
       <x:c r="A8" s="5" t="s">
-        <x:v>465</x:v>
+        <x:v>460</x:v>
       </x:c>
       <x:c r="B8" s="5" t="s">
+        <x:v>451</x:v>
+      </x:c>
+      <x:c r="C8" s="5" t="s">
+        <x:v>461</x:v>
+      </x:c>
+      <x:c r="D8" s="5" t="s">
+        <x:v>453</x:v>
+      </x:c>
+      <x:c r="E8" s="5" t="s">
+        <x:v>454</x:v>
+      </x:c>
+      <x:c r="F8" s="5" t="s">
+        <x:v>455</x:v>
+      </x:c>
+      <x:c r="G8" s="7" t="s">
         <x:v>456</x:v>
-      </x:c>
-      <x:c r="C8" s="5" t="s">
-        <x:v>466</x:v>
-      </x:c>
-      <x:c r="D8" s="5" t="s">
-        <x:v>458</x:v>
-      </x:c>
-      <x:c r="E8" s="5" t="s">
-        <x:v>459</x:v>
-      </x:c>
-      <x:c r="F8" s="5" t="s">
-        <x:v>460</x:v>
-      </x:c>
-      <x:c r="G8" s="7" t="s">
-        <x:v>461</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="42" customHeight="1">
       <x:c r="A9" s="6" t="s">
-        <x:v>467</x:v>
+        <x:v>462</x:v>
       </x:c>
       <x:c r="B9" s="6" t="s">
-        <x:v>468</x:v>
+        <x:v>463</x:v>
       </x:c>
       <x:c r="C9" s="6" t="s">
-        <x:v>469</x:v>
+        <x:v>464</x:v>
       </x:c>
       <x:c r="D9" s="6" t="s">
-        <x:v>458</x:v>
+        <x:v>453</x:v>
       </x:c>
       <x:c r="E9" s="6" t="s">
-        <x:v>459</x:v>
+        <x:v>454</x:v>
       </x:c>
       <x:c r="F9" s="6" t="s">
-        <x:v>460</x:v>
+        <x:v>455</x:v>
       </x:c>
       <x:c r="G9" s="7" t="s">
-        <x:v>461</x:v>
+        <x:v>456</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="42" customHeight="1">
       <x:c r="A10" s="5" t="s">
-        <x:v>470</x:v>
+        <x:v>465</x:v>
       </x:c>
       <x:c r="B10" s="5" t="s">
-        <x:v>468</x:v>
+        <x:v>463</x:v>
       </x:c>
       <x:c r="C10" s="5" t="s">
-        <x:v>471</x:v>
+        <x:v>466</x:v>
       </x:c>
       <x:c r="D10" s="5" t="s">
-        <x:v>464</x:v>
+        <x:v>459</x:v>
       </x:c>
       <x:c r="E10" s="5" t="s">
-        <x:v>459</x:v>
+        <x:v>454</x:v>
       </x:c>
       <x:c r="F10" s="5" t="s">
-        <x:v>460</x:v>
+        <x:v>455</x:v>
       </x:c>
       <x:c r="G10" s="7" t="s">
-        <x:v>461</x:v>
+        <x:v>456</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="42" customHeight="1">
       <x:c r="A11" s="6" t="s">
-        <x:v>472</x:v>
+        <x:v>467</x:v>
       </x:c>
       <x:c r="B11" s="6" t="s">
+        <x:v>451</x:v>
+      </x:c>
+      <x:c r="C11" s="6" t="s">
+        <x:v>468</x:v>
+      </x:c>
+      <x:c r="D11" s="6" t="s">
+        <x:v>453</x:v>
+      </x:c>
+      <x:c r="E11" s="6" t="s">
+        <x:v>454</x:v>
+      </x:c>
+      <x:c r="F11" s="6" t="s">
+        <x:v>455</x:v>
+      </x:c>
+      <x:c r="G11" s="7" t="s">
         <x:v>456</x:v>
-      </x:c>
-      <x:c r="C11" s="6" t="s">
-        <x:v>473</x:v>
-      </x:c>
-      <x:c r="D11" s="6" t="s">
-        <x:v>458</x:v>
-      </x:c>
-      <x:c r="E11" s="6" t="s">
-        <x:v>459</x:v>
-      </x:c>
-      <x:c r="F11" s="6" t="s">
-        <x:v>460</x:v>
-      </x:c>
-      <x:c r="G11" s="7" t="s">
-        <x:v>461</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="42" customHeight="1">
       <x:c r="A12" s="5" t="s">
-        <x:v>474</x:v>
+        <x:v>469</x:v>
       </x:c>
       <x:c r="B12" s="5" t="s">
+        <x:v>451</x:v>
+      </x:c>
+      <x:c r="C12" s="5" t="s">
+        <x:v>470</x:v>
+      </x:c>
+      <x:c r="D12" s="5" t="s">
+        <x:v>453</x:v>
+      </x:c>
+      <x:c r="E12" s="5" t="s">
+        <x:v>454</x:v>
+      </x:c>
+      <x:c r="F12" s="5" t="s">
+        <x:v>455</x:v>
+      </x:c>
+      <x:c r="G12" s="7" t="s">
         <x:v>456</x:v>
-      </x:c>
-      <x:c r="C12" s="5" t="s">
-        <x:v>475</x:v>
-      </x:c>
-      <x:c r="D12" s="5" t="s">
-        <x:v>458</x:v>
-      </x:c>
-      <x:c r="E12" s="5" t="s">
-        <x:v>459</x:v>
-      </x:c>
-      <x:c r="F12" s="5" t="s">
-        <x:v>460</x:v>
-      </x:c>
-      <x:c r="G12" s="7" t="s">
-        <x:v>461</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="42" customHeight="1">
       <x:c r="A13" s="6" t="s">
-        <x:v>476</x:v>
+        <x:v>471</x:v>
       </x:c>
       <x:c r="B13" s="6" t="s">
+        <x:v>451</x:v>
+      </x:c>
+      <x:c r="C13" s="6" t="s">
+        <x:v>472</x:v>
+      </x:c>
+      <x:c r="D13" s="6" t="s">
+        <x:v>453</x:v>
+      </x:c>
+      <x:c r="E13" s="6" t="s">
+        <x:v>454</x:v>
+      </x:c>
+      <x:c r="F13" s="6" t="s">
+        <x:v>455</x:v>
+      </x:c>
+      <x:c r="G13" s="7" t="s">
         <x:v>456</x:v>
-      </x:c>
-      <x:c r="C13" s="6" t="s">
-        <x:v>477</x:v>
-      </x:c>
-      <x:c r="D13" s="6" t="s">
-        <x:v>458</x:v>
-      </x:c>
-      <x:c r="E13" s="6" t="s">
-        <x:v>459</x:v>
-      </x:c>
-      <x:c r="F13" s="6" t="s">
-        <x:v>460</x:v>
-      </x:c>
-      <x:c r="G13" s="7" t="s">
-        <x:v>461</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="42" customHeight="1">
       <x:c r="A14" s="5" t="s">
-        <x:v>478</x:v>
+        <x:v>473</x:v>
       </x:c>
       <x:c r="B14" s="5" t="s">
-        <x:v>468</x:v>
+        <x:v>463</x:v>
       </x:c>
       <x:c r="C14" s="5" t="s">
-        <x:v>479</x:v>
+        <x:v>474</x:v>
       </x:c>
       <x:c r="D14" s="5" t="s">
-        <x:v>458</x:v>
+        <x:v>453</x:v>
       </x:c>
       <x:c r="E14" s="5" t="s">
-        <x:v>459</x:v>
+        <x:v>454</x:v>
       </x:c>
       <x:c r="F14" s="5" t="s">
-        <x:v>460</x:v>
+        <x:v>455</x:v>
       </x:c>
       <x:c r="G14" s="7" t="s">
-        <x:v>461</x:v>
+        <x:v>456</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="42" customHeight="1">
       <x:c r="A15" s="6" t="s">
-        <x:v>480</x:v>
+        <x:v>475</x:v>
       </x:c>
       <x:c r="B15" s="6" t="s">
-        <x:v>468</x:v>
+        <x:v>463</x:v>
       </x:c>
       <x:c r="C15" s="6" t="s">
-        <x:v>481</x:v>
+        <x:v>476</x:v>
       </x:c>
       <x:c r="D15" s="6" t="s">
-        <x:v>458</x:v>
+        <x:v>453</x:v>
       </x:c>
       <x:c r="E15" s="6" t="s">
-        <x:v>459</x:v>
+        <x:v>454</x:v>
       </x:c>
       <x:c r="F15" s="6" t="s">
-        <x:v>460</x:v>
+        <x:v>455</x:v>
       </x:c>
       <x:c r="G15" s="7" t="s">
-        <x:v>461</x:v>
+        <x:v>456</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="42" customHeight="1">
       <x:c r="A16" s="5" t="s">
-        <x:v>482</x:v>
+        <x:v>477</x:v>
       </x:c>
       <x:c r="B16" s="5" t="s">
-        <x:v>468</x:v>
+        <x:v>463</x:v>
       </x:c>
       <x:c r="C16" s="5" t="s">
-        <x:v>483</x:v>
+        <x:v>478</x:v>
       </x:c>
       <x:c r="D16" s="5" t="s">
-        <x:v>458</x:v>
+        <x:v>453</x:v>
       </x:c>
       <x:c r="E16" s="5" t="s">
-        <x:v>459</x:v>
+        <x:v>454</x:v>
       </x:c>
       <x:c r="F16" s="5" t="s">
-        <x:v>460</x:v>
+        <x:v>455</x:v>
       </x:c>
       <x:c r="G16" s="7" t="s">
-        <x:v>461</x:v>
+        <x:v>456</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="42" customHeight="1">
       <x:c r="A17" s="6" t="s">
-        <x:v>484</x:v>
+        <x:v>479</x:v>
       </x:c>
       <x:c r="B17" s="6" t="s">
-        <x:v>468</x:v>
+        <x:v>463</x:v>
       </x:c>
       <x:c r="C17" s="6" t="s">
-        <x:v>485</x:v>
+        <x:v>480</x:v>
       </x:c>
       <x:c r="D17" s="6" t="s">
-        <x:v>458</x:v>
+        <x:v>453</x:v>
       </x:c>
       <x:c r="E17" s="6" t="s">
-        <x:v>459</x:v>
+        <x:v>454</x:v>
       </x:c>
       <x:c r="F17" s="6" t="s">
-        <x:v>460</x:v>
+        <x:v>455</x:v>
       </x:c>
       <x:c r="G17" s="7" t="s">
-        <x:v>461</x:v>
+        <x:v>456</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="42" customHeight="1">
       <x:c r="A18" s="5" t="s">
-        <x:v>486</x:v>
+        <x:v>481</x:v>
       </x:c>
       <x:c r="B18" s="5" t="s">
+        <x:v>451</x:v>
+      </x:c>
+      <x:c r="C18" s="5" t="s">
+        <x:v>482</x:v>
+      </x:c>
+      <x:c r="D18" s="5" t="s">
+        <x:v>483</x:v>
+      </x:c>
+      <x:c r="E18" s="5" t="s">
+        <x:v>454</x:v>
+      </x:c>
+      <x:c r="F18" s="5" t="s">
+        <x:v>455</x:v>
+      </x:c>
+      <x:c r="G18" s="7" t="s">
         <x:v>456</x:v>
-      </x:c>
-      <x:c r="C18" s="5" t="s">
-        <x:v>487</x:v>
-      </x:c>
-      <x:c r="D18" s="5" t="s">
-        <x:v>488</x:v>
-      </x:c>
-      <x:c r="E18" s="5" t="s">
-        <x:v>459</x:v>
-      </x:c>
-      <x:c r="F18" s="5" t="s">
-        <x:v>460</x:v>
-      </x:c>
-      <x:c r="G18" s="7" t="s">
-        <x:v>461</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="42" customHeight="1">
       <x:c r="A19" s="6" t="s">
-        <x:v>489</x:v>
+        <x:v>484</x:v>
       </x:c>
       <x:c r="B19" s="6" t="s">
+        <x:v>451</x:v>
+      </x:c>
+      <x:c r="C19" s="6" t="s">
+        <x:v>485</x:v>
+      </x:c>
+      <x:c r="D19" s="6" t="s">
+        <x:v>483</x:v>
+      </x:c>
+      <x:c r="E19" s="6" t="s">
+        <x:v>454</x:v>
+      </x:c>
+      <x:c r="F19" s="6" t="s">
+        <x:v>455</x:v>
+      </x:c>
+      <x:c r="G19" s="7" t="s">
         <x:v>456</x:v>
-      </x:c>
-      <x:c r="C19" s="6" t="s">
-        <x:v>490</x:v>
-      </x:c>
-      <x:c r="D19" s="6" t="s">
-        <x:v>488</x:v>
-      </x:c>
-      <x:c r="E19" s="6" t="s">
-        <x:v>459</x:v>
-      </x:c>
-      <x:c r="F19" s="6" t="s">
-        <x:v>460</x:v>
-      </x:c>
-      <x:c r="G19" s="7" t="s">
-        <x:v>461</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="42" customHeight="1">
       <x:c r="A20" s="5" t="s">
-        <x:v>491</x:v>
+        <x:v>486</x:v>
       </x:c>
       <x:c r="B20" s="5" t="s">
+        <x:v>451</x:v>
+      </x:c>
+      <x:c r="C20" s="5" t="s">
+        <x:v>487</x:v>
+      </x:c>
+      <x:c r="D20" s="5" t="s">
+        <x:v>483</x:v>
+      </x:c>
+      <x:c r="E20" s="5" t="s">
+        <x:v>454</x:v>
+      </x:c>
+      <x:c r="F20" s="5" t="s">
+        <x:v>455</x:v>
+      </x:c>
+      <x:c r="G20" s="7" t="s">
         <x:v>456</x:v>
-      </x:c>
-      <x:c r="C20" s="5" t="s">
-        <x:v>492</x:v>
-      </x:c>
-      <x:c r="D20" s="5" t="s">
-        <x:v>488</x:v>
-      </x:c>
-      <x:c r="E20" s="5" t="s">
-        <x:v>459</x:v>
-      </x:c>
-      <x:c r="F20" s="5" t="s">
-        <x:v>460</x:v>
-      </x:c>
-      <x:c r="G20" s="7" t="s">
-        <x:v>461</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="42" customHeight="1">
       <x:c r="A21" s="6" t="s">
-        <x:v>493</x:v>
+        <x:v>488</x:v>
       </x:c>
       <x:c r="B21" s="6" t="s">
+        <x:v>451</x:v>
+      </x:c>
+      <x:c r="C21" s="6" t="s">
+        <x:v>489</x:v>
+      </x:c>
+      <x:c r="D21" s="6" t="s">
+        <x:v>483</x:v>
+      </x:c>
+      <x:c r="E21" s="6" t="s">
+        <x:v>454</x:v>
+      </x:c>
+      <x:c r="F21" s="6" t="s">
+        <x:v>455</x:v>
+      </x:c>
+      <x:c r="G21" s="7" t="s">
         <x:v>456</x:v>
-      </x:c>
-      <x:c r="C21" s="6" t="s">
-        <x:v>494</x:v>
-      </x:c>
-      <x:c r="D21" s="6" t="s">
-        <x:v>488</x:v>
-      </x:c>
-      <x:c r="E21" s="6" t="s">
-        <x:v>459</x:v>
-      </x:c>
-      <x:c r="F21" s="6" t="s">
-        <x:v>460</x:v>
-      </x:c>
-      <x:c r="G21" s="7" t="s">
-        <x:v>461</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="42" customHeight="1">
       <x:c r="A22" s="5" t="s">
-        <x:v>495</x:v>
+        <x:v>490</x:v>
       </x:c>
       <x:c r="B22" s="5" t="s">
+        <x:v>451</x:v>
+      </x:c>
+      <x:c r="C22" s="5" t="s">
+        <x:v>491</x:v>
+      </x:c>
+      <x:c r="D22" s="5" t="s">
+        <x:v>483</x:v>
+      </x:c>
+      <x:c r="E22" s="5" t="s">
+        <x:v>454</x:v>
+      </x:c>
+      <x:c r="F22" s="5" t="s">
+        <x:v>455</x:v>
+      </x:c>
+      <x:c r="G22" s="7" t="s">
         <x:v>456</x:v>
-      </x:c>
-      <x:c r="C22" s="5" t="s">
-        <x:v>496</x:v>
-      </x:c>
-      <x:c r="D22" s="5" t="s">
-        <x:v>488</x:v>
-      </x:c>
-      <x:c r="E22" s="5" t="s">
-        <x:v>459</x:v>
-      </x:c>
-      <x:c r="F22" s="5" t="s">
-        <x:v>460</x:v>
-      </x:c>
-      <x:c r="G22" s="7" t="s">
-        <x:v>461</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="42" customHeight="1">
       <x:c r="A23" s="6" t="s">
-        <x:v>497</x:v>
+        <x:v>492</x:v>
       </x:c>
       <x:c r="B23" s="6" t="s">
+        <x:v>451</x:v>
+      </x:c>
+      <x:c r="C23" s="6" t="s">
+        <x:v>493</x:v>
+      </x:c>
+      <x:c r="D23" s="6" t="s">
+        <x:v>483</x:v>
+      </x:c>
+      <x:c r="E23" s="6" t="s">
+        <x:v>454</x:v>
+      </x:c>
+      <x:c r="F23" s="6" t="s">
+        <x:v>455</x:v>
+      </x:c>
+      <x:c r="G23" s="7" t="s">
         <x:v>456</x:v>
-      </x:c>
-      <x:c r="C23" s="6" t="s">
-        <x:v>498</x:v>
-      </x:c>
-      <x:c r="D23" s="6" t="s">
-        <x:v>488</x:v>
-      </x:c>
-      <x:c r="E23" s="6" t="s">
-        <x:v>459</x:v>
-      </x:c>
-      <x:c r="F23" s="6" t="s">
-        <x:v>460</x:v>
-      </x:c>
-      <x:c r="G23" s="7" t="s">
-        <x:v>461</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="42" customHeight="1">
       <x:c r="A24" s="5" t="s">
-        <x:v>499</x:v>
+        <x:v>494</x:v>
       </x:c>
       <x:c r="B24" s="5" t="s">
+        <x:v>451</x:v>
+      </x:c>
+      <x:c r="C24" s="5" t="s">
+        <x:v>495</x:v>
+      </x:c>
+      <x:c r="D24" s="5" t="s">
+        <x:v>483</x:v>
+      </x:c>
+      <x:c r="E24" s="5" t="s">
+        <x:v>454</x:v>
+      </x:c>
+      <x:c r="F24" s="5" t="s">
+        <x:v>455</x:v>
+      </x:c>
+      <x:c r="G24" s="7" t="s">
         <x:v>456</x:v>
-      </x:c>
-      <x:c r="C24" s="5" t="s">
-        <x:v>500</x:v>
-      </x:c>
-      <x:c r="D24" s="5" t="s">
-        <x:v>488</x:v>
-      </x:c>
-      <x:c r="E24" s="5" t="s">
-        <x:v>459</x:v>
-      </x:c>
-      <x:c r="F24" s="5" t="s">
-        <x:v>460</x:v>
-      </x:c>
-      <x:c r="G24" s="7" t="s">
-        <x:v>461</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="42" customHeight="1">
       <x:c r="A25" s="6" t="s">
-        <x:v>501</x:v>
+        <x:v>496</x:v>
       </x:c>
       <x:c r="B25" s="6" t="s">
+        <x:v>451</x:v>
+      </x:c>
+      <x:c r="C25" s="6" t="s">
+        <x:v>497</x:v>
+      </x:c>
+      <x:c r="D25" s="6" t="s">
+        <x:v>483</x:v>
+      </x:c>
+      <x:c r="E25" s="6" t="s">
+        <x:v>454</x:v>
+      </x:c>
+      <x:c r="F25" s="6" t="s">
+        <x:v>455</x:v>
+      </x:c>
+      <x:c r="G25" s="7" t="s">
         <x:v>456</x:v>
-      </x:c>
-      <x:c r="C25" s="6" t="s">
-        <x:v>502</x:v>
-      </x:c>
-      <x:c r="D25" s="6" t="s">
-        <x:v>488</x:v>
-      </x:c>
-      <x:c r="E25" s="6" t="s">
-        <x:v>459</x:v>
-      </x:c>
-      <x:c r="F25" s="6" t="s">
-        <x:v>460</x:v>
-      </x:c>
-      <x:c r="G25" s="7" t="s">
-        <x:v>461</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="42" customHeight="1">
       <x:c r="A26" s="5" t="s">
-        <x:v>503</x:v>
+        <x:v>498</x:v>
       </x:c>
       <x:c r="B26" s="5" t="s">
+        <x:v>451</x:v>
+      </x:c>
+      <x:c r="C26" s="5" t="s">
+        <x:v>499</x:v>
+      </x:c>
+      <x:c r="D26" s="5" t="s">
+        <x:v>483</x:v>
+      </x:c>
+      <x:c r="E26" s="5" t="s">
+        <x:v>454</x:v>
+      </x:c>
+      <x:c r="F26" s="5" t="s">
+        <x:v>455</x:v>
+      </x:c>
+      <x:c r="G26" s="7" t="s">
         <x:v>456</x:v>
-      </x:c>
-      <x:c r="C26" s="5" t="s">
-        <x:v>504</x:v>
-      </x:c>
-      <x:c r="D26" s="5" t="s">
-        <x:v>488</x:v>
-      </x:c>
-      <x:c r="E26" s="5" t="s">
-        <x:v>459</x:v>
-      </x:c>
-      <x:c r="F26" s="5" t="s">
-        <x:v>460</x:v>
-      </x:c>
-      <x:c r="G26" s="7" t="s">
-        <x:v>461</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="42" customHeight="1">
       <x:c r="A27" s="6" t="s">
-        <x:v>505</x:v>
+        <x:v>500</x:v>
       </x:c>
       <x:c r="B27" s="6" t="s">
+        <x:v>451</x:v>
+      </x:c>
+      <x:c r="C27" s="6" t="s">
+        <x:v>501</x:v>
+      </x:c>
+      <x:c r="D27" s="6" t="s">
+        <x:v>483</x:v>
+      </x:c>
+      <x:c r="E27" s="6" t="s">
+        <x:v>454</x:v>
+      </x:c>
+      <x:c r="F27" s="6" t="s">
+        <x:v>455</x:v>
+      </x:c>
+      <x:c r="G27" s="7" t="s">
         <x:v>456</x:v>
-      </x:c>
-      <x:c r="C27" s="6" t="s">
-        <x:v>506</x:v>
-      </x:c>
-      <x:c r="D27" s="6" t="s">
-        <x:v>488</x:v>
-      </x:c>
-      <x:c r="E27" s="6" t="s">
-        <x:v>459</x:v>
-      </x:c>
-      <x:c r="F27" s="6" t="s">
-        <x:v>460</x:v>
-      </x:c>
-      <x:c r="G27" s="7" t="s">
-        <x:v>461</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="42" customHeight="1">
       <x:c r="A28" s="5" t="s">
-        <x:v>507</x:v>
+        <x:v>502</x:v>
       </x:c>
       <x:c r="B28" s="5" t="s">
+        <x:v>451</x:v>
+      </x:c>
+      <x:c r="C28" s="5" t="s">
+        <x:v>503</x:v>
+      </x:c>
+      <x:c r="D28" s="5" t="s">
+        <x:v>483</x:v>
+      </x:c>
+      <x:c r="E28" s="5" t="s">
+        <x:v>454</x:v>
+      </x:c>
+      <x:c r="F28" s="5" t="s">
+        <x:v>455</x:v>
+      </x:c>
+      <x:c r="G28" s="7" t="s">
         <x:v>456</x:v>
-      </x:c>
-      <x:c r="C28" s="5" t="s">
-        <x:v>508</x:v>
-      </x:c>
-      <x:c r="D28" s="5" t="s">
-        <x:v>488</x:v>
-      </x:c>
-      <x:c r="E28" s="5" t="s">
-        <x:v>459</x:v>
-      </x:c>
-      <x:c r="F28" s="5" t="s">
-        <x:v>460</x:v>
-      </x:c>
-      <x:c r="G28" s="7" t="s">
-        <x:v>461</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="42" customHeight="1">
       <x:c r="A29" s="6" t="s">
-        <x:v>509</x:v>
+        <x:v>504</x:v>
       </x:c>
       <x:c r="B29" s="6" t="s">
+        <x:v>451</x:v>
+      </x:c>
+      <x:c r="C29" s="6" t="s">
+        <x:v>505</x:v>
+      </x:c>
+      <x:c r="D29" s="6" t="s">
+        <x:v>483</x:v>
+      </x:c>
+      <x:c r="E29" s="6" t="s">
+        <x:v>454</x:v>
+      </x:c>
+      <x:c r="F29" s="6" t="s">
+        <x:v>455</x:v>
+      </x:c>
+      <x:c r="G29" s="7" t="s">
         <x:v>456</x:v>
-      </x:c>
-      <x:c r="C29" s="6" t="s">
-        <x:v>510</x:v>
-      </x:c>
-      <x:c r="D29" s="6" t="s">
-        <x:v>488</x:v>
-      </x:c>
-      <x:c r="E29" s="6" t="s">
-        <x:v>459</x:v>
-      </x:c>
-      <x:c r="F29" s="6" t="s">
-        <x:v>460</x:v>
-      </x:c>
-      <x:c r="G29" s="7" t="s">
-        <x:v>461</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="42" customHeight="1">
       <x:c r="A30" s="5" t="s">
-        <x:v>511</x:v>
+        <x:v>506</x:v>
       </x:c>
       <x:c r="B30" s="5" t="s">
+        <x:v>451</x:v>
+      </x:c>
+      <x:c r="C30" s="5" t="s">
+        <x:v>507</x:v>
+      </x:c>
+      <x:c r="D30" s="5" t="s">
+        <x:v>483</x:v>
+      </x:c>
+      <x:c r="E30" s="5" t="s">
+        <x:v>454</x:v>
+      </x:c>
+      <x:c r="F30" s="5" t="s">
+        <x:v>455</x:v>
+      </x:c>
+      <x:c r="G30" s="7" t="s">
         <x:v>456</x:v>
-      </x:c>
-      <x:c r="C30" s="5" t="s">
-        <x:v>512</x:v>
-      </x:c>
-      <x:c r="D30" s="5" t="s">
-        <x:v>488</x:v>
-      </x:c>
-      <x:c r="E30" s="5" t="s">
-        <x:v>459</x:v>
-      </x:c>
-      <x:c r="F30" s="5" t="s">
-        <x:v>460</x:v>
-      </x:c>
-      <x:c r="G30" s="7" t="s">
-        <x:v>461</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="42" customHeight="1">
       <x:c r="A31" s="6" t="s">
-        <x:v>513</x:v>
+        <x:v>508</x:v>
       </x:c>
       <x:c r="B31" s="6" t="s">
+        <x:v>451</x:v>
+      </x:c>
+      <x:c r="C31" s="6" t="s">
+        <x:v>509</x:v>
+      </x:c>
+      <x:c r="D31" s="6" t="s">
+        <x:v>483</x:v>
+      </x:c>
+      <x:c r="E31" s="6" t="s">
+        <x:v>454</x:v>
+      </x:c>
+      <x:c r="F31" s="6" t="s">
+        <x:v>455</x:v>
+      </x:c>
+      <x:c r="G31" s="7" t="s">
         <x:v>456</x:v>
-      </x:c>
-      <x:c r="C31" s="6" t="s">
-        <x:v>514</x:v>
-      </x:c>
-      <x:c r="D31" s="6" t="s">
-        <x:v>488</x:v>
-      </x:c>
-      <x:c r="E31" s="6" t="s">
-        <x:v>459</x:v>
-      </x:c>
-      <x:c r="F31" s="6" t="s">
-        <x:v>460</x:v>
-      </x:c>
-      <x:c r="G31" s="7" t="s">
-        <x:v>461</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="42" customHeight="1">
       <x:c r="A32" s="5" t="s">
-        <x:v>515</x:v>
+        <x:v>510</x:v>
       </x:c>
       <x:c r="B32" s="5" t="s">
+        <x:v>451</x:v>
+      </x:c>
+      <x:c r="C32" s="5" t="s">
+        <x:v>511</x:v>
+      </x:c>
+      <x:c r="D32" s="5" t="s">
+        <x:v>483</x:v>
+      </x:c>
+      <x:c r="E32" s="5" t="s">
+        <x:v>454</x:v>
+      </x:c>
+      <x:c r="F32" s="5" t="s">
+        <x:v>455</x:v>
+      </x:c>
+      <x:c r="G32" s="7" t="s">
         <x:v>456</x:v>
-      </x:c>
-      <x:c r="C32" s="5" t="s">
-        <x:v>516</x:v>
-      </x:c>
-      <x:c r="D32" s="5" t="s">
-        <x:v>488</x:v>
-      </x:c>
-      <x:c r="E32" s="5" t="s">
-        <x:v>459</x:v>
-      </x:c>
-      <x:c r="F32" s="5" t="s">
-        <x:v>460</x:v>
-      </x:c>
-      <x:c r="G32" s="7" t="s">
-        <x:v>461</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="42" customHeight="1">
       <x:c r="A33" s="6" t="s">
-        <x:v>517</x:v>
+        <x:v>512</x:v>
       </x:c>
       <x:c r="B33" s="6" t="s">
+        <x:v>451</x:v>
+      </x:c>
+      <x:c r="C33" s="6" t="s">
+        <x:v>513</x:v>
+      </x:c>
+      <x:c r="D33" s="6" t="s">
+        <x:v>483</x:v>
+      </x:c>
+      <x:c r="E33" s="6" t="s">
+        <x:v>454</x:v>
+      </x:c>
+      <x:c r="F33" s="6" t="s">
+        <x:v>455</x:v>
+      </x:c>
+      <x:c r="G33" s="7" t="s">
         <x:v>456</x:v>
-      </x:c>
-      <x:c r="C33" s="6" t="s">
-        <x:v>518</x:v>
-      </x:c>
-      <x:c r="D33" s="6" t="s">
-        <x:v>488</x:v>
-      </x:c>
-      <x:c r="E33" s="6" t="s">
-        <x:v>459</x:v>
-      </x:c>
-      <x:c r="F33" s="6" t="s">
-        <x:v>460</x:v>
-      </x:c>
-      <x:c r="G33" s="7" t="s">
-        <x:v>461</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="42" customHeight="1">
       <x:c r="A34" s="5" t="s">
-        <x:v>519</x:v>
+        <x:v>514</x:v>
       </x:c>
       <x:c r="B34" s="5" t="s">
+        <x:v>451</x:v>
+      </x:c>
+      <x:c r="C34" s="5" t="s">
+        <x:v>515</x:v>
+      </x:c>
+      <x:c r="D34" s="5" t="s">
+        <x:v>483</x:v>
+      </x:c>
+      <x:c r="E34" s="5" t="s">
+        <x:v>454</x:v>
+      </x:c>
+      <x:c r="F34" s="5" t="s">
+        <x:v>455</x:v>
+      </x:c>
+      <x:c r="G34" s="7" t="s">
         <x:v>456</x:v>
-      </x:c>
-      <x:c r="C34" s="5" t="s">
-        <x:v>520</x:v>
-      </x:c>
-      <x:c r="D34" s="5" t="s">
-        <x:v>488</x:v>
-      </x:c>
-      <x:c r="E34" s="5" t="s">
-        <x:v>459</x:v>
-      </x:c>
-      <x:c r="F34" s="5" t="s">
-        <x:v>460</x:v>
-      </x:c>
-      <x:c r="G34" s="7" t="s">
-        <x:v>461</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="42" customHeight="1">
       <x:c r="A35" s="6" t="s">
-        <x:v>521</x:v>
+        <x:v>516</x:v>
       </x:c>
       <x:c r="B35" s="6" t="s">
+        <x:v>451</x:v>
+      </x:c>
+      <x:c r="C35" s="6" t="s">
+        <x:v>517</x:v>
+      </x:c>
+      <x:c r="D35" s="6" t="s">
+        <x:v>483</x:v>
+      </x:c>
+      <x:c r="E35" s="6" t="s">
+        <x:v>454</x:v>
+      </x:c>
+      <x:c r="F35" s="6" t="s">
+        <x:v>455</x:v>
+      </x:c>
+      <x:c r="G35" s="7" t="s">
         <x:v>456</x:v>
-      </x:c>
-      <x:c r="C35" s="6" t="s">
-        <x:v>522</x:v>
-      </x:c>
-      <x:c r="D35" s="6" t="s">
-        <x:v>488</x:v>
-      </x:c>
-      <x:c r="E35" s="6" t="s">
-        <x:v>459</x:v>
-      </x:c>
-      <x:c r="F35" s="6" t="s">
-        <x:v>460</x:v>
-      </x:c>
-      <x:c r="G35" s="7" t="s">
-        <x:v>461</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="42" customHeight="1">
       <x:c r="A36" s="5" t="s">
-        <x:v>523</x:v>
+        <x:v>518</x:v>
       </x:c>
       <x:c r="B36" s="5" t="s">
+        <x:v>451</x:v>
+      </x:c>
+      <x:c r="C36" s="5" t="s">
+        <x:v>519</x:v>
+      </x:c>
+      <x:c r="D36" s="5" t="s">
+        <x:v>483</x:v>
+      </x:c>
+      <x:c r="E36" s="5" t="s">
+        <x:v>454</x:v>
+      </x:c>
+      <x:c r="F36" s="5" t="s">
+        <x:v>455</x:v>
+      </x:c>
+      <x:c r="G36" s="7" t="s">
         <x:v>456</x:v>
-      </x:c>
-      <x:c r="C36" s="5" t="s">
-        <x:v>524</x:v>
-      </x:c>
-      <x:c r="D36" s="5" t="s">
-        <x:v>488</x:v>
-      </x:c>
-      <x:c r="E36" s="5" t="s">
-        <x:v>459</x:v>
-      </x:c>
-      <x:c r="F36" s="5" t="s">
-        <x:v>460</x:v>
-      </x:c>
-      <x:c r="G36" s="7" t="s">
-        <x:v>461</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="42" customHeight="1">
       <x:c r="A37" s="6" t="s">
-        <x:v>525</x:v>
+        <x:v>520</x:v>
       </x:c>
       <x:c r="B37" s="6" t="s">
-        <x:v>468</x:v>
+        <x:v>463</x:v>
       </x:c>
       <x:c r="C37" s="6" t="s">
-        <x:v>526</x:v>
+        <x:v>521</x:v>
       </x:c>
       <x:c r="D37" s="6" t="s">
-        <x:v>488</x:v>
+        <x:v>483</x:v>
       </x:c>
       <x:c r="E37" s="6" t="s">
-        <x:v>459</x:v>
+        <x:v>454</x:v>
       </x:c>
       <x:c r="F37" s="6" t="s">
-        <x:v>460</x:v>
+        <x:v>455</x:v>
       </x:c>
       <x:c r="G37" s="7" t="s">
-        <x:v>461</x:v>
+        <x:v>456</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="42" customHeight="1">
       <x:c r="A38" s="5" t="s">
-        <x:v>527</x:v>
+        <x:v>522</x:v>
       </x:c>
       <x:c r="B38" s="5" t="s">
-        <x:v>468</x:v>
+        <x:v>463</x:v>
       </x:c>
       <x:c r="C38" s="5" t="s">
-        <x:v>528</x:v>
+        <x:v>523</x:v>
       </x:c>
       <x:c r="D38" s="5" t="s">
-        <x:v>488</x:v>
+        <x:v>483</x:v>
       </x:c>
       <x:c r="E38" s="5" t="s">
-        <x:v>459</x:v>
+        <x:v>454</x:v>
       </x:c>
       <x:c r="F38" s="5" t="s">
-        <x:v>460</x:v>
+        <x:v>455</x:v>
       </x:c>
       <x:c r="G38" s="7" t="s">
-        <x:v>461</x:v>
+        <x:v>456</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="42" customHeight="1">
       <x:c r="A39" s="6" t="s">
-        <x:v>529</x:v>
+        <x:v>524</x:v>
       </x:c>
       <x:c r="B39" s="6" t="s">
-        <x:v>468</x:v>
+        <x:v>463</x:v>
       </x:c>
       <x:c r="C39" s="6" t="s">
-        <x:v>530</x:v>
+        <x:v>525</x:v>
       </x:c>
       <x:c r="D39" s="6" t="s">
-        <x:v>488</x:v>
+        <x:v>483</x:v>
       </x:c>
       <x:c r="E39" s="6" t="s">
-        <x:v>459</x:v>
+        <x:v>454</x:v>
       </x:c>
       <x:c r="F39" s="6" t="s">
-        <x:v>460</x:v>
+        <x:v>455</x:v>
       </x:c>
       <x:c r="G39" s="7" t="s">
-        <x:v>461</x:v>
+        <x:v>456</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="42" customHeight="1">
       <x:c r="A40" s="5" t="s">
-        <x:v>531</x:v>
+        <x:v>526</x:v>
       </x:c>
       <x:c r="B40" s="5" t="s">
-        <x:v>468</x:v>
+        <x:v>463</x:v>
       </x:c>
       <x:c r="C40" s="5" t="s">
-        <x:v>532</x:v>
+        <x:v>527</x:v>
       </x:c>
       <x:c r="D40" s="5" t="s">
-        <x:v>488</x:v>
+        <x:v>483</x:v>
       </x:c>
       <x:c r="E40" s="5" t="s">
-        <x:v>459</x:v>
+        <x:v>454</x:v>
       </x:c>
       <x:c r="F40" s="5" t="s">
-        <x:v>460</x:v>
+        <x:v>455</x:v>
       </x:c>
       <x:c r="G40" s="7" t="s">
-        <x:v>461</x:v>
+        <x:v>456</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="42" customHeight="1">
       <x:c r="A41" s="6" t="s">
-        <x:v>533</x:v>
+        <x:v>528</x:v>
       </x:c>
       <x:c r="B41" s="6" t="s">
-        <x:v>468</x:v>
+        <x:v>463</x:v>
       </x:c>
       <x:c r="C41" s="6" t="s">
-        <x:v>534</x:v>
+        <x:v>529</x:v>
       </x:c>
       <x:c r="D41" s="6" t="s">
-        <x:v>488</x:v>
+        <x:v>483</x:v>
       </x:c>
       <x:c r="E41" s="6" t="s">
-        <x:v>459</x:v>
+        <x:v>454</x:v>
       </x:c>
       <x:c r="F41" s="6" t="s">
-        <x:v>460</x:v>
+        <x:v>455</x:v>
       </x:c>
       <x:c r="G41" s="7" t="s">
-        <x:v>461</x:v>
+        <x:v>456</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="42" customHeight="1">
       <x:c r="A42" s="5" t="s">
-        <x:v>535</x:v>
+        <x:v>530</x:v>
       </x:c>
       <x:c r="B42" s="5" t="s">
-        <x:v>468</x:v>
+        <x:v>463</x:v>
       </x:c>
       <x:c r="C42" s="5" t="s">
-        <x:v>536</x:v>
+        <x:v>531</x:v>
       </x:c>
       <x:c r="D42" s="5" t="s">
-        <x:v>488</x:v>
+        <x:v>483</x:v>
       </x:c>
       <x:c r="E42" s="5" t="s">
-        <x:v>459</x:v>
+        <x:v>454</x:v>
       </x:c>
       <x:c r="F42" s="5" t="s">
-        <x:v>460</x:v>
+        <x:v>455</x:v>
       </x:c>
       <x:c r="G42" s="7" t="s">
-        <x:v>461</x:v>
+        <x:v>456</x:v>
       </x:c>
     </x:row>
     <x:row r="43" ht="42" customHeight="1">
       <x:c r="A43" s="6" t="s">
-        <x:v>537</x:v>
+        <x:v>532</x:v>
       </x:c>
       <x:c r="B43" s="6" t="s">
-        <x:v>468</x:v>
+        <x:v>463</x:v>
       </x:c>
       <x:c r="C43" s="6" t="s">
-        <x:v>538</x:v>
+        <x:v>533</x:v>
       </x:c>
       <x:c r="D43" s="6" t="s">
-        <x:v>488</x:v>
+        <x:v>483</x:v>
       </x:c>
       <x:c r="E43" s="6" t="s">
-        <x:v>459</x:v>
+        <x:v>454</x:v>
       </x:c>
       <x:c r="F43" s="6" t="s">
-        <x:v>460</x:v>
+        <x:v>455</x:v>
       </x:c>
       <x:c r="G43" s="7" t="s">
-        <x:v>461</x:v>
+        <x:v>456</x:v>
       </x:c>
     </x:row>
     <x:row r="44" ht="42" customHeight="1">
       <x:c r="A44" s="5" t="s">
-        <x:v>539</x:v>
+        <x:v>534</x:v>
       </x:c>
       <x:c r="B44" s="5" t="s">
-        <x:v>468</x:v>
+        <x:v>463</x:v>
       </x:c>
       <x:c r="C44" s="5" t="s">
-        <x:v>540</x:v>
+        <x:v>535</x:v>
       </x:c>
       <x:c r="D44" s="5" t="s">
-        <x:v>488</x:v>
+        <x:v>483</x:v>
       </x:c>
       <x:c r="E44" s="5" t="s">
-        <x:v>459</x:v>
+        <x:v>454</x:v>
       </x:c>
       <x:c r="F44" s="5" t="s">
-        <x:v>460</x:v>
+        <x:v>455</x:v>
       </x:c>
       <x:c r="G44" s="7" t="s">
-        <x:v>461</x:v>
+        <x:v>456</x:v>
       </x:c>
     </x:row>
     <x:row r="45" ht="42" customHeight="1">
       <x:c r="A45" s="6" t="s">
-        <x:v>541</x:v>
+        <x:v>536</x:v>
       </x:c>
       <x:c r="B45" s="6" t="s">
-        <x:v>468</x:v>
+        <x:v>463</x:v>
       </x:c>
       <x:c r="C45" s="6" t="s">
-        <x:v>542</x:v>
+        <x:v>537</x:v>
       </x:c>
       <x:c r="D45" s="6" t="s">
-        <x:v>488</x:v>
+        <x:v>483</x:v>
       </x:c>
       <x:c r="E45" s="6" t="s">
-        <x:v>459</x:v>
+        <x:v>454</x:v>
       </x:c>
       <x:c r="F45" s="6" t="s">
-        <x:v>460</x:v>
+        <x:v>455</x:v>
       </x:c>
       <x:c r="G45" s="7" t="s">
-        <x:v>461</x:v>
+        <x:v>456</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="42" customHeight="1">
       <x:c r="A46" s="5" t="s">
-        <x:v>543</x:v>
+        <x:v>538</x:v>
       </x:c>
       <x:c r="B46" s="5" t="s">
-        <x:v>468</x:v>
+        <x:v>463</x:v>
       </x:c>
       <x:c r="C46" s="5" t="s">
-        <x:v>544</x:v>
+        <x:v>539</x:v>
       </x:c>
       <x:c r="D46" s="5" t="s">
-        <x:v>488</x:v>
+        <x:v>483</x:v>
       </x:c>
       <x:c r="E46" s="5" t="s">
-        <x:v>459</x:v>
+        <x:v>454</x:v>
       </x:c>
       <x:c r="F46" s="5" t="s">
-        <x:v>460</x:v>
+        <x:v>455</x:v>
       </x:c>
       <x:c r="G46" s="7" t="s">
-        <x:v>461</x:v>
+        <x:v>456</x:v>
       </x:c>
     </x:row>
     <x:row r="47" ht="42" customHeight="1">
       <x:c r="A47" s="6" t="s">
-        <x:v>545</x:v>
+        <x:v>540</x:v>
       </x:c>
       <x:c r="B47" s="6" t="s">
-        <x:v>468</x:v>
+        <x:v>463</x:v>
       </x:c>
       <x:c r="C47" s="6" t="s">
-        <x:v>546</x:v>
+        <x:v>541</x:v>
       </x:c>
       <x:c r="D47" s="6" t="s">
-        <x:v>488</x:v>
+        <x:v>483</x:v>
       </x:c>
       <x:c r="E47" s="6" t="s">
-        <x:v>459</x:v>
+        <x:v>454</x:v>
       </x:c>
       <x:c r="F47" s="6" t="s">
-        <x:v>460</x:v>
+        <x:v>455</x:v>
       </x:c>
       <x:c r="G47" s="7" t="s">
-        <x:v>461</x:v>
+        <x:v>456</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="42" customHeight="1">
       <x:c r="A48" s="5" t="s">
-        <x:v>547</x:v>
+        <x:v>542</x:v>
       </x:c>
       <x:c r="B48" s="5" t="s">
-        <x:v>468</x:v>
+        <x:v>463</x:v>
       </x:c>
       <x:c r="C48" s="5" t="s">
-        <x:v>548</x:v>
+        <x:v>543</x:v>
       </x:c>
       <x:c r="D48" s="5" t="s">
-        <x:v>488</x:v>
+        <x:v>483</x:v>
       </x:c>
       <x:c r="E48" s="5" t="s">
-        <x:v>459</x:v>
+        <x:v>454</x:v>
       </x:c>
       <x:c r="F48" s="5" t="s">
-        <x:v>460</x:v>
+        <x:v>455</x:v>
       </x:c>
       <x:c r="G48" s="7" t="s">
-        <x:v>461</x:v>
+        <x:v>456</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="42" customHeight="1">
       <x:c r="A49" s="6" t="s">
-        <x:v>549</x:v>
+        <x:v>544</x:v>
       </x:c>
       <x:c r="B49" s="6" t="s">
-        <x:v>468</x:v>
+        <x:v>463</x:v>
       </x:c>
       <x:c r="C49" s="6" t="s">
-        <x:v>550</x:v>
+        <x:v>545</x:v>
       </x:c>
       <x:c r="D49" s="6" t="s">
-        <x:v>488</x:v>
+        <x:v>483</x:v>
       </x:c>
       <x:c r="E49" s="6" t="s">
-        <x:v>459</x:v>
+        <x:v>454</x:v>
       </x:c>
       <x:c r="F49" s="6" t="s">
-        <x:v>460</x:v>
+        <x:v>455</x:v>
       </x:c>
       <x:c r="G49" s="7" t="s">
-        <x:v>461</x:v>
+        <x:v>456</x:v>
       </x:c>
     </x:row>
     <x:row r="50" ht="42" customHeight="1">
       <x:c r="A50" s="5" t="s">
-        <x:v>551</x:v>
+        <x:v>546</x:v>
       </x:c>
       <x:c r="B50" s="5" t="s">
-        <x:v>468</x:v>
+        <x:v>463</x:v>
       </x:c>
       <x:c r="C50" s="5" t="s">
-        <x:v>552</x:v>
+        <x:v>547</x:v>
       </x:c>
       <x:c r="D50" s="5" t="s">
-        <x:v>488</x:v>
+        <x:v>483</x:v>
       </x:c>
       <x:c r="E50" s="5" t="s">
-        <x:v>459</x:v>
+        <x:v>454</x:v>
       </x:c>
       <x:c r="F50" s="5" t="s">
-        <x:v>460</x:v>
+        <x:v>455</x:v>
       </x:c>
       <x:c r="G50" s="7" t="s">
-        <x:v>461</x:v>
+        <x:v>456</x:v>
       </x:c>
     </x:row>
     <x:row r="51" ht="42" customHeight="1">
       <x:c r="A51" s="6" t="s">
-        <x:v>553</x:v>
+        <x:v>548</x:v>
       </x:c>
       <x:c r="B51" s="6" t="s">
-        <x:v>468</x:v>
+        <x:v>463</x:v>
       </x:c>
       <x:c r="C51" s="6" t="s">
-        <x:v>554</x:v>
+        <x:v>549</x:v>
       </x:c>
       <x:c r="D51" s="6" t="s">
-        <x:v>488</x:v>
+        <x:v>483</x:v>
       </x:c>
       <x:c r="E51" s="6" t="s">
-        <x:v>459</x:v>
+        <x:v>454</x:v>
       </x:c>
       <x:c r="F51" s="6" t="s">
-        <x:v>460</x:v>
+        <x:v>455</x:v>
       </x:c>
       <x:c r="G51" s="7" t="s">
-        <x:v>461</x:v>
+        <x:v>456</x:v>
       </x:c>
     </x:row>
     <x:row r="52" ht="42" customHeight="1">
       <x:c r="A52" s="5" t="s">
-        <x:v>555</x:v>
+        <x:v>550</x:v>
       </x:c>
       <x:c r="B52" s="5" t="s">
-        <x:v>468</x:v>
+        <x:v>463</x:v>
       </x:c>
       <x:c r="C52" s="5" t="s">
-        <x:v>556</x:v>
+        <x:v>551</x:v>
       </x:c>
       <x:c r="D52" s="5" t="s">
-        <x:v>488</x:v>
+        <x:v>483</x:v>
       </x:c>
       <x:c r="E52" s="5" t="s">
-        <x:v>459</x:v>
+        <x:v>454</x:v>
       </x:c>
       <x:c r="F52" s="5" t="s">
-        <x:v>460</x:v>
+        <x:v>455</x:v>
       </x:c>
       <x:c r="G52" s="7" t="s">
-        <x:v>461</x:v>
+        <x:v>456</x:v>
       </x:c>
     </x:row>
     <x:row r="53" ht="42" customHeight="1">
       <x:c r="A53" s="6" t="s">
-        <x:v>557</x:v>
+        <x:v>552</x:v>
       </x:c>
       <x:c r="B53" s="6" t="s">
-        <x:v>468</x:v>
+        <x:v>463</x:v>
       </x:c>
       <x:c r="C53" s="6" t="s">
-        <x:v>558</x:v>
+        <x:v>553</x:v>
       </x:c>
       <x:c r="D53" s="6" t="s">
-        <x:v>488</x:v>
+        <x:v>483</x:v>
       </x:c>
       <x:c r="E53" s="6" t="s">
-        <x:v>459</x:v>
+        <x:v>454</x:v>
       </x:c>
       <x:c r="F53" s="6" t="s">
-        <x:v>460</x:v>
+        <x:v>455</x:v>
       </x:c>
       <x:c r="G53" s="7" t="s">
-        <x:v>461</x:v>
+        <x:v>456</x:v>
       </x:c>
     </x:row>
     <x:row r="54" ht="42" customHeight="1">
       <x:c r="A54" s="5" t="s">
-        <x:v>559</x:v>
+        <x:v>554</x:v>
       </x:c>
       <x:c r="B54" s="5" t="s">
-        <x:v>468</x:v>
+        <x:v>463</x:v>
       </x:c>
       <x:c r="C54" s="5" t="s">
-        <x:v>560</x:v>
+        <x:v>555</x:v>
       </x:c>
       <x:c r="D54" s="5" t="s">
-        <x:v>488</x:v>
+        <x:v>483</x:v>
       </x:c>
       <x:c r="E54" s="5" t="s">
-        <x:v>459</x:v>
+        <x:v>454</x:v>
       </x:c>
       <x:c r="F54" s="5" t="s">
-        <x:v>460</x:v>
+        <x:v>455</x:v>
       </x:c>
       <x:c r="G54" s="7" t="s">
-        <x:v>461</x:v>
+        <x:v>456</x:v>
       </x:c>
     </x:row>
     <x:row r="55" ht="42" customHeight="1">
       <x:c r="A55" s="6" t="s">
-        <x:v>561</x:v>
+        <x:v>556</x:v>
       </x:c>
       <x:c r="B55" s="6" t="s">
-        <x:v>468</x:v>
+        <x:v>463</x:v>
       </x:c>
       <x:c r="C55" s="6" t="s">
-        <x:v>562</x:v>
+        <x:v>557</x:v>
       </x:c>
       <x:c r="D55" s="6" t="s">
-        <x:v>488</x:v>
+        <x:v>483</x:v>
       </x:c>
       <x:c r="E55" s="6" t="s">
-        <x:v>459</x:v>
+        <x:v>454</x:v>
       </x:c>
       <x:c r="F55" s="6" t="s">
-        <x:v>460</x:v>
+        <x:v>455</x:v>
       </x:c>
       <x:c r="G55" s="7" t="s">
-        <x:v>461</x:v>
+        <x:v>456</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R82e9f932a39d44ca"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R332a81a2a1594386"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>